<commit_message>
Say where an untraceable name came from
When the name a strategy cannot find in the plan is the name of the budget programme
funding it, the strategy came from the budget document and its perfect match is a name
matching itself. That case now has its own flag and its own detector, so it is counted
rather than argued about.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -665,12 +665,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -680,17 +680,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>One usable budget year out of four documents</t>
+          <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
+          <t>Four Bruneian strategies carry the untraceable flag, and in all four the name they cannot find in the plan is the name of the budget programme funding them: 'Research costs for public higher education institutions', 'Green Building initiatives under the 12th National Development Plan' and two more. On the page they read as plan strategies with a perfect budget match and a confident rationale. They are budget lines that reached the strategy inventory, so the rationale is the model explaining why a line matches itself. This is the same root as W3 seen from the other end: W3 finds strategies with no plan text, W6 finds where their names came from instead.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
+          <t>See F3 in FIXES.xlsx. The transcript prompt is the fix. Meanwhile the budget-named flag on the country explorer marks every one of them, and audit check A16 counts them.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -705,52 +705,99 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>D10 in the detected sheet</t>
+          <t>D11 in the detected sheet; the budget-named flag in the explorer</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>One usable budget year out of four documents</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>D10 in the detected sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>A programme-strategy pair matched twice, once by each pass</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>54 Thailand pairs, 53 Brazil, 2 Brunei carry two rationales because the strategy pass and the reverse pass both reached them. The panel credits the pair once and the money is right. It only misleads if something counts rows and calls them edges, which the union dashboard did until the tile was split into pairs and rows.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Nothing to fix in the data. Any new consumer must count pairs, not rows.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>D9 in the detected sheet; the 'twice' filter in the audit view</t>
         </is>
@@ -767,7 +814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -872,7 +919,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -887,17 +934,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Strategy with no plan text behind it</t>
+          <t>Strategy named after the budget line funding it</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FINAL_PANEL.xlsx / panel</t>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2 strategy(ies) cite no component intervention and no plan paragraph. A strategy the plan does not state is a strategy that entered from the budget side, and its funding is money attributed to something the plan never asked for.</t>
+          <t>2 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
@@ -905,168 +952,209 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>Green Building initiatives under the 12th Na &lt;- named after budget line Green Building initiatives under the 12th Na
+Research costs for public higher education i &lt;- named after budget line Research costs for public higher education i</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no plan text behind it</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) cite no component intervention and no plan paragraph. A strategy the plan does not state is a strategy that entered from the budget side, and its funding is money attributed to something the plan never asked for.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>Payment for medical treatment services at Gleneagles Jerudong Park Med
 Purchase of medicines, medical consumables and laboratory testing need</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>2 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>FY2025 reconciliation_mismatch 1: programs sum to 1,912.5 but strategy_total is 1,949.8 (gap 37.3) - a program line is likel
 FY2025 reconciliation_mismatch 3: programs sum to 626.7 but strategy_total is 624.9 (gap -1.8) - a program line is likely mi</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>A strategy total its own programmes do not add up to</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / reconciliation</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>2 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>FY2025 strategy 1: printed 1,949.8, programmes sum to 1,912.5, apart by 37.3
 FY2025 strategy 3: printed 624.9, programmes sum to 626.7, apart by -1.8</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>brazil</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>One budget year only</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>budget_layer_all_years.xlsx</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-    </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
 FY2024 0151 Protection of indigenous lands, territorial management and e
@@ -1075,41 +1163,41 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
 Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
@@ -1117,41 +1205,41 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>1144 | Sustainable Agriculture
 4101 | Public and Government Communication
@@ -1159,81 +1247,81 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>brunei</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>One budget year only</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>budget_layer_all_years.xlsx</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
 Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -1241,41 +1329,41 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>27 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Construction programme for sewerage and waste drainage infrastructure 
 National security, defence and public safety infrastructure
@@ -1288,41 +1376,41 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
 Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
@@ -1335,41 +1423,41 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
 FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
@@ -1380,41 +1468,41 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
 FY2024 0905 Special operations: internal debt service (i  668,292.5
@@ -1427,41 +1515,41 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>19 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
 FY2024 1191 -&gt; family farming and agroecology (x3)
@@ -1474,122 +1562,122 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
 FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>D9</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>brunei</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>One pair matched twice, once per pass</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>FINAL_PANEL.xlsx / match_review</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>FY2025 3.3 -&gt; miftaahun najaah scheme (x2)</t>
-        </is>
-      </c>
-    </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 3.3 -&gt; miftaahun najaah scheme (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
 FY2026 3.8 Program on Public Sector Personnel  429,643.3
@@ -1602,41 +1690,41 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
 FY2023 5.7 -&gt; strategic program on supporting creation (x2)
@@ -1723,7 +1811,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>3</v>
@@ -1732,7 +1820,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -1783,7 +1871,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-13 08:23 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-13 08:51 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
A18: a strategy that consolidates nothing did not come from the plan
Brunei fails it twice. Stage 4 is handed the budget programme list as its target
granularity and, short of plan material, answered with two of those names.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -685,12 +685,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Four Bruneian strategies carry the untraceable flag, and in all four the name they cannot find in the plan is the name of the budget programme funding them: 'Research costs for public higher education institutions', 'Green Building initiatives under the 12th National Development Plan' and two more. On the page they read as plan strategies with a perfect budget match and a confident rationale. They are budget lines that reached the strategy inventory, so the rationale is the model explaining why a line matches itself. This is the same root as W3 seen from the other end: W3 finds strategies with no plan text, W6 finds where their names came from instead.</t>
+          <t>Four Bruneian strategies carry the untraceable flag and in all four the name they cannot find in the plan is the name of the budget programme funding them. The mechanism is now proved rather than suspected: run_stage4 hands Prompt 4 the list of budget programme codes and names as its target granularity (the buckets block). Brunei's stage 3 produced 1,077 interventions from the three NDP documents and not one of them mentions Gleneagles, medicines or research costs, while 'Gleneagles' appears in the budget speech and in no NDP. Short of plan material, the model took bucket names and emitted them as strategies. Two carry no component intervention at all; two carry a component whose name is also the budget line's. Stage 6 then matched each to the programme whose name it is, so the match is correct as a string and empty as evidence, and the rationale is the model explaining why a name matches itself.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>See F3 in FIXES.xlsx. The transcript prompt is the fix. Meanwhile the budget-named flag on the country explorer marks every one of them, and audit check A16 counts them.</t>
+          <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>D11 in the detected sheet; the budget-named flag in the explorer</t>
+          <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-13 08:51 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-13 11:43 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
D12: an output produced by a prompt that has since been edited
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -571,7 +571,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -581,22 +581,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>brazil, brunei</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Strategies are tagged with risks they do not respond to</t>
+          <t>Brazil's and Brunei's budget layers were extracted by a version of Prompt 5 that no longer exists</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Brazil's 'National Defense' carries Democratic Backsliding and Shifts in Globalisation. It is a standing function of the state funded every year, not a response to either risk. The tagging keys on topical adjacency rather than on the plan claiming the strategy addresses the risk, which inflates every risk chart on every page. It passes every arithmetic check because the tags are internally consistent, and it is invisible to source-fidelity checking because no figure is wrong. Three Brazilian and three Bruneian strategies carry five or more of the eleven risks.</t>
+          <t>Prompt 5 was amended on 2026-08-12 with rules 3a and 4a, which recover a programme whose table row wraps and whose amount is printed in the narrative instead, and which force a numbering check so a gap in the programme codes cannot pass. That edit found Thailand's missing 2.14 and 2.15 and closed a 36,964.5 reconciliation gap that had been recorded as intentional for weeks. Thailand was re-run under the new prompt. Brazil's budget extraction is from 2026-08-09 and Brunei's from 2026-08-10, so both are still under the old rule. Brunei's two unreconciled strategy-years (FY2025 strategy 1 short by 37.3, strategy 3 over by 1.8) are exactly the shape that edit was written to fix.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>See F2 in FIXES.xlsx. Prompt 4 must require a quotation from the strategy's own text for each risk it names, and must not tag a standing function on sector adjacency alone. Re-running stage 4 changes related_risks, risk_salience and every risk view downstream.</t>
+          <t>See F7 in FIXES.xlsx: re-run stage 5 for Brazil (2 documents) and Brunei (4), then rebuild both panels. Detector D12 now reports any output older than the prompt that produced it, so this cannot go unnoticed again.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -611,14 +611,14 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
+          <t>D12 in the detected sheet; D8 for Brunei's unreconciled years</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>brunei</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Strategies that entered the panel from the budget document rather than from the plan</t>
+          <t>Strategies are tagged with risks they do not respond to</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Two Bruneian strategies ('Purchase of medicines, medical consumables and laboratory testing needs' and 'Payment for medical treatment services at Gleneagles Jerudong') carry no component intervention and cite no plan paragraph. They are budget line names that reached the strategy inventory. Their funding is real money attributed to something the plan never asked for, and they sit in the same column as strategies the plan does state.</t>
+          <t>Brazil's 'National Defense' carries Democratic Backsliding and Shifts in Globalisation. It is a standing function of the state funded every year, not a response to either risk. The tagging keys on topical adjacency rather than on the plan claiming the strategy addresses the risk, which inflates every risk chart on every page. It passes every arithmetic check because the tags are internally consistent, and it is invisible to source-fidelity checking because no figure is wrong. Three Brazilian and three Bruneian strategies carry five or more of the eleven risks.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>See F3 in FIXES.xlsx. Brunei's plan text is a speech, so stage 3 recovers little from it and stage 4 fills the gap from the budget side. The transcript prompt is the fix; until it exists these rows should be excluded from any count of plan strategies rather than silently included.</t>
+          <t>See F2 in FIXES.xlsx. Prompt 4 must require a quotation from the strategy's own text for each risk it names, and must not tag a standing function on sector adjacency alone. Re-running stage 4 changes related_risks, risk_salience and every risk view downstream.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -658,14 +658,14 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
+          <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -680,17 +680,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
+          <t>Strategies that entered the panel from the budget document rather than from the plan</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Four Bruneian strategies carry the untraceable flag and in all four the name they cannot find in the plan is the name of the budget programme funding them. The mechanism is now proved rather than suspected: run_stage4 hands Prompt 4 the list of budget programme codes and names as its target granularity (the buckets block). Brunei's stage 3 produced 1,077 interventions from the three NDP documents and not one of them mentions Gleneagles, medicines or research costs, while 'Gleneagles' appears in the budget speech and in no NDP. Short of plan material, the model took bucket names and emitted them as strategies. Two carry no component intervention at all; two carry a component whose name is also the budget line's. Stage 6 then matched each to the programme whose name it is, so the match is correct as a string and empty as evidence, and the rationale is the model explaining why a name matches itself.</t>
+          <t>Two Bruneian strategies ('Purchase of medicines, medical consumables and laboratory testing needs' and 'Payment for medical treatment services at Gleneagles Jerudong') carry no component intervention and cite no plan paragraph. They are budget line names that reached the strategy inventory. Their funding is real money attributed to something the plan never asked for, and they sit in the same column as strategies the plan does state.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.</t>
+          <t>See F3 in FIXES.xlsx. Brunei's plan text is a speech, so stage 3 recovers little from it and stage 4 fills the gap from the budget side. The transcript prompt is the fix; until it exists these rows should be excluded from any count of plan strategies rather than silently included.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -705,19 +705,19 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
+          <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -727,17 +727,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>One usable budget year out of four documents</t>
+          <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
+          <t>Four Bruneian strategies carry the untraceable flag and in all four the name they cannot find in the plan is the name of the budget programme funding them. The mechanism is now proved rather than suspected: run_stage4 hands Prompt 4 the list of budget programme codes and names as its target granularity (the buckets block). Brunei's stage 3 produced 1,077 interventions from the three NDP documents and not one of them mentions Gleneagles, medicines or research costs, while 'Gleneagles' appears in the budget speech and in no NDP. Short of plan material, the model took bucket names and emitted them as strategies. Two carry no component intervention at all; two carry a component whose name is also the budget line's. Stage 6 then matched each to the programme whose name it is, so the match is correct as a string and empty as evidence, and the rationale is the model explaining why a name matches itself.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
+          <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -752,52 +752,99 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>D10 in the detected sheet</t>
+          <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>One usable budget year out of four documents</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>D10 in the detected sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>A programme-strategy pair matched twice, once by each pass</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>54 Thailand pairs, 53 Brazil, 2 Brunei carry two rationales because the strategy pass and the reverse pass both reached them. The panel credits the pair once and the money is right. It only misleads if something counts rows and calls them edges, which the union dashboard did until the tile was split into pairs and rows.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Nothing to fix in the data. Any new consumer must count pairs, not rows.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>D9 in the detected sheet; the 'twice' filter in the audit view</t>
         </is>
@@ -814,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -919,7 +966,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -929,22 +976,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>brunei</t>
+          <t>brazil</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Strategy named after the budget line funding it</t>
+          <t>An output predates the prompt that produced it</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+          <t>Files/llm/brazil/</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+          <t>2 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
@@ -952,209 +999,293 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
+          <t>brazil_budget_2021.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12
+brazil_budget_2024.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>Green Building initiatives under the 12th Na &lt;- named after budget line Green Building initiatives under the 12th Na
 Research costs for public higher education i &lt;- named after budget line Research costs for public higher education i</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brunei/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>4 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>brunei_budget_2021.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2022.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2025.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2026.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>D3</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Strategy with no plan text behind it</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>2 strategy(ies) cite no component intervention and no plan paragraph. A strategy the plan does not state is a strategy that entered from the budget side, and its funding is money attributed to something the plan never asked for.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Payment for medical treatment services at Gleneagles Jerudong Park Med
 Purchase of medicines, medical consumables and laboratory testing need</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>2 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>FY2025 reconciliation_mismatch 1: programs sum to 1,912.5 but strategy_total is 1,949.8 (gap 37.3) - a program line is likel
 FY2025 reconciliation_mismatch 3: programs sum to 626.7 but strategy_total is 624.9 (gap -1.8) - a program line is likely mi</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>A strategy total its own programmes do not add up to</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / reconciliation</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>2 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>FY2025 strategy 1: printed 1,949.8, programmes sum to 1,912.5, apart by 37.3
 FY2025 strategy 3: printed 624.9, programmes sum to 626.7, apart by -1.8</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>One budget year only</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
 FY2024 0151 Protection of indigenous lands, territorial management and e
@@ -1163,41 +1294,41 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
 Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
@@ -1205,41 +1336,41 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>1144 | Sustainable Agriculture
 4101 | Public and Government Communication
@@ -1247,81 +1378,81 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>One budget year only</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
 Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -1329,41 +1460,41 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>27 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Construction programme for sewerage and waste drainage infrastructure 
 National security, defence and public safety infrastructure
@@ -1376,41 +1507,41 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
 Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
@@ -1423,41 +1554,41 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
 FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
@@ -1468,41 +1599,41 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
 FY2024 0905 Special operations: internal debt service (i  668,292.5
@@ -1515,41 +1646,41 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>19 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
 FY2024 1191 -&gt; family farming and agroecology (x3)
@@ -1562,122 +1693,122 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
 FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>FY2025 3.3 -&gt; miftaahun najaah scheme (x2)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
 FY2026 3.8 Program on Public Sector Personnel  429,643.3
@@ -1690,41 +1821,41 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
 FY2023 5.7 -&gt; strategic program on supporting creation (x2)
@@ -1792,7 +1923,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>4</v>
@@ -1801,7 +1932,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1811,7 +1942,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>3</v>
@@ -1820,7 +1951,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -1871,7 +2002,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-13 14:50 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-13 15:03 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Add bhutan, brazil, brunei, kiribati, thailand to the dashboard
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -628,22 +628,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>kiribati</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Strategies are tagged with risks they do not respond to</t>
+          <t>A budget document can be the right document, parsed perfectly, and still extract nothing</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Brazil's 'National Defense' carries Democratic Backsliding and Shifts in Globalisation. It is a standing function of the state funded every year, not a response to either risk. The tagging keys on topical adjacency rather than on the plan claiming the strategy addresses the risk, which inflates every risk chart on every page. It passes every arithmetic check because the tags are internally consistent, and it is invisible to source-fidelity checking because no figure is wrong. Three Brazilian and three Bruneian strategies carry five or more of the eleven risks.</t>
+          <t>Kiribati cost $6.21 and produced no budget lines at all, in two different ways. First against the Recurrent Budget, which is the densest table in the whole set at 16.8 rows a page and whose rows are objects of expenditure: 219 Local catering, 227 External travel, 230 Cleaning. Nothing in it maps to a plan strategy. Then against the Development Budget, which IS the right document, is organised by KV20 pillar, carries project codes and titles, and parsed cleanly into 64 tables. It still returned nothing, because Table 7A has ten numeric columns of which six are years: Total Project Cost, Accumulated Balance, 2024 Budget, 2024 Revised, 2024 Warrant, 2024 Estimated Balance, 2025 Budget, 2026 Estimate. Prompt 5 assumes one amount column and a strategy total to reconcile against, and the ministry rows carry no totals. The first project has 4,427 under 2024 Warrant and nothing under 2025 Budget. The model returning an empty array is the correct answer to a question that was not asked properly.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>See F2 in FIXES.xlsx. Prompt 4 must require a quotation from the strategy's own text for each risk it names, and must not tag a standing function on sector adjacency alone. Re-running stage 4 changes related_risks, risk_salience and every risk view downstream.</t>
+          <t>See F8 in FIXES.xlsx. Two failure modes, two detectors, both now in document_shape.py: a LINE ITEMS verdict for a table whose rows are objects of expenditure, and a year-column count that says a fiscal-year column has to be named in the config before Prompt 5 sees the table.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -653,19 +653,19 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
+          <t>D12 and the shape probe; Files/llm/kiribati/kiribati_budget_*.xlsx, 0 rows each</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -675,22 +675,22 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>brunei</t>
+          <t>bhutan, ghana, malaysia</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Strategies that entered the panel from the budget document rather than from the plan</t>
+          <t>Four of seven candidate countries cannot be run on the budget documents we hold, each for a different reason</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Two Bruneian strategies ('Purchase of medicines, medical consumables and laboratory testing needs' and 'Payment for medical treatment services at Gleneagles Jerudong') carry no component intervention and cite no plan paragraph. They are budget line names that reached the strategy inventory. Their funding is real money attributed to something the plan never asked for, and they sit in the same column as strategies the plan does state.</t>
+          <t>A stage 5 probe on one document per country, $4.10 in total, settled what three rounds of text heuristics could not. Kenya yields 631 programmes from 1,149 pages and Jamaica 208 from 706, both clean vote-to-programme hierarchies. Ghana yields zero: its FY2024 budget statement is a narrative policy document and the appropriations sit in an appendix file we hold for FY2015 only. Bhutan yields zero: its Budget Report is a fiscal analysis whose largest table is state-owned enterprise accounts, revenue, expenses and profit before tax, with no appropriations anywhere in it. Malaysia yields 71 programmes from 584 pages, correctly formed but far too few for a document of that size, so it is under-extracting rather than failing. Kiribati is W8. The pattern is that a country fails on its DOCUMENTS long before it fails on its prompts, and no amount of reading the text locally establishes which.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>See F3 in FIXES.xlsx. Brunei's plan text is a speech, so stage 3 recovers little from it and stage 4 fills the gap from the budget side. The transcript prompt is the fix; until it exists these rows should be excluded from any count of plan strategies rather than silently included.</t>
+          <t>See F9. Probe one document before committing a country: 02_Automation/stage5_probe.py, $0.15 to $2.64 a document against $8 to $48 a country. Ghana and Bhutan need their appropriation documents sourced; Malaysia needs its under-extraction diagnosed before it is worth $48.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -700,19 +700,19 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
+          <t>Files/llm/_probe/*.xlsx; Kenya 631 programmes, Jamaica 208, Malaysia 71, Ghana 0, Bhutan 0, Kiribati 0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -722,22 +722,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>brunei</t>
+          <t>all</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
+          <t>Strategies are tagged with risks they do not respond to</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Four Bruneian strategies carry the untraceable flag and in all four the name they cannot find in the plan is the name of the budget programme funding them. The mechanism is now proved rather than suspected: run_stage4 hands Prompt 4 the list of budget programme codes and names as its target granularity (the buckets block). Brunei's stage 3 produced 1,077 interventions from the three NDP documents and not one of them mentions Gleneagles, medicines or research costs, while 'Gleneagles' appears in the budget speech and in no NDP. Short of plan material, the model took bucket names and emitted them as strategies. Two carry no component intervention at all; two carry a component whose name is also the budget line's. Stage 6 then matched each to the programme whose name it is, so the match is correct as a string and empty as evidence, and the rationale is the model explaining why a name matches itself.</t>
+          <t>Brazil's 'National Defense' carries Democratic Backsliding and Shifts in Globalisation. It is a standing function of the state funded every year, not a response to either risk. The tagging keys on topical adjacency rather than on the plan claiming the strategy addresses the risk, which inflates every risk chart on every page. It passes every arithmetic check because the tags are internally consistent, and it is invisible to source-fidelity checking because no figure is wrong. Three Brazilian and three Bruneian strategies carry five or more of the eleven risks.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.</t>
+          <t>See F2 in FIXES.xlsx. Prompt 4 must require a quotation from the strategy's own text for each risk it names, and must not tag a standing function on sector adjacency alone. Re-running stage 4 changes related_risks, risk_salience and every risk view downstream.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -752,19 +752,19 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
+          <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>W4</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>One usable budget year out of four documents</t>
+          <t>Strategies that entered the panel from the budget document rather than from the plan</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
+          <t>Two Bruneian strategies ('Purchase of medicines, medical consumables and laboratory testing needs' and 'Payment for medical treatment services at Gleneagles Jerudong') carry no component intervention and cite no plan paragraph. They are budget line names that reached the strategy inventory. Their funding is real money attributed to something the plan never asked for, and they sit in the same column as strategies the plan does state.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
+          <t>See F3 in FIXES.xlsx. Brunei's plan text is a speech, so stage 3 recovers little from it and stage 4 fills the gap from the budget side. The transcript prompt is the fix; until it exists these rows should be excluded from any count of plan strategies rather than silently included.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -799,52 +799,146 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>D10 in the detected sheet</t>
+          <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Four Bruneian strategies carry the untraceable flag and in all four the name they cannot find in the plan is the name of the budget programme funding them. The mechanism is now proved rather than suspected: run_stage4 hands Prompt 4 the list of budget programme codes and names as its target granularity (the buckets block). Brunei's stage 3 produced 1,077 interventions from the three NDP documents and not one of them mentions Gleneagles, medicines or research costs, while 'Gleneagles' appears in the budget speech and in no NDP. Short of plan material, the model took bucket names and emitted them as strategies. Two carry no component intervention at all; two carry a component whose name is also the budget line's. Stage 6 then matched each to the programme whose name it is, so the match is correct as a string and empty as evidence, and the rationale is the model explaining why a name matches itself.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>One usable budget year out of four documents</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>D10 in the detected sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>W5</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>A programme-strategy pair matched twice, once by each pass</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>54 Thailand pairs, 53 Brazil, 2 Brunei carry two rationales because the strategy pass and the reverse pass both reached them. The panel credits the pair once and the money is right. It only misleads if something counts rows and calls them edges, which the union dashboard did until the tile was split into pairs and rows.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Nothing to fix in the data. Any new consumer must count pairs, not rows.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>D9 in the detected sheet; the 'twice' filter in the audit view</t>
         </is>
@@ -2002,7 +2096,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-13 15:03 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-15 09:24 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Add brazil, brunei, jamaica, kenya, thailand to the dashboard
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -1002,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1355,78 +1355,266 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>brazil</t>
+          <t>jamaica</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>One budget year only</t>
+          <t>Flag raised while combining the budget years</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>budget_layer_all_years.xlsx</t>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+          <t>41 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>FY2019 reconciliation_mismatch 01: programs sum to 5,419,260.0 but strategy_total is 3,738,254.0 (gap -1,681,006.0) - a progr
+FY2019 reconciliation_mismatch 05: programs sum to 495,930.0 but strategy_total is 273,408.0 (gap -222,522.0) - a program lin
+FY2019 reconciliation_mismatch 06: programs sum to 156,267.0 but strategy_total is 56,267.0 (gap -100,000.0) - a program line
+FY2019 reconciliation_mismatch 20: programs sum to 2,997,389.0 but strategy_total is 49,739.0 (gap -2,947,650.0) - a program 
+FY2019 reconciliation_mismatch 21: programs sum to 2,611,812.0 but strategy_total is 38,768.0 (gap -2,573,044.0) - a program 
+FY2019 reconciliation_mismatch 22: programs sum to 6,596,981.0 but strategy_total is 186,121.0 (gap -6,410,860.0) - a program
+FY2019 reconciliation_mismatch 23: programs sum to 435,892.0 but strategy_total is 93,664.0 (gap -342,228.0) - a program line
+FY2019 reconciliation_mismatch 24: programs sum to 273,000.0 but strategy_total is 71,741.0 (gap -201,259.0) - a program line</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>41 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 strategy 01: printed 3,738,254.0, programmes sum to 5,419,260.0, apart by -1,681,006.0
+FY2019 strategy 05: printed 273,408.0, programmes sum to 495,930.0, apart by -222,522.0
+FY2019 strategy 06: printed 56,267.0, programmes sum to 156,267.0, apart by -100,000.0
+FY2019 strategy 20: printed 49,739.0, programmes sum to 2,997,389.0, apart by -2,947,650.0
+FY2019 strategy 21: printed 38,768.0, programmes sum to 2,611,812.0, apart by -2,573,044.0
+FY2019 strategy 22: printed 186,121.0, programmes sum to 6,596,981.0, apart by -6,410,860.0
+FY2019 strategy 23: printed 93,664.0, programmes sum to 435,892.0, apart by -342,228.0
+FY2019 strategy 24: printed 71,741.0, programmes sum to 273,000.0, apart by -201,259.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>8 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 reconciliation_mismatch 0106000: programs sum to 349,247,063.0 but strategy_total is 276,081,719.0 (gap -73,165,344.0) - a 
+FY2020 reconciliation_mismatch 0508000: programs sum to 2,991,357,360.0 but strategy_total is 164,025,309.0 (gap -2,827,332,051.0)
+FY2020 reconciliation_mismatch 1014000: programs sum to 7,655,824,962.0 but strategy_total is 0.0 (gap -7,655,824,962.0) - a progr
+FY2020 reconciliation_mismatch 1018000: programs sum to 10,066,601,747.0 but strategy_total is 10,873,301,747.0 (gap 806,700,000.0
+FY2025 reconciliation_mismatch 0106000: programs sum to 418,347,116.0 but strategy_total is 346,691,310.0 (gap -71,655,806.0) - a 
+FY2025 reconciliation_mismatch 0508000: programs sum to 3,536,217,818.0 but strategy_total is 435,378,299.0 (gap -3,100,839,519.0)
+FY2025 reconciliation_mismatch 0709000: programs sum to 234,021,081.0 but strategy_total is 233,471,082.0 (gap -549,999.0) - a pro
+FY2025 reconciliation_mismatch 0710000: programs sum to 4,177,242,813.0 but strategy_total is 2,000,000.0 (gap -4,175,242,813.0) -</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 strategy 0106000: printed 276,081,719.0, programmes sum to 349,247,063.0, apart by -73,165,344.0
+FY2020 strategy 0508000: printed 164,025,309.0, programmes sum to 2,991,357,360.0, apart by -2,827,332,051.0
+FY2020 strategy 1014000: printed 0.0, programmes sum to 7,655,824,962.0, apart by -7,655,824,962.0
+FY2020 strategy 1018000: printed 10,873,301,747.0, programmes sum to 10,066,601,747.0, apart by 806,700,000.0
+FY2025 strategy 0106000: printed 346,691,310.0, programmes sum to 418,347,116.0, apart by -71,655,806.0
+FY2025 strategy 0508000: printed 435,378,299.0, programmes sum to 3,536,217,818.0, apart by -3,100,839,519.0
+FY2025 strategy 0709000: printed 233,471,082.0, programmes sum to 234,021,081.0, apart by -549,999.0
+FY2025 strategy 0710000: printed 2,000,000.0, programmes sum to 4,177,242,813.0, apart by -4,175,242,813.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
 FY2024 0151 Protection of indigenous lands, territorial management and e
@@ -1435,41 +1623,41 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
 Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
@@ -1477,41 +1665,41 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>1144 | Sustainable Agriculture
 4101 | Public and Government Communication
@@ -1519,81 +1707,81 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>One budget year only</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
 Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -1601,41 +1789,41 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>27 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Construction programme for sewerage and waste drainage infrastructure 
 National security, defence and public safety infrastructure
@@ -1648,41 +1836,410 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>44 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 01.004 Regional and International Cooperation
+FY2019 03.110 Agro Industries
+FY2019 05.578 Geological, Geo Technical Regulatory Services
+FY2019 06.005 Disaster Management
+FY2019 06.232 Toll Road Authority
+FY2019 07.230 Road Traffic and Safety
+FY2019 07.558 Improvement of Public Transport
+FY2019 09.002 Training</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>1 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Health service delivery and public health pr -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>117 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Public Service Management and Administration
+Civil Registration and Vital Statistics
+Youth Development
+Support for Social Intervention
+Support for National Poverty Reduction
+General Assistance Grants
+Social Security and Welfare Services
+Policy Facilitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>775 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>775</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 blank_amount 01: amount is blank/unparseable.
+FY2019 blank_amount 03: amount is blank/unparseable.
+FY2019 blank_amount 05: amount is blank/unparseable.
+FY2019 blank_amount 06: amount is blank/unparseable.
+FY2019 blank_amount 06: amount is blank/unparseable.
+FY2019 blank_amount 07: amount is blank/unparseable.
+FY2019 blank_amount 07: amount is blank/unparseable.
+FY2019 blank_amount 09: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0105000.0105060 NAMATA
+FY2020 0120000.0120040 Fisheries Research &amp; Development
+FY2020 0620000.0620020 Police Vetting
+FY2020 0703000.0703050 Coordination of Vision 2030
+FY2020 0712000.0712050 Finance Management Services
+FY2020 0715000.0715060 International Relations and Cooperation
+FY2020 0733000.0733040 Peace and Conflict Management
+FY2020 0740000.0740010 Government Clearing Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Promotion and Development of MSMEs -&gt; 5 risks: Climate Change, Demographic Shifts, Resource and Energy Pressures, Shifts in Glo
+Product and Market Development for MSMEs -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Agricultural Research &amp; Development -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand
+Drought Management -&gt; 5 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Res
+Management of Diaspora Affairs -&gt; 5 risks: Demographic Shifts, Pandemics, Resource and Energy Pressures, Shifts in Globalis
+Foreign Relation and Diplomacy -&gt; 7 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada
+0320000 | Industrial Promotion and Developme -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+0610000 | Dispensation of Justice -&gt; 5 risks: Climate Change, Democratic Backsliding, Increased Polarisation, Pandemics, Techn</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>264 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>264</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Livestock Production and Management
+Livestock Diseases Management and Control
+Livestock Products Value Addition and Marketing
+Irrigation and Drainage
+Promotion and Development of MSMEs
+Product and Market Development for MSMEs
+Digitization and Financial Inclusion for MSMEs
+Business financing &amp; incubation for MSMEs</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>1455 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>1455</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
+FY2020 blank_amount 0120000: amount is blank/unparseable.
+FY2020 blank_amount 0620000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0712000: amount is blank/unparseable.
+FY2020 blank_amount 0715000: amount is blank/unparseable.
+FY2020 blank_amount 0733000: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
 Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
@@ -1695,41 +2252,41 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
 FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
@@ -1740,41 +2297,41 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
 FY2024 0905 Special operations: internal debt service (i  668,292.5
@@ -1787,41 +2344,41 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>19 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
 FY2024 1191 -&gt; family farming and agroecology (x3)
@@ -1834,122 +2391,216 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
 FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>FY2025 3.3 -&gt; miftaahun najaah scheme (x2)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>323 distinct programme(s) across 411 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 25.10099 Contingencies  49,466,200.0
+FY2024 21.10715 Delivery of Instruction  41,321,880.0
+FY2024 22.10715 Delivery of Instruction  41,183,070.0
+FY2019 25.10099 Undistributed Allocation  37,718,834.0
+FY2022 02.137 Management of Public Finances  33,187,287.0
+FY2022 22.10715 Delivery of Instruction  30,917,965.0
+FY2022 21.10715 Delivery of Instruction  30,603,907.0
+FY2024 25.21686 Contingency Provision  24,524,372.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>716 distinct programme(s) across 985 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 2091.0509000 Teacher Resource Management  347,685,463,808.0
+FY2025 0509000.0509010 Teacher Management- Primary  201,136,266,225.0
+FY2025 1091.0202000 Road Transport  198,961,988,075.0
+FY2025 0801000.0801010 National Defense  169,815,800,000.0
+FY2025 1041.0801000 Defence  169,815,800,000.0
+FY2020 0509000.0509010 Teacher Management- Primary  164,840,984,624.0
+FY2025 0509000.0509020 Teacher management - Secondary  142,015,327,079.0
+FY2025 1065.0504000 University Education  124,387,898,039.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
 FY2026 3.8 Program on Public Sector Personnel  429,643.3
@@ -1962,41 +2613,41 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
 FY2023 5.7 -&gt; strategic program on supporting creation (x2)
@@ -2020,7 +2671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2098,19 +2749,57 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E6" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2143,7 +2832,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-15 09:42 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-15 10:06 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Add brazil, brunei, fiji, jamaica, kenya, thailand to the dashboard
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1412,28 +1412,122 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>28 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 22: programs sum to 321,245.4 but strategy_total is 321,245.6 (gap 0.2) - a program line is li
+FY2017 reconciliation_mismatch 24: programs sum to 113,354.0 but strategy_total is 113,354.1 (gap 0.1) - a program line is li
+FY2017 reconciliation_mismatch 25: programs sum to 23,096.7 but strategy_total is 23,096.6 (gap -0.1) - a program line is lik
+FY2017 reconciliation_mismatch 33: programs sum to 28,538.8 but strategy_total is 42,329.9 (gap 13,791.1) - a program line is
+FY2017 reconciliation_mismatch 40: programs sum to 133,737.9 but strategy_total is 134,178.0 (gap 440.1) - a program line is 
+FY2017 reconciliation_mismatch 50: programs sum to 615,572.2 but strategy_total is 628,116.8 (gap 12,544.6) - a program line 
+FY2017 reconciliation_mismatch 52: programs sum to 364,701.0 but strategy_total is 354,607.9 (gap -10,093.1) - a program line
+FY2018 reconciliation_mismatch 2: programs sum to 23,891.3 but strategy_total is 14,262.3 (gap -9,629.0) - a program line is</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>28 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 22: printed 321,245.6, programmes sum to 321,245.4, apart by 0.2
+FY2017 strategy 24: printed 113,354.1, programmes sum to 113,354.0, apart by 0.1
+FY2017 strategy 25: printed 23,096.6, programmes sum to 23,096.7, apart by -0.1
+FY2017 strategy 33: printed 42,329.9, programmes sum to 28,538.8, apart by 13,791.1
+FY2017 strategy 40: printed 134,178.0, programmes sum to 133,737.9, apart by 440.1
+FY2017 strategy 50: printed 628,116.8, programmes sum to 615,572.2, apart by 12,544.6
+FY2017 strategy 52: printed 354,607.9, programmes sum to 364,701.0, apart by -10,093.1
+FY2018 strategy 2: printed 14,262.3, programmes sum to 23,891.3, apart by -9,629.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>147 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>147</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>FY2019 reconciliation_mismatch 01000: programs sum to 83,000.0 but strategy_total is 290,111.0 (gap 207,111.0) - a program line 
 FY2019 reconciliation_mismatch 02000: programs sum to 232,536.0 but strategy_total is 1,089,639.0 (gap 857,103.0) - a program li
@@ -1446,41 +1540,41 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>A strategy total its own programmes do not add up to</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / reconciliation</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>147 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>147</v>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>FY2019 strategy 01000: printed 290,111.0, programmes sum to 83,000.0, apart by 207,111.0
 FY2019 strategy 02000: printed 1,089,639.0, programmes sum to 232,536.0, apart by 857,103.0
@@ -1493,41 +1587,41 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>A programme code is not unique within a year</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>7 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>FY2025 programme 0106000: 346,691,310.0 and 364,590,743.0  (under budget strategies 1094, 1095)
 FY2025 programme 0207000: 231,885,786.0 and 278,922,194.0  (under budget strategies 1122, 1123)
@@ -1539,82 +1633,82 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>D11</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Strategy named after the budget line funding it</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel + match_review</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>2 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Promotion and Development of MSMEs &lt;- named after budget line MSMEs Development and Promotion
 Product and Market Development for MSMEs &lt;- named after budget line Market Linkages for MSMEs</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>8 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>FY2020 reconciliation_mismatch 0106000: programs sum to 349,247,063.0 but strategy_total is 276,081,719.0 (gap -73,165,344.0) - a 
 FY2020 reconciliation_mismatch 0508000: programs sum to 2,991,357,360.0 but strategy_total is 164,025,309.0 (gap -2,827,332,051.0)
@@ -1627,41 +1721,41 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>A strategy total its own programmes do not add up to</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / reconciliation</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>8 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>FY2020 strategy 0106000: printed 276,081,719.0, programmes sum to 349,247,063.0, apart by -73,165,344.0
 FY2020 strategy 0508000: printed 164,025,309.0, programmes sum to 2,991,357,360.0, apart by -2,827,332,051.0
@@ -1674,81 +1768,81 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>One budget year only</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
 FY2024 0151 Protection of indigenous lands, territorial management and e
@@ -1757,41 +1851,41 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
 Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
@@ -1799,41 +1893,41 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>1144 | Sustainable Agriculture
 4101 | Public and Government Communication
@@ -1841,81 +1935,81 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>One budget year only</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
 Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -1923,41 +2017,41 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>27 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Construction programme for sewerage and waste drainage infrastructure 
 National security, defence and public safety infrastructure
@@ -1970,41 +2064,221 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>1 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 30.5 Land Drainage and Flood Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>23 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>43.1 | Roads, Bridges and Jetties -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+21.2 | Primary Education -&gt; 6 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
+20.1 | Fiji Police -&gt; 6 risks: Democratic Backsliding, Demographic Shifts, Environmental Degradation and Pollut
+24.2 | Social Welfare -&gt; 5 risks: Climate Change, Demographic Shifts, Resource and Energy Pressures, Shifts in Glo
+22.2 | Health Services -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan
+35.1 | Sugar Development -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Res
+Department of Tourism -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+16.3 | Department of Communication -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>7 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>50.6 | Standard Expenditure Group 6
+227 | Public-Private Partnership Infrastructure and Service Delivery E
+102 | Financial Sector Modernisation and Inclusion Measures
+Audio-Visual Industry Development
+18.1 | Policy and Administration
+Unfunded Strategy | Parliamentary Governance, Oversight and Democratic
+Unfunded Strategy | Democratic Governance, Rule of Law and Institution</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>20 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 program_missing_in_year 23: program '23.2' (Housing) exists in ['2018', '2019'] but is absent in ['2017'] - check whet
+FY2017 program_missing_in_year 26: program '26.1' (Higher Education Institutions) exists in ['2018', '2019'] but is absent in
+FY2017,2018 program_missing_in_year 13: program '13.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '2
+FY2017,2018 program_missing_in_year 34: program '34.6' (Micro, Small and Medium Enterprises Central Coordinating Agency) exists in
+FY2017,2018 program_missing_in_year 4: program '4.3' (Public Enterprises) exists in ['2019'] but is absent in ['2017', '2018'] - 
+FY2017,2018 program_missing_in_year 9: program '9.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '20
+FY2018,2019 program_missing_in_year 18: program '18.4' (Rehabilitation and Rural Housing) exists in ['2017'] but is absent in ['20
+FY2018,2019 program_missing_in_year 30: program '30.5' (Land Drainage and Flood Protection) exists in ['2017'] but is absent in ['</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>18 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>FY2019 28023 Administration of Justice
 FY2019 28026 Administration of Justice
@@ -2017,81 +2291,81 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>1 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Health service delivery and public health pr -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>70 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Public Service Management and Administration
 Civil Registration and Vital Statistics
@@ -2104,41 +2378,41 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>61 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>FY2019 blank_amount 28023: amount is blank/unparseable.
 FY2019 blank_amount 28023: amount is blank/unparseable.
@@ -2151,41 +2425,41 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>FY2020 0105060 NAMATA
 FY2020 0120040 Fisheries Research &amp; Development
@@ -2198,41 +2472,41 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>0610000 | Dispensation of Justice -&gt; 5 risks: Climate Change, Democratic Backsliding, Increased Polarisation, Pandemics, Techn
 Foreign Relation and Diplomacy -&gt; 7 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada
@@ -2245,41 +2519,41 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>10 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>NAMATA
 0906000 | Labour, Employment and Safety Services
@@ -2292,41 +2566,41 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>470 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>470</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
 FY2020 blank_amount 0120000: amount is blank/unparseable.
@@ -2339,41 +2613,41 @@
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
 Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
@@ -2386,41 +2660,41 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
 FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
@@ -2431,41 +2705,41 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G38" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
 FY2024 0905 Special operations: internal debt service (i  668,292.5
@@ -2478,41 +2752,41 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>19 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
 FY2024 1191 -&gt; family farming and agroecology (x3)
@@ -2525,122 +2799,216 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
 FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>FY2025 3.3 -&gt; miftaahun najaah scheme (x2)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>43 distinct programme(s) across 91 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 50.10 Standard Expenditure Group 10  442,060.3
+FY2018 52.2 Programme 2 - Domestic Loans  267,901.9
+FY2017 52.2 Programme 2 - Domestic Loans  243,496.9
+FY2019 52.2 Domestic Loans  233,042.5
+FY2019 22.1 Policy and Administration  123,905.0
+FY2018 52.1 Programme 1 - Overseas Loans  123,372.4
+FY2019 52.1 Overseas Loans  121,320.4
+FY2017 52.1 Programme 1 - Overseas Loans  111,111.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>16 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 15.1 -&gt; justice (x2)
+FY2017 23.1 -&gt; housing (x2)
+FY2017 31.2 -&gt; fisheries (x2)
+FY2017 33.2 -&gt; mineral resources (x2)
+FY2017 34.2 -&gt; economic and trade unit (x2)
+FY2017 34.2 -&gt; economic and trade unit - investment pro (x2)
+FY2017 34.5 -&gt; department of tourism (x2)
+FY2018 23.2 -&gt; housing (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>58 distinct programme(s) across 124 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>FY2019 20017 Re-Payment of Loans  138,321,395.0
 FY2019 20018 Interest Charges  136,125,364.0
@@ -2653,81 +3021,81 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>FY2019 19048 -&gt; integrated spatial planning and developm (x2)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>404 distinct programme(s) across 502 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>FY2025 0509010 Teacher Management- Primary  201,136,266,225.0
 FY2025 0801000 Defence  169,815,800,000.0
@@ -2740,41 +3108,41 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>100 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>FY2020 0102010 -&gt; housing development and human settlement (x2)
 FY2020 0102030 -&gt; housing development and human settlement (x2)
@@ -2787,41 +3155,41 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
 FY2026 3.8 Program on Public Sector Personnel  429,643.3
@@ -2834,41 +3202,41 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
 FY2023 5.7 -&gt; strategic program on supporting creation (x2)
@@ -2892,7 +3260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2970,7 +3338,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>jamaica</t>
+          <t>fiji</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -2989,11 +3357,11 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>kenya</t>
+          <t>jamaica</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>4</v>
@@ -3002,25 +3370,44 @@
         <v>2</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>thailand</t>
+          <t>kenya</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3053,7 +3440,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-15 15:17 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-15 16:31 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Add brazil, brunei, fiji, jamaica, kenya, maldives, thailand to the dashboard
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1771,78 +1771,172 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>D10</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>brazil</t>
+          <t>maldives</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>One budget year only</t>
+          <t>Flag raised while combining the budget years</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>budget_layer_all_years.xlsx</t>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+          <t>52 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>FY2017 reconciliation_mismatch 1: programs sum to 371,971,798.0 but strategy_total is 101,334,724.0 (gap -270,637,074.0) - a
+FY2017 reconciliation_mismatch 10: programs sum to 603,169,808.0 but strategy_total is 35,391,792.0 (gap -567,778,016.0) - a 
+FY2017 reconciliation_mismatch 11: programs sum to 84,903,354.0 but strategy_total is 59,843,651.0 (gap -25,059,703.0) - a pr
+FY2017 reconciliation_mismatch 12: programs sum to 0.0 but strategy_total is 6,993,896.0 (gap 6,993,896.0) - a program line i
+FY2017 reconciliation_mismatch 13: programs sum to 0.0 but strategy_total is 3,626,872.0 (gap 3,626,872.0) - a program line i
+FY2017 reconciliation_mismatch 14: programs sum to 0.0 but strategy_total is 9,198,520.0 (gap 9,198,520.0) - a program line i
+FY2017 reconciliation_mismatch 15: programs sum to 0.0 but strategy_total is 4,223,952.0 (gap 4,223,952.0) - a program line i
+FY2017 reconciliation_mismatch 16: programs sum to 0.0 but strategy_total is 44,828,700.0 (gap 44,828,700.0) - a program line</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>52 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 1: printed 101,334,724.0, programmes sum to 371,971,798.0, apart by -270,637,074.0
+FY2017 strategy 2: printed 208,402,975.0, programmes sum to 1,780,849,664.0, apart by -1,572,446,689.0
+FY2017 strategy 3: printed 10,854,474.0, programmes sum to 291,704,544.0, apart by -280,850,070.0
+FY2017 strategy 4: printed 367,654,006.0, programmes sum to 952,692,855.0, apart by -585,038,849.0
+FY2017 strategy 5: printed 35,615,361.0, programmes sum to 796,853,288.0, apart by -761,237,927.0
+FY2017 strategy 6: printed 19,009,362.0, programmes sum to 2,294,511,756.0, apart by -2,275,502,394.0
+FY2017 strategy 7: printed 22,661,255.0, programmes sum to 266,705,093.0, apart by -244,043,838.0
+FY2017 strategy 8: printed 27,923,748.0, programmes sum to 494,853,833.0, apart by -466,930,085.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
 FY2024 0151 Protection of indigenous lands, territorial management and e
@@ -1851,41 +1945,41 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
 Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
@@ -1893,41 +1987,41 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>1144 | Sustainable Agriculture
 4101 | Public and Government Communication
@@ -1935,81 +2029,81 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>One budget year only</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
 Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -2017,41 +2111,41 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>27 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G25" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Construction programme for sewerage and waste drainage infrastructure 
 National security, defence and public safety infrastructure
@@ -2064,81 +2158,81 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>fiji</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>1 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>FY2017 30.5 Land Drainage and Flood Protection</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>fiji</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>23 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="G27" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>43.1 | Roads, Bridges and Jetties -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
 21.2 | Primary Education -&gt; 6 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -2151,41 +2245,41 @@
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>fiji</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>7 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>50.6 | Standard Expenditure Group 6
 227 | Public-Private Partnership Infrastructure and Service Delivery E
@@ -2197,41 +2291,41 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>fiji</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>20 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>FY2017 program_missing_in_year 23: program '23.2' (Housing) exists in ['2018', '2019'] but is absent in ['2017'] - check whet
 FY2017 program_missing_in_year 26: program '26.1' (Higher Education Institutions) exists in ['2018', '2019'] but is absent in
@@ -2244,41 +2338,41 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>18 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>FY2019 28023 Administration of Justice
 FY2019 28026 Administration of Justice
@@ -2291,81 +2385,81 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>1 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Health service delivery and public health pr -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>70 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>70</v>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Public Service Management and Administration
 Civil Registration and Vital Statistics
@@ -2378,41 +2472,41 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>61 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>FY2019 blank_amount 28023: amount is blank/unparseable.
 FY2019 blank_amount 28023: amount is blank/unparseable.
@@ -2425,41 +2519,41 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>FY2020 0105060 NAMATA
 FY2020 0120040 Fisheries Research &amp; Development
@@ -2472,41 +2566,41 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>0610000 | Dispensation of Justice -&gt; 5 risks: Climate Change, Democratic Backsliding, Increased Polarisation, Pandemics, Techn
 Foreign Relation and Diplomacy -&gt; 7 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada
@@ -2519,41 +2613,41 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>10 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>NAMATA
 0906000 | Labour, Employment and Safety Services
@@ -2566,41 +2660,41 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>470 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>470</v>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
 FY2020 blank_amount 0120000: amount is blank/unparseable.
@@ -2613,41 +2707,229 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>110 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 1.5 ieri
+FY2017 20.003 Beim ein ige, She's jeg;
+FY2017 26.009 jeg 932
+FY2018 1.003 Sp 322 9892
+FY2018 19.004 Amd Marmido
+FY2018 22.003 :22 823, VP 29335
+FY2018 22.066 gå sirve HABE ich give
+FY2018 22.073 eisen Pixie</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Fisheries production infrastructure and valu -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Climate adaptation, disaster risk management -&gt; 7 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Fisheries governance, management, monitoring -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Aquaculture and mariculture development -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Climate-smart agriculture, biosecurity, and  -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand
+Tourism employment, skills development, and  -&gt; 5 risks: Democratic Backsliding, Demographic Shifts, Increased Polarisation, Shifts in Gl
+Youth Protection, Inclusion and Housing Supp -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Integrated waste management and circular eco -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>164 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>164</v>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Affordable housing provision
+Labour market governance, fair pay, migration management, and worker p
+Education governance, administration and child risk information system
+School education quality, curriculum, teacher development and digital 
+Family and Community-Based Social Support Programme
+Hajj and Umrah service management and pilgrim support
+Biodiversity conservation, protected areas, and ecosystem restoration
+Climate adaptation, disaster risk management and emergency preparednes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>962 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 blank_amount 1: amount is blank/unparseable.
+FY2017 blank_amount 20: amount is blank/unparseable.
+FY2017 blank_amount 26: amount is blank/unparseable.
+FY2017 blank_amount 37: amount is blank/unparseable.
+FY2017 blank_amount 38: amount is blank/unparseable.
+FY2017 blank_amount 39: amount is blank/unparseable.
+FY2018 blank_amount 1: amount is blank/unparseable.
+FY2018 blank_amount 13: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
 Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
@@ -2660,41 +2942,41 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G43" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
 FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
@@ -2705,41 +2987,41 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="G44" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
 FY2024 0905 Special operations: internal debt service (i  668,292.5
@@ -2752,41 +3034,41 @@
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>19 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="G45" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
 FY2024 1191 -&gt; family farming and agroecology (x3)
@@ -2799,122 +3081,122 @@
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G46" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
 FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="G47" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H47" s="2" t="inlineStr">
         <is>
           <t>FY2025 3.3 -&gt; miftaahun najaah scheme (x2)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>fiji</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>43 distinct programme(s) across 91 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="G48" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H48" s="2" t="inlineStr">
         <is>
           <t>FY2017 50.10 Standard Expenditure Group 10  442,060.3
 FY2018 52.2 Programme 2 - Domestic Loans  267,901.9
@@ -2927,41 +3209,41 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>fiji</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>16 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G43" s="2" t="n">
+      <c r="G49" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H49" s="2" t="inlineStr">
         <is>
           <t>FY2017 15.1 -&gt; justice (x2)
 FY2017 23.1 -&gt; housing (x2)
@@ -2974,41 +3256,41 @@
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>58 distinct programme(s) across 124 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="G50" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H50" s="2" t="inlineStr">
         <is>
           <t>FY2019 20017 Re-Payment of Loans  138,321,395.0
 FY2019 20018 Interest Charges  136,125,364.0
@@ -3021,81 +3303,81 @@
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="G51" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H45" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>FY2019 19048 -&gt; integrated spatial planning and developm (x2)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>404 distinct programme(s) across 502 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="G52" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="H52" s="2" t="inlineStr">
         <is>
           <t>FY2025 0509010 Teacher Management- Primary  201,136,266,225.0
 FY2025 0801000 Defence  169,815,800,000.0
@@ -3108,41 +3390,41 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>kenya</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>100 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="G53" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
         <is>
           <t>FY2020 0102010 -&gt; housing development and human settlement (x2)
 FY2020 0102030 -&gt; housing development and human settlement (x2)
@@ -3155,41 +3437,88 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>656 distinct programme(s) across 827 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 19.002 et Lille Da Pi, ja gien  6,994,664,737.0
+FY2018 19.001 die Ci 29, 9 28?  1,504,471,755.0
+FY2017 30.001 xixe"jin Ds sind ja sei?  1,490,542,683.0
+FY2017 6.3 And a great قوم  1,473,416,147.0
+FY2017 2.1 ing in  1,455,757,190.0
+FY2017 21.002 وفيد ؤونه قومه مادونه  1,334,531,645.0
+FY2017 19.003 ¿ ¿ iii  1,225,233,300.0
+FY2017 20.002 - pij, ;22 29,99  1,019,664,729.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G55" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="H55" s="2" t="inlineStr">
         <is>
           <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
 FY2026 3.8 Program on Public Sector Personnel  429,643.3
@@ -3202,41 +3531,41 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G49" s="2" t="n">
+      <c r="G56" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="H49" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
 FY2023 5.7 -&gt; strategic program on supporting creation (x2)
@@ -3260,7 +3589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3395,19 +3724,38 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>thailand</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B8" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E8" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -3440,7 +3788,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-15 21:30 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-15 21:37 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Mark the stage 5 and stage 6 key fixes closed in the issue register
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Stage 5 returns one programme per Head, about a third of the programmes the document lists</t>
+          <t>Stage 5 returned one programme per Head; now extracted deterministically from the Head summary tables</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1255,12 +1255,12 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Worth about 100 extra programme rows per year, not the several hundred first thought, so it does not justify open-ended prompt iteration. The next thing to try is a deterministic pass over the summary tables rather than a prompt: a programme row there is the one whose first cell begins with two numbers, which is a rule a parser can apply and a model keeps declining to.</t>
+          <t>Fixed, and not by a prompt. extract_budget_tables.py reads the per-Head summary tables straight from the parsed markdown, where a programme row is the one whose first cell begins with two numbers. The rule is regexes in jamaica.json under 'budget_tables'; the script itself holds no country logic. The layer went from 172 programme rows to 341, edges from 92 to 399, strategies with no budget from 68 to 7, and the mapped share from 6.8% to 91.3%. Recall resolves at 66% where it could not be estimated at all. One trap for the next document: codes must be digits-and-dots, because _clean_code keeps only \d+(\.\d+)* and silently trimmed the first hyphenated attempt back to the Head.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Files/llm/_probe/_probe_jamaica_budget_2024.xlsx; the head summary tables in the DI markdown</t>
+          <t>01_Pipeline/scripts/extract_budget_tables.py; 02_Automation/inputs/jamaica.json budget_tables</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1343,38 +1343,703 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>28 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 programme 0032: 1.4 and 77.9 and 331.9 and 469.5 and 633.9 and 756.5 and 850.8 and 904.4 and 1,021.0 and 1,192.6 and 1,532.3 and 1,607.8 and 1,809.5 and 1,853.5 and 2,003.2 and 3,005.3 and 3,497.2 and 5,553.3 and 10,446.6 and 10,768.5 and 30,770.3 and 67,724.5 and 77,570.6 and 114,021.9  (under budget strategies 03, 04, 05, 06, 07, 08, 09, 10, 11, 12, 13, 14, 15, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28)
+FY2024 programme 0901: 1,984.7 and 64,985.7  (under budget strategies 28, 99)
+FY2024 programme 0902: 216.8 and 500.0 and 2,000.0 and 6,362.3 and 6,415.9 and 26,568.8 and 27,153.3  (under budget strategies 05, 11, 12, 19, 20, 23, 28)
+FY2024 programme 0903: 2,007.3 and 557,096.8  (under budget strategies 09, 28)
+FY2024 programme 0909: 0.0 and 0.3 and 0.8 and 5.3 and 149.6 and 246.0 and 1,502.0 and 116,778.3  (under budget strategies 04, 07, 12, 19, 23, 25, 26, 28)
+FY2024 programme 0910: 0.1 and 0.7 and 4.4 and 1,525.5  (under budget strategies 10, 14, 26, 28)
+FY2024 programme 1144: 0.0 and 14,910.1  (under budget strategies 20, 28)
+FY2024 programme 1149: 20.2 and 54.2  (under budget strategies 04, 14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brazil/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>brazil_budget_2021.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12
+brazil_budget_2024.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Green Building initiatives under the 12th Na &lt;- named after budget line Green Building initiatives under the 12th Na
+Infrastructure provision for enhancement of  &lt;- named after budget line Preparation and upgrading works for infrastr
+Research costs for public higher education i &lt;- named after budget line Research costs for public higher education i</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brunei/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>4 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>brunei_budget_2021.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2022.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2025.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2026.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no plan text behind it</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) cite no component intervention and no plan paragraph. A strategy the plan does not state is a strategy that entered from the budget side, and its funding is money attributed to something the plan never asked for.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Payment for medical treatment services at Gleneagles Jerudong Park Med
+Purchase of medicines, medical consumables and laboratory testing need</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 reconciliation_mismatch 1: programs sum to 1,912.5 but strategy_total is 1,949.8 (gap 37.3) - a program line is likel
+FY2025 reconciliation_mismatch 3: programs sum to 626.7 but strategy_total is 624.9 (gap -1.8) - a program line is likely mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 strategy 1: printed 1,949.8, programmes sum to 1,912.5, apart by 37.3
+FY2025 strategy 3: printed 624.9, programmes sum to 626.7, apart by -1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>28 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 22: programs sum to 321,245.4 but strategy_total is 321,245.6 (gap 0.2) - a program line is li
+FY2017 reconciliation_mismatch 24: programs sum to 113,354.0 but strategy_total is 113,354.1 (gap 0.1) - a program line is li
+FY2017 reconciliation_mismatch 25: programs sum to 23,096.7 but strategy_total is 23,096.6 (gap -0.1) - a program line is lik
+FY2017 reconciliation_mismatch 33: programs sum to 28,538.8 but strategy_total is 42,329.9 (gap 13,791.1) - a program line is
+FY2017 reconciliation_mismatch 40: programs sum to 133,737.9 but strategy_total is 134,178.0 (gap 440.1) - a program line is 
+FY2017 reconciliation_mismatch 50: programs sum to 615,572.2 but strategy_total is 628,116.8 (gap 12,544.6) - a program line 
+FY2017 reconciliation_mismatch 52: programs sum to 364,701.0 but strategy_total is 354,607.9 (gap -10,093.1) - a program line
+FY2018 reconciliation_mismatch 2: programs sum to 23,891.3 but strategy_total is 14,262.3 (gap -9,629.0) - a program line is</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>28 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 22: printed 321,245.6, programmes sum to 321,245.4, apart by 0.2
+FY2017 strategy 24: printed 113,354.1, programmes sum to 113,354.0, apart by 0.1
+FY2017 strategy 25: printed 23,096.6, programmes sum to 23,096.7, apart by -0.1
+FY2017 strategy 33: printed 42,329.9, programmes sum to 28,538.8, apart by 13,791.1
+FY2017 strategy 40: printed 134,178.0, programmes sum to 133,737.9, apart by 440.1
+FY2017 strategy 50: printed 628,116.8, programmes sum to 615,572.2, apart by 12,544.6
+FY2017 strategy 52: printed 354,607.9, programmes sum to 364,701.0, apart by -10,093.1
+FY2018 strategy 2: printed 14,262.3, programmes sum to 23,891.3, apart by -9,629.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>74 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 reconciliation_mismatch 01000: programs sum to 83,000.0 but strategy_total is 290,111.0 (gap 207,111.0) - a program line 
+FY2019 reconciliation_mismatch 08000: programs sum to 642,858.0 but strategy_total is 469,975.0 (gap -172,883.0) - a program lin
+FY2019 reconciliation_mismatch 09000: programs sum to 712,147.0 but strategy_total is 833,920.0 (gap 121,773.0) - a program line
+FY2019 reconciliation_mismatch 15010: programs sum to 0.0 but strategy_total is 697,424.0 (gap 697,424.0) - a program line is li
+FY2019 reconciliation_mismatch 15020: programs sum to 900,480.0 but strategy_total is 10,480.0 (gap -890,000.0) - a program line
+FY2019 reconciliation_mismatch 16049: programs sum to 489,234.0 but strategy_total is 225,234.0 (gap -264,000.0) - a program lin
+FY2019 reconciliation_mismatch 17000: programs sum to 6,345,325.0 but strategy_total is 11,525,361.0 (gap 5,180,036.0) - a progr
+FY2019 reconciliation_mismatch 19046: programs sum to 1,085,718.0 but strategy_total is 1,078,318.0 (gap -7,400.0) - a program l</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>74 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 strategy 01000: printed 290,111.0, programmes sum to 83,000.0, apart by 207,111.0
+FY2019 strategy 08000: printed 469,975.0, programmes sum to 642,858.0, apart by -172,883.0
+FY2019 strategy 09000: printed 833,920.0, programmes sum to 712,147.0, apart by 121,773.0
+FY2019 strategy 15010: printed 697,424.0, programmes sum to 0.0, apart by 697,424.0
+FY2019 strategy 15020: printed 10,480.0, programmes sum to 900,480.0, apart by -890,000.0
+FY2019 strategy 16049: printed 225,234.0, programmes sum to 489,234.0, apart by -264,000.0
+FY2019 strategy 17000: printed 11,525,361.0, programmes sum to 6,345,325.0, apart by 5,180,036.0
+FY2019 strategy 19046: printed 1,078,318.0, programmes sum to 1,085,718.0, apart by -7,400.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>7 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 programme 0106000: 346,691,310.0 and 364,590,743.0  (under budget strategies 1094, 1095)
+FY2025 programme 0207000: 231,885,786.0 and 278,922,194.0  (under budget strategies 1122, 1123)
+FY2025 programme 0412000: 651,366,934.0 and 16,529,119,104.0  (under budget strategies 1082, 1083)
+FY2025 programme 0508000: 297,799,258.0 and 435,378,299.0 and 4,677,027,195.0  (under budget strategies 1064, 1065, 1066)
+FY2025 programme 0709000: 233,471,082.0 and 444,125,877.0  (under budget strategies 1072, 1213)
+FY2025 programme 0710000: 2,000,000.0 and 8,769,275,002.0  (under budget strategies 1072, 1213)
+FY2025 programme 1018000: 30,500,000.0 and 12,916,448,407.0  (under budget strategies 1331, 1332)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Promotion and Development of MSMEs &lt;- named after budget line MSMEs Development and Promotion
+Product and Market Development for MSMEs &lt;- named after budget line Market Linkages for MSMEs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>8 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 reconciliation_mismatch 0106000: programs sum to 349,247,063.0 but strategy_total is 276,081,719.0 (gap -73,165,344.0) - a 
+FY2020 reconciliation_mismatch 0508000: programs sum to 2,991,357,360.0 but strategy_total is 164,025,309.0 (gap -2,827,332,051.0)
+FY2020 reconciliation_mismatch 1014000: programs sum to 7,655,824,962.0 but strategy_total is 0.0 (gap -7,655,824,962.0) - a progr
+FY2020 reconciliation_mismatch 1018000: programs sum to 10,066,601,747.0 but strategy_total is 10,873,301,747.0 (gap 806,700,000.0
+FY2025 reconciliation_mismatch 0106000: programs sum to 418,347,116.0 but strategy_total is 346,691,310.0 (gap -71,655,806.0) - a 
+FY2025 reconciliation_mismatch 0508000: programs sum to 3,536,217,818.0 but strategy_total is 435,378,299.0 (gap -3,100,839,519.0)
+FY2025 reconciliation_mismatch 0709000: programs sum to 234,021,081.0 but strategy_total is 233,471,082.0 (gap -549,999.0) - a pro
+FY2025 reconciliation_mismatch 0710000: programs sum to 4,177,242,813.0 but strategy_total is 2,000,000.0 (gap -4,175,242,813.0) -</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 strategy 0106000: printed 276,081,719.0, programmes sum to 349,247,063.0, apart by -73,165,344.0
+FY2020 strategy 0508000: printed 164,025,309.0, programmes sum to 2,991,357,360.0, apart by -2,827,332,051.0
+FY2020 strategy 1014000: printed 0.0, programmes sum to 7,655,824,962.0, apart by -7,655,824,962.0
+FY2020 strategy 1018000: printed 10,873,301,747.0, programmes sum to 10,066,601,747.0, apart by 806,700,000.0
+FY2025 strategy 0106000: printed 346,691,310.0, programmes sum to 418,347,116.0, apart by -71,655,806.0
+FY2025 strategy 0508000: printed 435,378,299.0, programmes sum to 3,536,217,818.0, apart by -3,100,839,519.0
+FY2025 strategy 0709000: printed 233,471,082.0, programmes sum to 234,021,081.0, apart by -549,999.0
+FY2025 strategy 0710000: printed 2,000,000.0, programmes sum to 4,177,242,813.0, apart by -4,175,242,813.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>138 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>138</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>FY2022 reconciliation_mismatch 1: programs sum to 19,215,800.0 but strategy_total is 13,533,000.0 (gap -5,682,800.0) - a pro
 FY2022 reconciliation_mismatch 10: programs sum to 3,621,353,400.0 but strategy_total is 5,254,500.0 (gap -3,616,098,900.0) -
@@ -1387,41 +2052,41 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>A strategy total its own programmes do not add up to</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / reconciliation</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>138 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>138</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>FY2022 strategy 1: printed 13,533,000.0, programmes sum to 19,215,800.0, apart by -5,682,800.0
 FY2022 strategy 2: printed 1,337,000.0, programmes sum to 2,500,000.0, apart by -1,163,000.0
@@ -1434,41 +2099,929 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>52 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 1: programs sum to 371,971,798.0 but strategy_total is 101,334,724.0 (gap -270,637,074.0) - a
+FY2017 reconciliation_mismatch 10: programs sum to 603,169,808.0 but strategy_total is 35,391,792.0 (gap -567,778,016.0) - a 
+FY2017 reconciliation_mismatch 11: programs sum to 84,903,354.0 but strategy_total is 59,843,651.0 (gap -25,059,703.0) - a pr
+FY2017 reconciliation_mismatch 12: programs sum to 0.0 but strategy_total is 6,993,896.0 (gap 6,993,896.0) - a program line i
+FY2017 reconciliation_mismatch 13: programs sum to 0.0 but strategy_total is 3,626,872.0 (gap 3,626,872.0) - a program line i
+FY2017 reconciliation_mismatch 14: programs sum to 0.0 but strategy_total is 9,198,520.0 (gap 9,198,520.0) - a program line i
+FY2017 reconciliation_mismatch 15: programs sum to 0.0 but strategy_total is 4,223,952.0 (gap 4,223,952.0) - a program line i
+FY2017 reconciliation_mismatch 16: programs sum to 0.0 but strategy_total is 44,828,700.0 (gap 44,828,700.0) - a program line</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>52 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 1: printed 101,334,724.0, programmes sum to 371,971,798.0, apart by -270,637,074.0
+FY2017 strategy 2: printed 208,402,975.0, programmes sum to 1,780,849,664.0, apart by -1,572,446,689.0
+FY2017 strategy 3: printed 10,854,474.0, programmes sum to 291,704,544.0, apart by -280,850,070.0
+FY2017 strategy 4: printed 367,654,006.0, programmes sum to 952,692,855.0, apart by -585,038,849.0
+FY2017 strategy 5: printed 35,615,361.0, programmes sum to 796,853,288.0, apart by -761,237,927.0
+FY2017 strategy 6: printed 19,009,362.0, programmes sum to 2,294,511,756.0, apart by -2,275,502,394.0
+FY2017 strategy 7: printed 22,661,255.0, programmes sum to 266,705,093.0, apart by -244,043,838.0
+FY2017 strategy 8: printed 27,923,748.0, programmes sum to 494,853,833.0, apart by -466,930,085.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
+FY2024 0151 Protection of indigenous lands, territorial management and e
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIAIS
+FY2024 1144 AGROPECUARIA SUSTENTAVEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
+Public Security with Citizenship -&gt; 6 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>1144 | Sustainable Agriculture
+4101 | Public and Government Communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
+Natural disaster management -&gt; 5 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>25 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Construction programme for sewerage and waste drainage infrastructure 
+National security, defence and public safety infrastructure
+Public sector performance and welfare data systems
+Road and bridge infrastructure modernisation programme
+Social welfare, community and civic facilities development
+Environmental regulation and impact assessment enforcement
+Integrated industrial diversification, FDI and MSME competitiveness st
+Industrial and business site infrastructure provision</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 30.5 Land Drainage and Flood Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>23 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>43.1 | Roads, Bridges and Jetties -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+21.2 | Primary Education -&gt; 6 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
+20.1 | Fiji Police -&gt; 6 risks: Democratic Backsliding, Demographic Shifts, Environmental Degradation and Pollut
+22.2 | Health Services -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan
+24.2 | Social Welfare -&gt; 5 risks: Climate Change, Demographic Shifts, Resource and Energy Pressures, Shifts in Glo
+35.1 | Sugar Development -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Res
+Department of Tourism -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+16.3 | Department of Communication -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>5 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>50.6 | Standard Expenditure Group 6
+227 | Public-Private Partnership Infrastructure and Service Delivery E
+102 | Financial Sector Modernisation and Inclusion Measures
+Audio-Visual Industry Development
+18.1 | Policy and Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>20 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 program_missing_in_year 23: program '23.2' (Housing) exists in ['2018', '2019'] but is absent in ['2017'] - check whet
+FY2017 program_missing_in_year 26: program '26.1' (Higher Education Institutions) exists in ['2018', '2019'] but is absent in
+FY2017,2018 program_missing_in_year 13: program '13.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '2
+FY2017,2018 program_missing_in_year 34: program '34.6' (Micro, Small and Medium Enterprises Central Coordinating Agency) exists in
+FY2017,2018 program_missing_in_year 4: program '4.3' (Public Enterprises) exists in ['2019'] but is absent in ['2017', '2018'] - 
+FY2017,2018 program_missing_in_year 9: program '9.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '20
+FY2018,2019 program_missing_in_year 18: program '18.4' (Rehabilitation and Rural Housing) exists in ['2017'] but is absent in ['20
+FY2018,2019 program_missing_in_year 30: program '30.5' (Land Drainage and Flood Protection) exists in ['2017'] but is absent in ['</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>1 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Health service delivery and public health pr -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>7 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Praedial Larceny Prevention Co- ordination
+10576 | Vision 2030 Jamaica National Development Plan
+10662 | International Programme Management
+10572 | Support for Development Planning
+Anti-Dumping and Subsidies
+Maritime Organizations
+Support for Growth Inducement Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>200 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2019 program_missing_in_year 03000: program '03000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.157' (Government Audit Services) exists in ['2022', '2024'] but is abs
+FY2019 program_missing_in_year 06000: program '06000.1.03.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 06000: program '06000.1.03.158' (Public Service Personnel Management) exists in ['2022', '2024'] 
+FY2019 program_missing_in_year 07000: program '07000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 07000: program '07000.1.99.139' (Protection of Children's Rights) exists in ['2022', '2024'] but 
+FY2019 program_missing_in_year 07000: program '07000.1.99.159' (Combatting Human Trafficking) exists in ['2022', '2024'] but is </t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0105060 NAMATA
+FY2020 0120040 Fisheries Research &amp; Development
+FY2020 0620020 Police Vetting
+FY2020 0703050 Coordination of Vision 2030
+FY2020 0712050 Finance Management Services
+FY2020 0715060 International Relations and Cooperation
+FY2020 0733040 Peace and Conflict Management
+FY2020 0740010 Government Clearing Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>12 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>0610000 | Dispensation of Justice -&gt; 5 risks: Climate Change, Democratic Backsliding, Increased Polarisation, Pandemics, Techn
+Foreign Relation and Diplomacy -&gt; 7 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada
+0111000 | Fisheries Development and Manageme -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Promotion and Development of MSMEs -&gt; 5 risks: Climate Change, Demographic Shifts, Resource and Energy Pressures, Shifts in Glo
+0320000 | Industrial Promotion and Developme -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Product and Market Development for MSMEs -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Standards and Qualitry Infrastucture &amp; Resea -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Agricultural Research &amp; Development -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>NAMATA
+0706060 | Infrastructure, science, technology and innovation
+0629000 | General Administration and Support Services
+0304010 | Governance and Accountability
+0309010 | Promotion of Local Content
+0215030 | General Administration and Support Services
+National Health Procurement Board Establishment
+Perishable Goods Storage and Export Facilitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>470 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
+FY2020 blank_amount 0120000: amount is blank/unparseable.
+FY2020 blank_amount 0620000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0712000: amount is blank/unparseable.
+FY2020 blank_amount 0715000: amount is blank/unparseable.
+FY2020 blank_amount 0733000: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>36 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>FY2022 28.030600 Maintenance, Repair and Overhaul (KTMB)
 FY2022 28.031000 Maintenance of the AwAS System
@@ -1481,41 +3034,41 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>25 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Healthcare Service Delivery Improvement -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
 National security, border management and def -&gt; 7 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -1528,41 +3081,41 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>17 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Bumiputera Socioeconomic Empowerment
 Fiscal Institutions Strengthening and Budget Management Improvement
@@ -1575,41 +3128,41 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>3929 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>3929</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FY2022 malformed_code_repaired 1: program_code '010000' looked malformed and was normalized to '1.010000' - verify against s
 FY2022 malformed_code_repaired 1: program_code '020000' looked malformed and was normalized to '1.020000' - verify against s
@@ -1622,41 +3175,785 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>110 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 1.5 ieri
+FY2017 20.003 Beim ein ige, She's jeg;
+FY2017 26.009 jeg 932
+FY2018 1.003 Sp 322 9892
+FY2018 19.004 Amd Marmido
+FY2018 22.003 :22 823, VP 29335
+FY2018 22.066 gå sirve HABE ich give
+FY2018 22.073 eisen Pixie</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Fisheries production infrastructure and valu -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Climate adaptation, disaster risk management -&gt; 7 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Fisheries governance, management, monitoring -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Aquaculture and mariculture development -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Climate-smart agriculture, biosecurity, and  -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand
+Tourism employment, skills development, and  -&gt; 5 risks: Democratic Backsliding, Demographic Shifts, Increased Polarisation, Shifts in Gl
+Youth Protection, Inclusion and Housing Supp -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Integrated waste management and circular eco -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>157 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Affordable housing provision
+Labour market governance, fair pay, migration management, and worker p
+Education governance, administration and child risk information system
+Family and Community-Based Social Support Programme
+Hajj and Umrah service management and pilgrim support
+Biodiversity conservation, protected areas, and ecosystem restoration
+Climate adaptation, disaster risk management and emergency preparednes
+Innovation, start-up incubation, and digital public information</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>962 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 blank_amount 1: amount is blank/unparseable.
+FY2017 blank_amount 20: amount is blank/unparseable.
+FY2017 blank_amount 26: amount is blank/unparseable.
+FY2017 blank_amount 37: amount is blank/unparseable.
+FY2017 blank_amount 38: amount is blank/unparseable.
+FY2017 blank_amount 39: amount is blank/unparseable.
+FY2018 blank_amount 1: amount is blank/unparseable.
+FY2018 blank_amount 13: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
+Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
+Strategic Program on Value Creation Agricult -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Strategic Program on Development of Educatio -&gt; 5 risks: Democratic Backsliding, Demographic Shifts, Increased Polarisation, Pandemics, T
+Strategic Program on Supporting Development  -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+Strategic Program on Developing National Pre -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan
+Strategic Program on Area Development and Sm -&gt; 8 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Integrated Program on Creating Income from T -&gt; 7 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023,2024 program_missing_in_year 4: program '4.12' (Program on Public Sector Personnel) exists in ['2025', '2026'] but is abse
+FY2023,2024,2026 program_missing_in_year 2: program '2.17' (Program on Public Sector Personnel) exists in ['2025'] but is absent in ['
+FY2023,2025 program_missing_in_year 7: program '7.3' (Program on Expenditures for Replenishment of Treasury Account Balance) exis
+FY2024,2025 program_missing_in_year 1: program '1.14' (Program on Public Sector Personnel) exists in ['2023', '2026'] but is abse</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
+FY2024 0905 Special operations: internal debt service (i  668,292.5
+FY2024 0903 OPERACOES ESPECIAIS: TRANSFERENCIAS CONSTITU  557,096.8
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIA  116,778.3
+FY2024 0999 Contingency reserve  89,578.8
+FY2024 0906 Special operations: external debt service (i  46,080.6
+FY2024 0908 Special operations: refinancing of external   27,246.5
+FY2024 0902 Special operations: financing with return  26,568.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>39 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 1144 -&gt; 1144 | sustainable agriculture (x2)
+FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
+FY2024 1158 -&gt; 1158 | climate emergency response (x3)
+FY2024 1191 -&gt; family farming and agroecology (x3)
+FY2024 1191 -&gt; supply and food sovereignty (x2)
+FY2024 2304 -&gt; science, technology and innovation for s (x2)
+FY2024 2305 -&gt; communications for inclusion and transfo (x2)
+FY2024 2308 -&gt; 2308 | consolidation of the national sci (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
+FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>14 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 1.14 -&gt; green building initiatives under the 12t (x2)
+FY2025 1.17 -&gt; flood prevention projects under the 12th (x2)
+FY2025 1.20 -&gt; capacity enhancement programme for irrig (x2)
+FY2025 1.22 -&gt; paddy buy-back scheme and purchase of hy (x2)
+FY2025 1.3 -&gt; water supply and sewerage system upgradi (x2)
+FY2025 1.7 -&gt; medical and health infrastructure develo (x2)
+FY2025 1.8 -&gt; bru-hims 2.0 system project (x2)
+FY2025 2.1 -&gt; infrastructure provision for enhancement (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>42 distinct programme(s) across 88 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 50.10 Standard Expenditure Group 10  442,060.3
+FY2018 52.2 Programme 2 - Domestic Loans  267,901.9
+FY2017 52.2 Programme 2 - Domestic Loans  243,496.9
+FY2019 52.2 Domestic Loans  233,042.5
+FY2019 22.1 Policy and Administration  123,905.0
+FY2018 52.1 Programme 1 - Overseas Loans  123,372.4
+FY2019 52.1 Overseas Loans  121,320.4
+FY2017 52.1 Programme 1 - Overseas Loans  111,111.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>70 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 14.1 -&gt; 14.1 | disaster management (x2)
+FY2017 14.2 -&gt; 14.2 | meteorological services (x2)
+FY2017 15.1 -&gt; justice (x2)
+FY2017 18.4 -&gt; 18.4 | rehabilitation and rural housing (x2)
+FY2017 21.2 -&gt; 21.2 | primary education (x2)
+FY2017 21.3 -&gt; 21.3 | secondary education (x2)
+FY2017 21.4 -&gt; 21.4 | curriculum development (x2)
+FY2017 21.5 -&gt; 21.5 | tertiary technical education (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>112 distinct programme(s) across 183 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 20000.6.99.137 Management of Public Finances  24,535,325.0
+FY2024 26022.1.01.001 Executive Direction and Administration  20,505,357.0
+FY2024 20019.1.99.136 Pensions and Retirement Benefits  13,856,376.0
+FY2022 42000.1.01.001 Executive Direction and Administration  12,968,255.0
+FY2022 20019.1.99.136 Pensions and Retirement Benefits  12,448,781.0
+FY2024 20012.1.02.146 Customs Management  11,295,545.0
+FY2022 26022.1.01.001 Executive Direction and Administration  11,233,758.0
+FY2024 42000.1.01.001 Executive Direction and Administration  10,473,308.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>50 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 15020.1.99.166 -&gt; civil registration and vital statistics (x2)
+FY2019 19000.6.01.301 -&gt; industrial development and export promot (x2)
+FY2019 19000.6.06.005 -&gt; disaster management (x2)
+FY2019 20056.1.02.149 -&gt; domestic tax administration programme (x2)
+FY2019 26024.1.04.167 -&gt; citizen security and justice capacity st (x2)
+FY2019 28000.1.03.154 -&gt; provision of legal aid services (x2)
+FY2019 28000.6.03.154 -&gt; provision of legal aid services (x2)
+FY2019 41000.1.04.254 -&gt; 12835 | supervision of technical and voc (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>382 distinct programme(s) across 476 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 0509010 Teacher Management- Primary  201,136,266,225.0
+FY2025 0801000 Defence  169,815,800,000.0
+FY2025 0509020 Teacher management - Secondary  142,015,327,079.0
+FY2020 0801010 National Defense  119,808,049,600.0
+FY2025 0717000 General Administration Planning and Support   76,480,295,458.0
+FY2025 0202010 Construction of Roads and Bridges  72,318,898,073.0
+FY2025 0202030 Maintenance of Roads  69,536,000,000.0
+FY2025 0706020 Community Development  63,235,701,088.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>169 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0101010 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0101020 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0101040 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0101050 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0102010 -&gt; housing development and human settlement (x2)
+FY2020 0102030 -&gt; housing development and human settlement (x2)
+FY2020 0108010 -&gt; crop development and management (x2)
+FY2020 0108020 -&gt; crop development and management (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>953 distinct programme(s) across 1894 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G59" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>FY2025 13.010000 FAEDAH, DIVIDEN DAN LAIN-LAIN KENAAN BAYARAN  54,700,000,500.0
 FY2024 13.010000 INTEREST, DIVIDENDS AND OTHER DEBT CHARGES O  49,800,000,000.0
@@ -1669,41 +3966,41 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>142 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G60" s="2" t="n">
         <v>142</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>FY2022 21.040000 -&gt; agriculture sector reinvigoration and fo (x2)
 FY2022 28.020100 -&gt; transport connectivity and logistics mod (x2)
@@ -1713,6 +4010,147 @@
 FY2022 42.030000 -&gt; healthcare service delivery improvement (x2)
 FY2022 42.030000 -&gt; pandemic preparedness, disease control a (x2)
 FY2022 42.060300 -&gt; healthcare research (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>637 distinct programme(s) across 808 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 19.002 et Lille Da Pi, ja gien  6,994,664,737.0
+FY2018 19.001 die Ci 29, 9 28?  1,504,471,755.0
+FY2017 30.001 xixe"jin Ds sind ja sei?  1,490,542,683.0
+FY2017 6.3 And a great قوم  1,473,416,147.0
+FY2017 2.1 ing in  1,455,757,190.0
+FY2017 21.002 وفيد ؤونه قومه مادونه  1,334,531,645.0
+FY2017 19.003 ¿ ¿ iii  1,225,233,300.0
+FY2017 20.002 - pij, ;22 29,99  1,019,664,729.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
+FY2026 3.8 Program on Public Sector Personnel  429,643.3
+FY2026 7.2 Program on Management of Public Debt  421,864.4
+FY2025 3.8 Program on Public Sector Personnel  416,438.4
+FY2025 7.2 Program on Management of Public Debt  410,253.7
+FY2024 3.8 Program on Public Sector Personnel  403,992.0
+FY2023 3.8 Program on Public Sector Personnel  403,945.1
+FY2026 4.2 Strategic Program on Decentralization to the  377,960.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
+FY2023 5.7 -&gt; strategic program on supporting creation (x2)
+FY2023 6.2 -&gt; integrated program on digital government (x2)
+FY2024 2.12 -&gt; strategic program on innovation research (x2)
+FY2024 2.14 -&gt; strategic program on supporting developm (x2)
+FY2024 2.2 -&gt; integrated program on development of fut (x2)
+FY2024 2.8 -&gt; strategic program on development of digi (x2)
+FY2024 2.9 -&gt; strategic program on supporting strong a (x2)</t>
         </is>
       </c>
     </row>
@@ -1727,7 +4165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1767,7 +4205,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>malaysia</t>
+          <t>brazil</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -1781,6 +4219,139 @@
       </c>
       <c r="E2" s="2" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1812,7 +4383,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-16 13:33 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-16 18:20 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Currency from config, programme rows keyed by identity, trend labels
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -544,12 +544,13 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Brazil's PPA repeats a programme code under many budget strategies, each line carrying its own amount: in FY2024 code 0032 appears under 24 budget strategies with 24 different amounts, from 1.4 to 114,021.9. Every consumer keying on (year, programme) has to pick one line and they do not pick alike. build_final_panel keeps whichever it read last, so 'Sustainable Agriculture' (code 1144) took the 0.0 line rather than the 14,910.1 one and is reported unfunded. The Supabase view v_funding_by_program summed every line with that code instead. 22 of Brazil's 83 matched programme-years are affected. Brazil's mapped financing is therefore somewhere between 1,599,372.2 (one line per code) and 1,670,991.4 (every line with that code), or 30.0% to 31.4% of the national budget. Neither end has been checked against the document.</t>
+          <t>Brazil's PPA repeats a programme code under many budget strategies, each line carrying its own amount: in FY2024 code 0032 appears under 24 budget strategies with 24 different amounts, from 1.4 to 114,021.9. Every consumer keying on (year, programme) has to pick one line and they do not pick alike. build_final_panel keeps whichever it read last, so 'Sustainable Agriculture' (code 1144) took the 0.0 line rather than the 14,910.1 one and is reported unfunded. The Supabase view v_funding_by_program summed every line with that code instead. 22 of Brazil's 83 matched programme-years are affected. Brazil's mapped financing is therefore somewhere between 1,599,372.2 (one line per code) and 1,670,991.4 (every line with that code), or 30.0% to 31.4% of the national budget. Neither end has been checked against the document.
+Update 2026-08-17. The panel no longer hides this. build_final_panel keys every sheet on the budget row rather than on the programme code, and resolves an edge with the strategy_code the model itself named, so code 0032 under 24 different heads now attaches 24 different amounts instead of whichever row was read last. Brazil's mapped total rose from 1,599,372.2 to 1,610,412.5, the difference being rows that were previously overwritten. Two codes (1158 and 2801 in FY2024) still appear twice in funding_by_program because they genuinely are two programmes, and audit check A3 now fails on them. That failure is this issue surfacing rather than a new fault: A3 assumes a programme code is unique within a year, which in Brazil it is not.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>See F1 in FIXES.xlsx. The unit is (year, budget strategy, programme), not (year, programme). Stage 6 must record which budget strategy the matched line sits under, load_budget must key on all three, and the Supabase view must join on all three. Until then the dashboard shows the lower bound.</t>
+          <t>See F1 in FIXES.xlsx. The unit is (year, budget strategy, programme), not (year, programme). Stage 6 must record which budget strategy the matched line sits under, load_budget must key on all three, and the Supabase view must join on all three. Until then the dashboard shows the lower bound. The remaining work is upstream: stage 5 should emit a code that is unique within the year, at which point A3 passes on its own.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -3483,7 +3484,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>19 distinct programme(s) across 19 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+          <t>40 distinct programme(s) across 97 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
@@ -3495,10 +3496,10 @@
 FY2024 0905 Special operations: internal debt service (i  668,292.5
 FY2024 0903 OPERACOES ESPECIAIS: TRANSFERENCIAS CONSTITU  557,096.8
 FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIA  116,778.3
+FY2024 0032 Management and maintenance programme of the   114,021.9
 FY2024 0999 Contingency reserve  89,578.8
-FY2024 0906 Special operations: external debt service (i  46,080.6
-FY2024 0908 Special operations: refinancing of external   27,246.5
-FY2024 0902 Special operations: financing with return  26,568.8</t>
+FY2024 0032 Management and maintenance programme of the   77,570.6
+FY2024 0032 Management and maintenance programme of the   67,724.5</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3854,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>382 distinct programme(s) across 476 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+          <t>384 distinct programme(s) across 484 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
@@ -4383,7 +4384,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-16 18:20 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-17 06:43 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Issue register carries a category
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,18 +460,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,40 +483,45 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>CATEGORY</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>SEVERITY</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>COUNTRY</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>WHAT IT IS</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>WHY IT MATTERS</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>WHAT WOULD FIX IT</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FIRST SEEN</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>EVIDENCE</t>
         </is>
@@ -527,43 +533,48 @@
           <t>W1</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>brazil</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>A programme code is not unique within a fiscal year, so no figure keyed on (year, programme) is exact</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Brazil's PPA repeats a programme code under many budget strategies, each line carrying its own amount: in FY2024 code 0032 appears under 24 budget strategies with 24 different amounts, from 1.4 to 114,021.9. Every consumer keying on (year, programme) has to pick one line and they do not pick alike. build_final_panel keeps whichever it read last, so 'Sustainable Agriculture' (code 1144) took the 0.0 line rather than the 14,910.1 one and is reported unfunded. The Supabase view v_funding_by_program summed every line with that code instead. 22 of Brazil's 83 matched programme-years are affected. Brazil's mapped financing is therefore somewhere between 1,599,372.2 (one line per code) and 1,670,991.4 (every line with that code), or 30.0% to 31.4% of the national budget. Neither end has been checked against the document.
 Update 2026-08-17. The panel no longer hides this. build_final_panel keys every sheet on the budget row rather than on the programme code, and resolves an edge with the strategy_code the model itself named, so code 0032 under 24 different heads now attaches 24 different amounts instead of whichever row was read last. Brazil's mapped total rose from 1,599,372.2 to 1,610,412.5, the difference being rows that were previously overwritten. Two codes (1158 and 2801 in FY2024) still appear twice in funding_by_program because they genuinely are two programmes, and audit check A3 now fails on them. That failure is this issue surfacing rather than a new fault: A3 assumes a programme code is unique within a year, which in Brazil it is not.</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>See F1 in FIXES.xlsx. The unit is (year, budget strategy, programme), not (year, programme). Stage 6 must record which budget strategy the matched line sits under, load_budget must key on all three, and the Supabase view must join on all three. Until then the dashboard shows the lower bound. The remaining work is upstream: stage 5 should emit a code that is unique within the year, at which point A3 passes on its own.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>D1 in the detected sheet; FY2024 codes 0032, 0901, 0902, 0903, 0909, 0910, 1144, 1149</t>
         </is>
@@ -575,42 +586,47 @@
           <t>W11</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>jamaica, kenya</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>A budget layer can join perfectly and still be wrong, and the coverage figure is where it shows</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Kenya reported 824 of 985 programme-years unmatched and Jamaica 254 of 411, so almost none of either country's money mapped. The cause was not the mapping: combine_budget_years defaults to a 'hierarchical' code style that prefixes a bare programme code with its strategy, turning Kenya's 0101010 into 0101000.0101010 while the mapping keyed on 0101010. The same default had already broken Brazil's 524 edges and the repair is documented in the function's own docstring; nothing carried that lesson to the next country. Setting program_code_style to standalone took both to zero unmatched. That fix then exposed the real defect underneath. Kenya is sound: its programme rows sum to 1.00 times its printed head totals and it maps 67.9% of the budget. Jamaica is not: 2.79, 2.84 and 15.06 times, because its estimates print Budget 1 Recurrent and Budget 2 Capital for every head and only 23 head totals were captured against 208 programmes. Its coverage came out at 186.1%, which is the number that made the problem visible.</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Kenya needs nothing further. Jamaica needs stage 5 re-run with a structure hint that emits a total for every head, keeps recurrent and capital apart in the code, and ignores the object-of-expenditure detail. Until then its coverage figure should not be read. More generally, program_code_style should be chosen by measurement rather than defaulted: a code that never matches and a code that matches too much look identical until the totals are compared.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>run_report unmatched_codes 824 -&gt; 0 and 254 -&gt; 0; budget_all_years head totals against programme sums per year</t>
         </is>
@@ -622,42 +638,47 @@
           <t>W7</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>brazil, brunei</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Brazil's and Brunei's budget layers were extracted by a version of Prompt 5 that no longer exists</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Prompt 5 was amended on 2026-08-12 with rules 3a and 4a, which recover a programme whose table row wraps and whose amount is printed in the narrative instead, and which force a numbering check so a gap in the programme codes cannot pass. That edit found Thailand's missing 2.14 and 2.15 and closed a 36,964.5 reconciliation gap that had been recorded as intentional for weeks. Thailand was re-run under the new prompt. Brazil's budget extraction is from 2026-08-09 and Brunei's from 2026-08-10, so both are still under the old rule. Brunei's two unreconciled strategy-years (FY2025 strategy 1 short by 37.3, strategy 3 over by 1.8) are exactly the shape that edit was written to fix.</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>See F7 in FIXES.xlsx: re-run stage 5 for Brazil (2 documents) and Brunei (4), then rebuild both panels. Detector D12 now reports any output older than the prompt that produced it, so this cannot go unnoticed again.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>D12 in the detected sheet; D8 for Brunei's unreconciled years</t>
         </is>
@@ -669,42 +690,47 @@
           <t>W8</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>kiribati</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>A budget document can be the right document, parsed perfectly, and still extract nothing</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Kiribati cost $6.21 and produced no budget lines at all, in two different ways. First against the Recurrent Budget, which is the densest table in the whole set at 16.8 rows a page and whose rows are objects of expenditure: 219 Local catering, 227 External travel, 230 Cleaning. Nothing in it maps to a plan strategy. Then against the Development Budget, which IS the right document, is organised by KV20 pillar, carries project codes and titles, and parsed cleanly into 64 tables. It still returned nothing, because Table 7A has ten numeric columns of which six are years: Total Project Cost, Accumulated Balance, 2024 Budget, 2024 Revised, 2024 Warrant, 2024 Estimated Balance, 2025 Budget, 2026 Estimate. Prompt 5 assumes one amount column and a strategy total to reconcile against, and the ministry rows carry no totals. The first project has 4,427 under 2024 Warrant and nothing under 2025 Budget. The model returning an empty array is the correct answer to a question that was not asked properly.</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>See F8 in FIXES.xlsx. Two failure modes, two detectors, both now in document_shape.py: a LINE ITEMS verdict for a table whose rows are objects of expenditure, and a year-column count that says a fiscal-year column has to be named in the config before Prompt 5 sees the table.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>D12 and the shape probe; Files/llm/kiribati/kiribati_budget_*.xlsx, 0 rows each</t>
         </is>
@@ -716,42 +742,47 @@
           <t>W10</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>23 of 40 budget heads do not reconcile, because head totals and programme rows are attributed differently</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Malaysia's Estimated Expenditure took four rounds to extract at all: 71 programme rows on Prompt 5 as written, 120 at a 12,000-token chunk size, 939 once told where its three levels sit, and 691 after a code pattern dropped the five-digit objects of expenditure it kept emitting anyway. What remains is that its three head series - Maksud Bekalan, Pembangunan and Tanggungan - all number from 1, so a bare '1' merges three ministries' money. Telling the model to write B.62, P.6 and T.12 did not take. Rebuilding the code in Python from source_location is worse, not better: 6 heads reconcile instead of 17, because the head TOTAL is printed on a summary page whose location does not name the head while its programme rows do, so the two land under different keys. The programme rows themselves are correct; it is their attribution to a head that is unreliable.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Per-strategy coverage for Malaysia should not be read until this is fixed. The national total and the strategy inventory are unaffected, as is every mapping. The fix is to have Prompt 5 emit the head's short code as printed in the page corner (B.62), which is on every page of the document, and to reject a strategy_total whose source_location does not name a head.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>stage5_probe on FY2026: 731 lines, 25 reconciliation problems, 100 rows dropped by the code pattern</t>
         </is>
@@ -763,42 +794,47 @@
           <t>W9</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>bhutan, ghana, malaysia</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Four of seven candidate countries cannot be run on the budget documents we hold, each for a different reason</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>A stage 5 probe on one document per country, $4.10 in total, settled what three rounds of text heuristics could not. Kenya yields 631 programmes from 1,149 pages and Jamaica 208 from 706, both clean vote-to-programme hierarchies. Ghana yields zero: its FY2024 budget statement is a narrative policy document and the appropriations sit in an appendix file we hold for FY2015 only. Bhutan yields zero: its Budget Report is a fiscal analysis whose largest table is state-owned enterprise accounts, revenue, expenses and profit before tax, with no appropriations anywhere in it. Malaysia yields 71 programmes from 584 pages, correctly formed but far too few for a document of that size, so it is under-extracting rather than failing. Kiribati is W8. The pattern is that a country fails on its DOCUMENTS long before it fails on its prompts, and no amount of reading the text locally establishes which.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>See F9. Probe one document before committing a country: 02_Automation/stage5_probe.py, $0.15 to $2.64 a document against $8 to $48 a country. Ghana and Bhutan need their appropriation documents sourced; Malaysia needs its under-extraction diagnosed before it is worth $48.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Files/llm/_probe/*.xlsx; Kenya 631 programmes, Jamaica 208, Malaysia 71, Ghana 0, Bhutan 0, Kiribati 0</t>
         </is>
@@ -810,42 +846,47 @@
           <t>W2</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Strategies are tagged with risks they do not respond to</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Brazil's 'National Defense' carries Democratic Backsliding and Shifts in Globalisation. It is a standing function of the state funded every year, not a response to either risk. The tagging keys on topical adjacency rather than on the plan claiming the strategy addresses the risk, which inflates every risk chart on every page. It passes every arithmetic check because the tags are internally consistent, and it is invisible to source-fidelity checking because no figure is wrong. Three Brazilian and three Bruneian strategies carry five or more of the eleven risks.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>See F2 in FIXES.xlsx. Prompt 4 must require a quotation from the strategy's own text for each risk it names, and must not tag a standing function on sector adjacency alone. Re-running stage 4 changes related_risks, risk_salience and every risk view downstream.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
         </is>
@@ -857,42 +898,47 @@
           <t>W3</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Strategies that entered the panel from the budget document rather than from the plan</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Two Bruneian strategies ('Purchase of medicines, medical consumables and laboratory testing needs' and 'Payment for medical treatment services at Gleneagles Jerudong') carry no component intervention and cite no plan paragraph. They are budget line names that reached the strategy inventory. Their funding is real money attributed to something the plan never asked for, and they sit in the same column as strategies the plan does state.</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>See F3 in FIXES.xlsx. Brunei's plan text is a speech, so stage 3 recovers little from it and stage 4 fills the gap from the budget side. The transcript prompt is the fix; until it exists these rows should be excluded from any count of plan strategies rather than silently included.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
         </is>
@@ -904,42 +950,47 @@
           <t>W6</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Four Bruneian strategies carry the untraceable flag and in all four the name they cannot find in the plan is the name of the budget programme funding them. The mechanism is now proved rather than suspected: run_stage4 hands Prompt 4 the list of budget programme codes and names as its target granularity (the buckets block). Brunei's stage 3 produced 1,077 interventions from the three NDP documents and not one of them mentions Gleneagles, medicines or research costs, while 'Gleneagles' appears in the budget speech and in no NDP. Short of plan material, the model took bucket names and emitted them as strategies. Two carry no component intervention at all; two carry a component whose name is also the budget line's. Stage 6 then matched each to the programme whose name it is, so the match is correct as a string and empty as evidence, and the rationale is the model explaining why a name matches itself.</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
         </is>
@@ -951,42 +1002,47 @@
           <t>W4</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>brunei</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>One usable budget year out of four documents</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Only FY2025 produced a budget layer. Nothing on Brunei can show a trend, its 97.4% of budget mapped rests on a single speech, and three strategy-years carry the whole reconciliation.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>See F3 in FIXES.xlsx, the same transcript prompt.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>D10 in the detected sheet</t>
         </is>
@@ -998,42 +1054,47 @@
           <t>W5</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>all</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>A programme-strategy pair matched twice, once by each pass</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>54 Thailand pairs, 53 Brazil, 2 Brunei carry two rationales because the strategy pass and the reverse pass both reached them. The panel credits the pair once and the money is right. It only misleads if something counts rows and calls them edges, which the union dashboard did until the tile was split into pairs and rows.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Nothing to fix in the data. Any new consumer must count pairs, not rows.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>D9 in the detected sheet; the 'twice' filter in the audit view</t>
         </is>
@@ -1045,42 +1106,47 @@
           <t>W12</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>maldives</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Document Intelligence renders the Maldives budgets as Arabic, not Thaana, so the programme names reaching the model are already gibberish</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Corrected 2026-08-16. This is a parsing failure, not a prompt failure. The FY2017 PDF holds 342,715 Thaana characters when read with a plain local extractor. The cached Document Intelligence markdown for the same file holds ZERO Thaana characters and 159,753 Arabic ones: DI mapped Thaana glyphs onto Arabic codepoints. Thaana and Arabic are both right-to-left and Thaana takes its diacritics from Arabic forms, which is the likely cause. The model therefore never saw Dhivehi and could only produce noise: 509 of 852 programme rows have no readable name. Proof that the prompt is not the problem: a rewritten hint demanding translation over transliteration returned names byte-identical to the previous run, while correctly fixing currency_unit to MVR million, which is the one field that does not depend on the script.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Do not spend on another stage 5 run until the parse is fixed; no prompt can recover text the parser destroyed. Document Intelligence has no locale for Dhivehi. The options are to parse these documents outside DI with a Thaana-capable extractor and accept the loss of table structure, or to treat Maldives as out of scope for the current toolchain. The translation hint is left in the config so it applies once the text arrives intact.</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>02_Automation/cache/di_&lt;hash&gt;.json for the FY2017 budget: 0 Thaana, 159,753 Arabic; pypdf on the same file: 342,715 Thaana</t>
         </is>
@@ -1092,42 +1158,47 @@
           <t>W13</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>kenya, fiji, jamaica, maldives, brunei</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>A printed strategy total smaller than the programmes beneath it, which surfaces as a ceiling failure once enough of them are matched</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>The ceiling test asks whether the matched programmes under a budget strategy sum to more than that strategy's own printed total. Ten strategy-years now fail across five countries, and in each the budget layer is inconsistent with itself before any edge is considered: Kenya FY2020 strategy 1014000 prints a total of 0 against programmes of 7,655,824,962, Kenya FY2025 strategy 0710000 prints 2,000,000 against 4,065,815,260, Maldives FY2017 strategy 5 prints 35,615,361 against 431,283,126, and Fiji FY2018 strategies 2, 3 and 21 print totals 9,629.0, 4,000.0 and 23,253.9 below their programme sums. Three more (Fiji FY2017 strategy 25, Fiji FY2018 strategy 34, Brunei FY2025 strategy 3) are rounding at 0.1 to 1.8 and are not real. The failures are not caused by the mapping: for every one of them the strategy-side pass alone already exceeded the total, so improving coverage only made a pre-existing extraction defect visible.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Stage 5, not stage 6. Have the extraction emit a total for every strategy and reconcile it against its own programme rows before the layer is written, so the contradiction is caught where it is created. Until then read the ceiling sheet as a report on the budget layer rather than on the edges, and treat a rounding-scale exceedance separately from a structural one.</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx ceiling sheet, status EXCEEDS TOTAL; audit_checks A4</t>
         </is>
@@ -1139,42 +1210,47 @@
           <t>W14</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>kenya, jamaica, brazil</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>The strategy inventory holds the same strategy twice, once bare and once prefixed with its budget code</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Kenya's inventory carries 22 strategies in both forms ('E-Government Services' and '0217000 | E-Government Services'), Jamaica 2 and Brazil 1. Both forms reach the panel as separate strategies, so each affected strategy is counted twice in every denominator the dashboard shows, including the share of strategies funded. It also breaks the reverse pass: the join cannot tell the two apart on the bare name, so it refuses rather than guessing, which is how Brazil lost the edge for 'Protection and Recovery of Biodiversity and Combating Deforestation'.</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Consolidate in stage 4, which is where the two forms are created. Pending that, de-duplicate in a strategyclean hygiene pass keeping the bare form, which costs nothing and corrects the denominators now.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Files/llm/&lt;slug&gt;/&lt;slug&gt;_strategyclean.xlsx; the ambiguous-join drops logged by stage 6b</t>
         </is>
@@ -1186,42 +1262,47 @@
           <t>W15</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>malaysia, brazil</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Stage 6 is shown only one programme per repeated code, so most of the budget was never a candidate for matching</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>run_stage6 builds its set of valid targets as {program_code: row} (stages.py:611). Where a bare programme code repeats within a year, that dict keeps only the LAST row, and every earlier one becomes unmatchable. Malaysia loses 2,166 of 2,815 programme rows this way (77%), Brazil 159 of 347 (46%), Kenya 8 of 985, and no other country is affected. It is worse than an omission: validate_stage6 then overwrites the edge's strategy_code and strategy_name from the single retained row (schemas.py:243-244), discarding the head the model itself named, so a matched edge is attributed to whichever ministry happened to be last in the file. In Malaysia FY2024, 93 of 127 codes sit under more than one head, yet not one mapping edge cites more than one head for a code, which is the signature of the collapse rather than of the budget.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Fixed. schemas.build_programme_index keys the candidate set on both the bare code and (strategy_code, program_code), and resolve_programme demands the head only where the code is genuinely ambiguous. validate_stage6 now uses the model's own strategy_code to disambiguate before replacing it with the matched row's. build_final_panel.ProgrammeLookup resolves the same way and additionally joins a bare mapping code to a hierarchical layer code. Stage 6 was replayed from cache for Malaysia: 1,566 edges now resolve where 0 did, only 3 records across five years still cannot be placed, and Malaysia's mapped share went from 0.0% to 86.9%. Brazil's colliding codes are unchanged and remain W1: the panel still takes the last row for a repeated code, because only the merge loop knows the head and the sheets built afterwards would disagree with it.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>stages.py:611; schemas.py:243-244; Files/llm/malaysia/malaysia_budget_*.xlsx vs mappings/</t>
         </is>
@@ -1233,45 +1314,518 @@
           <t>W16</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>jamaica</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Stage 5 returned one programme per Head; now extracted deterministically from the Head summary tables</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Counted from the Document Intelligence markdown for FY2024: the per-Head summary tables contain 162 programme rows across 59 Heads, and stage 5 returns 59. It emits the Head's own code as the programme code, so one row survives per Head. Three different structure hints were tried, including one written from the markdown itself, and all three returned 59. Reducing the chunk size to 12,000 cost three times as much and returned 59.
 An earlier note in this register said the repeated name 'Executive Direction and Administration' was an extraction artefact. It is not. That programme genuinely appears 39 times in FY2024, once under most ministries, and the document really does have only 72 distinct programme names. Jamaica's unresolved recall is therefore mostly a real property of its budget, where much of the money sits in ministry administration that the overhead rule correctly refuses to match, and only partly this under-extraction.</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Fixed, and not by a prompt. extract_budget_tables.py reads the per-Head summary tables straight from the parsed markdown, where a programme row is the one whose first cell begins with two numbers. The rule is regexes in jamaica.json under 'budget_tables'; the script itself holds no country logic. The layer went from 172 programme rows to 341, edges from 92 to 399, strategies with no budget from 68 to 7, and the mapped share from 6.8% to 91.3%. Recall resolves at 66% where it could not be estimated at all. One trap for the next document: codes must be digits-and-dots, because _clean_code keeps only \d+(\.\d+)* and silently trimmed the first hyphenated attempt back to the Head.</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>FIXED</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>01_Pipeline/scripts/extract_budget_tables.py; 02_Automation/inputs/jamaica.json budget_tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>W17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>The shared mapping prompt hard-codes one country's overhead vocabulary</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>6_mapping.txt lists seven programme-name fragments to refuse as overhead ("Supporting Creation of", "Fundamental Program on", "Replenishment of Treasury" and four more). They match 69 of Thailand's 273 programme names and ZERO across the other seven countries. Every country pays the tokens and takes the instruction, and for seven of them it describes programmes that do not exist, which is a bias in the matching with no upside.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Move the list into the per-country profile as an overhead_names key and leave the shared prompt describing the CLASS of thing to refuse rather than one country's wording. It invalidates the stage 6 cache, so it should ride with the next deliberate prompt change rather than on its own.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/prompts/6_mapping.txt L50-55</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>W18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>precision-recall</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Precision has never been measured, so only one side of the trade-off has a number</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Mapping recall is estimated per country. Of the edges the panel does contain, the share that are real is unknown, and nothing in the pipeline has ever been labelled by a person. Files/outputs/precision_sample.csv holds a stratified sample drawn for exactly this and every verdict cell is empty. Without it, any threshold on match quality would be set in units nobody has measured.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Mark about 100 edges in the union dashboard's Audit tab and run precision_labels.py, which reports precision by pass and by programme_breadth. If either separates good edges from bad, the dial already exists in fields on disk and no new paid field is needed.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Files/outputs/precision_sample.csv; 01_Pipeline/scripts/precision_labels.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>W19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>precision-recall</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>The reverse pass carries the same precision clamp as the forward pass it exists to correct</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>6b_programme_coverage.txt states in its own header that it exists to fix recall, and config.py calls it the recall lever. It then repeats the forward pass's instruction verbatim: "Precision (false positives are worse than false negatives)". The one counterweight is a basket-completeness paragraph. Whether the clamp is binding has never been tested.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Remove that line from 6b only and re-run one country, diffing against the coverage workbook already on disk. Jamaica was the obvious candidate until its budget turned out to be genuinely administration-heavy; Fiji is the cleaner test. Gated on W18, because without precision numbers a rise in edges cannot be read either way.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/prompts/6b_programme_coverage.txt L48-51</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>W20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>precision-recall</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Every recall figure is a ceiling, because the two passes are not independent</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Capture-recapture assumes the two captures are independent. Stage 6 and stage 6b use the same model, the same prompt family and the same extracted data, so an edge obvious to one is usually obvious to the other. That inflates the overlap, shrinks the estimated population and overstates recall. Fiji and Brazil clear the degeneracy guard only barely, so their 95% and 90% are near-subset artefacts and should not be quoted.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Run the reverse pass on a different model so the passes stop sharing one. Measured at roughly $30 to $35 across the fleet against $6 to $7 today, so it is worth doing once for the number rather than routinely.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/scripts/precision_recall.py L28-33</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>W21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Per-country settings are split across two config files that must agree, and nothing checks</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>A country is described twice: 02_Automation/inputs/&lt;slug&gt;.json for the LLM run and 01_Pipeline/countries/&lt;slug&gt;.json for the deterministic one. Eight knobs describe the same budget document across the two, applied at three different stages, and program_code_style in one has to be consistent with budget_tables and budget_program_code_take in the other. Three currency_unit values said million where the data was absolute and survived precisely because nothing read them.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>One document profile per country, in one file, with four mechanisms: how to read it, where the levels sit, how the codes are shaped, and how the amounts are labelled. The code is already generic; it is the configuration that is scattered.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>02_Automation/inputs/*.json; 01_Pipeline/countries/*.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>W22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>The intern pack ships a stale copy of the pipeline it is meant to hand over</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>05_Handoff/handoff/ carries its own copy of four pipeline scripts and the seven prompts so it can be sent on its own. They were copied by hand and nothing has compared them since. build_analytics_html.py is 811 lines behind, run_pipeline.py 361, and Prompt 5 is 14. Every difference is the pipeline moving ahead, so an intern following the pack reproduces bugs fixed months ago.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Decide whether the pack is maintained or retired. If maintained, generate it rather than copying it, which needs the pack's dependency set worked out because the live runner reaches for validators the pack does not have. check_handoff_drift.py measures the gap in the meantime.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>05_Handoff/scripts/check_handoff_drift.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>W23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Seven implementations of one list parser, and they do not agree</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>related_risks and the other multi-value columns are written in three shapes: semicolon-joined, a bare single value, and a raw JSON array from stage 4 that reaches the matches sheet in 657 rows and strategyclean in 1,009. Seven functions across the repo parse them and six handle all three. publish_run.as_list did not, and returned the whole bracketed string as one item.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Fixed in publish_run. The duplication is not: one parser in validation_common, imported by the rest, would make a fourth shape a one-place change instead of a seven-place hunt.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>03_Ingest_and_Publishing/scripts/publish_run.py as_list</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>W24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>A crashed stage reported as ok, and the run carried on from the previous panel</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>run_stage treated exit 1 as "ran" for every stage, because build_final_panel documents that code as "written, and QA found something". Only that script has the contract. A traceback in any stage read as ok, the guard on the next stage passed, and the dashboard was rebuilt from the panel still on disk. It bit twice in one session and both times the audit output looked healthy because it was reading the stale panel.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Fixed: only the script documenting that contract gets it, and never with a traceback in its output.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/scripts/run_pipeline.py run_stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>W25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>publishing</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>brazil, kenya</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>The database view joins programmes on their code alone</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>v_funding_by_program joins budget_lines to matches on (run_id, fiscal_year, program_code). Where a code repeats under several heads the join crosses them, so the view disagrees with the panel for the two countries where that happens. The dashboard works around it by reading the edges instead, which is why the page and the panel now agree, but the view is still wrong for anyone querying it directly.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Add budget_strategy_code to the join. The column is already published on matches, so it is a migration and no re-run.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>03_Ingest_and_Publishing/supabase/migrations/0001_init.sql L179</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1344,38 +1898,703 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>28 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 programme 0032: 1.4 and 77.9 and 331.9 and 469.5 and 633.9 and 756.5 and 850.8 and 904.4 and 1,021.0 and 1,192.6 and 1,532.3 and 1,607.8 and 1,809.5 and 1,853.5 and 2,003.2 and 3,005.3 and 3,497.2 and 5,553.3 and 10,446.6 and 10,768.5 and 30,770.3 and 67,724.5 and 77,570.6 and 114,021.9  (under budget strategies 03, 04, 05, 06, 07, 08, 09, 10, 11, 12, 13, 14, 15, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28)
+FY2024 programme 0901: 1,984.7 and 64,985.7  (under budget strategies 28, 99)
+FY2024 programme 0902: 216.8 and 500.0 and 2,000.0 and 6,362.3 and 6,415.9 and 26,568.8 and 27,153.3  (under budget strategies 05, 11, 12, 19, 20, 23, 28)
+FY2024 programme 0903: 2,007.3 and 557,096.8  (under budget strategies 09, 28)
+FY2024 programme 0909: 0.0 and 0.3 and 0.8 and 5.3 and 149.6 and 246.0 and 1,502.0 and 116,778.3  (under budget strategies 04, 07, 12, 19, 23, 25, 26, 28)
+FY2024 programme 0910: 0.1 and 0.7 and 4.4 and 1,525.5  (under budget strategies 10, 14, 26, 28)
+FY2024 programme 1144: 0.0 and 14,910.1  (under budget strategies 20, 28)
+FY2024 programme 1149: 20.2 and 54.2  (under budget strategies 04, 14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brazil/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>brazil_budget_2021.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12
+brazil_budget_2024.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Green Building initiatives under the 12th Na &lt;- named after budget line Green Building initiatives under the 12th Na
+Infrastructure provision for enhancement of  &lt;- named after budget line Preparation and upgrading works for infrastr
+Research costs for public higher education i &lt;- named after budget line Research costs for public higher education i</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brunei/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>4 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>brunei_budget_2021.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2022.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2025.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2026.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no plan text behind it</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) cite no component intervention and no plan paragraph. A strategy the plan does not state is a strategy that entered from the budget side, and its funding is money attributed to something the plan never asked for.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Payment for medical treatment services at Gleneagles Jerudong Park Med
+Purchase of medicines, medical consumables and laboratory testing need</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 reconciliation_mismatch 1: programs sum to 1,912.5 but strategy_total is 1,949.8 (gap 37.3) - a program line is likel
+FY2025 reconciliation_mismatch 3: programs sum to 626.7 but strategy_total is 624.9 (gap -1.8) - a program line is likely mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 strategy 1: printed 1,949.8, programmes sum to 1,912.5, apart by 37.3
+FY2025 strategy 3: printed 624.9, programmes sum to 626.7, apart by -1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>28 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 22: programs sum to 321,245.4 but strategy_total is 321,245.6 (gap 0.2) - a program line is li
+FY2017 reconciliation_mismatch 24: programs sum to 113,354.0 but strategy_total is 113,354.1 (gap 0.1) - a program line is li
+FY2017 reconciliation_mismatch 25: programs sum to 23,096.7 but strategy_total is 23,096.6 (gap -0.1) - a program line is lik
+FY2017 reconciliation_mismatch 33: programs sum to 28,538.8 but strategy_total is 42,329.9 (gap 13,791.1) - a program line is
+FY2017 reconciliation_mismatch 40: programs sum to 133,737.9 but strategy_total is 134,178.0 (gap 440.1) - a program line is 
+FY2017 reconciliation_mismatch 50: programs sum to 615,572.2 but strategy_total is 628,116.8 (gap 12,544.6) - a program line 
+FY2017 reconciliation_mismatch 52: programs sum to 364,701.0 but strategy_total is 354,607.9 (gap -10,093.1) - a program line
+FY2018 reconciliation_mismatch 2: programs sum to 23,891.3 but strategy_total is 14,262.3 (gap -9,629.0) - a program line is</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>28 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 22: printed 321,245.6, programmes sum to 321,245.4, apart by 0.2
+FY2017 strategy 24: printed 113,354.1, programmes sum to 113,354.0, apart by 0.1
+FY2017 strategy 25: printed 23,096.6, programmes sum to 23,096.7, apart by -0.1
+FY2017 strategy 33: printed 42,329.9, programmes sum to 28,538.8, apart by 13,791.1
+FY2017 strategy 40: printed 134,178.0, programmes sum to 133,737.9, apart by 440.1
+FY2017 strategy 50: printed 628,116.8, programmes sum to 615,572.2, apart by 12,544.6
+FY2017 strategy 52: printed 354,607.9, programmes sum to 364,701.0, apart by -10,093.1
+FY2018 strategy 2: printed 14,262.3, programmes sum to 23,891.3, apart by -9,629.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>74 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 reconciliation_mismatch 01000: programs sum to 83,000.0 but strategy_total is 290,111.0 (gap 207,111.0) - a program line 
+FY2019 reconciliation_mismatch 08000: programs sum to 642,858.0 but strategy_total is 469,975.0 (gap -172,883.0) - a program lin
+FY2019 reconciliation_mismatch 09000: programs sum to 712,147.0 but strategy_total is 833,920.0 (gap 121,773.0) - a program line
+FY2019 reconciliation_mismatch 15010: programs sum to 0.0 but strategy_total is 697,424.0 (gap 697,424.0) - a program line is li
+FY2019 reconciliation_mismatch 15020: programs sum to 900,480.0 but strategy_total is 10,480.0 (gap -890,000.0) - a program line
+FY2019 reconciliation_mismatch 16049: programs sum to 489,234.0 but strategy_total is 225,234.0 (gap -264,000.0) - a program lin
+FY2019 reconciliation_mismatch 17000: programs sum to 6,345,325.0 but strategy_total is 11,525,361.0 (gap 5,180,036.0) - a progr
+FY2019 reconciliation_mismatch 19046: programs sum to 1,085,718.0 but strategy_total is 1,078,318.0 (gap -7,400.0) - a program l</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>74 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 strategy 01000: printed 290,111.0, programmes sum to 83,000.0, apart by 207,111.0
+FY2019 strategy 08000: printed 469,975.0, programmes sum to 642,858.0, apart by -172,883.0
+FY2019 strategy 09000: printed 833,920.0, programmes sum to 712,147.0, apart by 121,773.0
+FY2019 strategy 15010: printed 697,424.0, programmes sum to 0.0, apart by 697,424.0
+FY2019 strategy 15020: printed 10,480.0, programmes sum to 900,480.0, apart by -890,000.0
+FY2019 strategy 16049: printed 225,234.0, programmes sum to 489,234.0, apart by -264,000.0
+FY2019 strategy 17000: printed 11,525,361.0, programmes sum to 6,345,325.0, apart by 5,180,036.0
+FY2019 strategy 19046: printed 1,078,318.0, programmes sum to 1,085,718.0, apart by -7,400.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>7 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 programme 0106000: 346,691,310.0 and 364,590,743.0  (under budget strategies 1094, 1095)
+FY2025 programme 0207000: 231,885,786.0 and 278,922,194.0  (under budget strategies 1122, 1123)
+FY2025 programme 0412000: 651,366,934.0 and 16,529,119,104.0  (under budget strategies 1082, 1083)
+FY2025 programme 0508000: 297,799,258.0 and 435,378,299.0 and 4,677,027,195.0  (under budget strategies 1064, 1065, 1066)
+FY2025 programme 0709000: 233,471,082.0 and 444,125,877.0  (under budget strategies 1072, 1213)
+FY2025 programme 0710000: 2,000,000.0 and 8,769,275,002.0  (under budget strategies 1072, 1213)
+FY2025 programme 1018000: 30,500,000.0 and 12,916,448,407.0  (under budget strategies 1331, 1332)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Promotion and Development of MSMEs &lt;- named after budget line MSMEs Development and Promotion
+Product and Market Development for MSMEs &lt;- named after budget line Market Linkages for MSMEs</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>8 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 reconciliation_mismatch 0106000: programs sum to 349,247,063.0 but strategy_total is 276,081,719.0 (gap -73,165,344.0) - a 
+FY2020 reconciliation_mismatch 0508000: programs sum to 2,991,357,360.0 but strategy_total is 164,025,309.0 (gap -2,827,332,051.0)
+FY2020 reconciliation_mismatch 1014000: programs sum to 7,655,824,962.0 but strategy_total is 0.0 (gap -7,655,824,962.0) - a progr
+FY2020 reconciliation_mismatch 1018000: programs sum to 10,066,601,747.0 but strategy_total is 10,873,301,747.0 (gap 806,700,000.0
+FY2025 reconciliation_mismatch 0106000: programs sum to 418,347,116.0 but strategy_total is 346,691,310.0 (gap -71,655,806.0) - a 
+FY2025 reconciliation_mismatch 0508000: programs sum to 3,536,217,818.0 but strategy_total is 435,378,299.0 (gap -3,100,839,519.0)
+FY2025 reconciliation_mismatch 0709000: programs sum to 234,021,081.0 but strategy_total is 233,471,082.0 (gap -549,999.0) - a pro
+FY2025 reconciliation_mismatch 0710000: programs sum to 4,177,242,813.0 but strategy_total is 2,000,000.0 (gap -4,175,242,813.0) -</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 strategy 0106000: printed 276,081,719.0, programmes sum to 349,247,063.0, apart by -73,165,344.0
+FY2020 strategy 0508000: printed 164,025,309.0, programmes sum to 2,991,357,360.0, apart by -2,827,332,051.0
+FY2020 strategy 1014000: printed 0.0, programmes sum to 7,655,824,962.0, apart by -7,655,824,962.0
+FY2020 strategy 1018000: printed 10,873,301,747.0, programmes sum to 10,066,601,747.0, apart by 806,700,000.0
+FY2025 strategy 0106000: printed 346,691,310.0, programmes sum to 418,347,116.0, apart by -71,655,806.0
+FY2025 strategy 0508000: printed 435,378,299.0, programmes sum to 3,536,217,818.0, apart by -3,100,839,519.0
+FY2025 strategy 0709000: printed 233,471,082.0, programmes sum to 234,021,081.0, apart by -549,999.0
+FY2025 strategy 0710000: printed 2,000,000.0, programmes sum to 4,177,242,813.0, apart by -4,175,242,813.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>138 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>138</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>FY2022 reconciliation_mismatch 1: programs sum to 19,215,800.0 but strategy_total is 13,533,000.0 (gap -5,682,800.0) - a pro
 FY2022 reconciliation_mismatch 10: programs sum to 3,621,353,400.0 but strategy_total is 5,254,500.0 (gap -3,616,098,900.0) -
@@ -1388,41 +2607,41 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>D8</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>A strategy total its own programmes do not add up to</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / reconciliation</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>138 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>138</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>FY2022 strategy 1: printed 13,533,000.0, programmes sum to 19,215,800.0, apart by -5,682,800.0
 FY2022 strategy 2: printed 1,337,000.0, programmes sum to 2,500,000.0, apart by -1,163,000.0
@@ -1435,41 +2654,928 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>52 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 1: programs sum to 371,971,798.0 but strategy_total is 101,334,724.0 (gap -270,637,074.0) - a
+FY2017 reconciliation_mismatch 10: programs sum to 603,169,808.0 but strategy_total is 35,391,792.0 (gap -567,778,016.0) - a 
+FY2017 reconciliation_mismatch 11: programs sum to 84,903,354.0 but strategy_total is 59,843,651.0 (gap -25,059,703.0) - a pr
+FY2017 reconciliation_mismatch 12: programs sum to 0.0 but strategy_total is 6,993,896.0 (gap 6,993,896.0) - a program line i
+FY2017 reconciliation_mismatch 13: programs sum to 0.0 but strategy_total is 3,626,872.0 (gap 3,626,872.0) - a program line i
+FY2017 reconciliation_mismatch 14: programs sum to 0.0 but strategy_total is 9,198,520.0 (gap 9,198,520.0) - a program line i
+FY2017 reconciliation_mismatch 15: programs sum to 0.0 but strategy_total is 4,223,952.0 (gap 4,223,952.0) - a program line i
+FY2017 reconciliation_mismatch 16: programs sum to 0.0 but strategy_total is 44,828,700.0 (gap 44,828,700.0) - a program line</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>52 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 1: printed 101,334,724.0, programmes sum to 371,971,798.0, apart by -270,637,074.0
+FY2017 strategy 2: printed 208,402,975.0, programmes sum to 1,780,849,664.0, apart by -1,572,446,689.0
+FY2017 strategy 3: printed 10,854,474.0, programmes sum to 291,704,544.0, apart by -280,850,070.0
+FY2017 strategy 4: printed 367,654,006.0, programmes sum to 952,692,855.0, apart by -585,038,849.0
+FY2017 strategy 5: printed 35,615,361.0, programmes sum to 796,853,288.0, apart by -761,237,927.0
+FY2017 strategy 6: printed 19,009,362.0, programmes sum to 2,294,511,756.0, apart by -2,275,502,394.0
+FY2017 strategy 7: printed 22,661,255.0, programmes sum to 266,705,093.0, apart by -244,043,838.0
+FY2017 strategy 8: printed 27,923,748.0, programmes sum to 494,853,833.0, apart by -466,930,085.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
+FY2024 0151 Protection of indigenous lands, territorial management and e
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIAIS
+FY2024 1144 AGROPECUARIA SUSTENTAVEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2801 | Neo-industrialization, Business Envir -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Reconstruction, Expansion and Deepening of S -&gt; 5 risks: Climate Change, Democratic Backsliding, Environmental Degradation and Pollution,
+Public Security with Citizenship -&gt; 6 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>1 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>4101 | Public and Government Communication</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Development of school and higher education i -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Management of infectious disease crises and  -&gt; 5 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
+Natural disaster management -&gt; 5 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>25 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Construction programme for sewerage and waste drainage infrastructure 
+National security, defence and public safety infrastructure
+Public sector performance and welfare data systems
+Road and bridge infrastructure modernisation programme
+Social welfare, community and civic facilities development
+Environmental regulation and impact assessment enforcement
+Integrated industrial diversification, FDI and MSME competitiveness st
+Industrial and business site infrastructure provision</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>1 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 30.5 Land Drainage and Flood Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>23 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>43.1 | Roads, Bridges and Jetties -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+21.2 | Primary Education -&gt; 6 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
+20.1 | Fiji Police -&gt; 6 risks: Democratic Backsliding, Demographic Shifts, Environmental Degradation and Pollut
+22.2 | Health Services -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan
+24.2 | Social Welfare -&gt; 5 risks: Climate Change, Demographic Shifts, Resource and Energy Pressures, Shifts in Glo
+35.1 | Sugar Development -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Res
+Department of Tourism -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+16.3 | Department of Communication -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>5 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>50.6 | Standard Expenditure Group 6
+227 | Public-Private Partnership Infrastructure and Service Delivery E
+102 | Financial Sector Modernisation and Inclusion Measures
+Audio-Visual Industry Development
+18.1 | Policy and Administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>20 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 program_missing_in_year 23: program '23.2' (Housing) exists in ['2018', '2019'] but is absent in ['2017'] - check whet
+FY2017 program_missing_in_year 26: program '26.1' (Higher Education Institutions) exists in ['2018', '2019'] but is absent in
+FY2017,2018 program_missing_in_year 13: program '13.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '2
+FY2017,2018 program_missing_in_year 34: program '34.6' (Micro, Small and Medium Enterprises Central Coordinating Agency) exists in
+FY2017,2018 program_missing_in_year 4: program '4.3' (Public Enterprises) exists in ['2019'] but is absent in ['2017', '2018'] - 
+FY2017,2018 program_missing_in_year 9: program '9.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '20
+FY2018,2019 program_missing_in_year 18: program '18.4' (Rehabilitation and Rural Housing) exists in ['2017'] but is absent in ['20
+FY2018,2019 program_missing_in_year 30: program '30.5' (Land Drainage and Flood Protection) exists in ['2017'] but is absent in ['</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>1 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Health service delivery and public health pr -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>7 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Praedial Larceny Prevention Co- ordination
+10576 | Vision 2030 Jamaica National Development Plan
+10662 | International Programme Management
+10572 | Support for Development Planning
+Anti-Dumping and Subsidies
+Maritime Organizations
+Support for Growth Inducement Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>200 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2019 program_missing_in_year 03000: program '03000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.157' (Government Audit Services) exists in ['2022', '2024'] but is abs
+FY2019 program_missing_in_year 06000: program '06000.1.03.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 06000: program '06000.1.03.158' (Public Service Personnel Management) exists in ['2022', '2024'] 
+FY2019 program_missing_in_year 07000: program '07000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 07000: program '07000.1.99.139' (Protection of Children's Rights) exists in ['2022', '2024'] but 
+FY2019 program_missing_in_year 07000: program '07000.1.99.159' (Combatting Human Trafficking) exists in ['2022', '2024'] but is </t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0105060 NAMATA
+FY2020 0120040 Fisheries Research &amp; Development
+FY2020 0620020 Police Vetting
+FY2020 0703050 Coordination of Vision 2030
+FY2020 0712050 Finance Management Services
+FY2020 0715060 International Relations and Cooperation
+FY2020 0733040 Peace and Conflict Management
+FY2020 0740010 Government Clearing Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>12 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>0610000 | Dispensation of Justice -&gt; 5 risks: Climate Change, Democratic Backsliding, Increased Polarisation, Pandemics, Techn
+Foreign Relation and Diplomacy -&gt; 7 risks: Biodiversity Loss, Climate Change, Democratic Backsliding, Environmental Degrada
+0111000 | Fisheries Development and Manageme -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Promotion and Development of MSMEs -&gt; 5 risks: Climate Change, Demographic Shifts, Resource and Energy Pressures, Shifts in Glo
+0320000 | Industrial Promotion and Developme -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Product and Market Development for MSMEs -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Standards and Qualitry Infrastucture &amp; Resea -&gt; 5 risks: Climate Change, Environmental Degradation and Pollution, Resource and Energy Pre
+Agricultural Research &amp; Development -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>NAMATA
+0706060 | Infrastructure, science, technology and innovation
+0629000 | General Administration and Support Services
+0304010 | Governance and Accountability
+0309010 | Promotion of Local Content
+0215030 | General Administration and Support Services
+National Health Procurement Board Establishment
+Perishable Goods Storage and Export Facilitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>470 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
+FY2020 blank_amount 0120000: amount is blank/unparseable.
+FY2020 blank_amount 0620000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0712000: amount is blank/unparseable.
+FY2020 blank_amount 0715000: amount is blank/unparseable.
+FY2020 blank_amount 0733000: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Programme lines carrying zero</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / budget_all_years</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>36 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G39" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>FY2022 28.030600 Maintenance, Repair and Overhaul (KTMB)
 FY2022 28.031000 Maintenance of the AwAS System
@@ -1482,41 +3588,41 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>D4</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Strategy tagged with five or more risks</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>25 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G40" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Healthcare Service Delivery Improvement -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
 National security, border management and def -&gt; 7 risks: Climate Change, Democratic Backsliding, Demographic Shifts, Increased Polarisati
@@ -1529,41 +3635,41 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>D5</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Strategy with no budget in any year</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>17 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G41" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Bumiputera Socioeconomic Empowerment
 Fiscal Institutions Strengthening and Budget Management Improvement
@@ -1576,41 +3682,41 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>D7</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Flag raised while combining the budget years</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>budget_layer_all_years.xlsx / data_quality</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>3929 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G42" s="2" t="n">
         <v>3929</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FY2022 malformed_code_repaired 1: program_code '010000' looked malformed and was normalized to '1.010000' - verify against s
 FY2022 malformed_code_repaired 1: program_code '020000' looked malformed and was normalized to '1.020000' - verify against s
@@ -1623,41 +3729,785 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>110 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 1.5 ieri
+FY2017 20.003 Beim ein ige, She's jeg;
+FY2017 26.009 jeg 932
+FY2018 1.003 Sp 322 9892
+FY2018 19.004 Amd Marmido
+FY2018 22.003 :22 823, VP 29335
+FY2018 22.066 gå sirve HABE ich give
+FY2018 22.073 eisen Pixie</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Fisheries production infrastructure and valu -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Climate adaptation, disaster risk management -&gt; 7 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Fisheries governance, management, monitoring -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Aquaculture and mariculture development -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Climate-smart agriculture, biosecurity, and  -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand
+Tourism employment, skills development, and  -&gt; 5 risks: Democratic Backsliding, Demographic Shifts, Increased Polarisation, Shifts in Gl
+Youth Protection, Inclusion and Housing Supp -&gt; 6 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Integrated waste management and circular eco -&gt; 5 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>157 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Affordable housing provision
+Labour market governance, fair pay, migration management, and worker p
+Education governance, administration and child risk information system
+Family and Community-Based Social Support Programme
+Hajj and Umrah service management and pilgrim support
+Biodiversity conservation, protected areas, and ecosystem restoration
+Climate adaptation, disaster risk management and emergency preparednes
+Innovation, start-up incubation, and digital public information</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>962 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 blank_amount 1: amount is blank/unparseable.
+FY2017 blank_amount 20: amount is blank/unparseable.
+FY2017 blank_amount 26: amount is blank/unparseable.
+FY2017 blank_amount 37: amount is blank/unparseable.
+FY2017 blank_amount 38: amount is blank/unparseable.
+FY2017 blank_amount 39: amount is blank/unparseable.
+FY2018 blank_amount 1: amount is blank/unparseable.
+FY2018 blank_amount 13: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Strategy tagged with five or more risks</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel (related_risks)</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>11 strategy(ies) name five or more of the eleven risks. Tagging on topical adjacency rather than on what the plan says the strategy responds to inflates every risk chart, and it is invisible in any arithmetic check because the tags are self-consistent.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Strategic Program on Supporting Realignment  -&gt; 5 risks: Democratic Backsliding, Growing Populism, Increased Polarisation, Shifts in Glob
+Strategic Program on Good Public Health Prom -&gt; 5 risks: Demographic Shifts, Environmental Degradation and Pollution, Pandemics, Resource
+Strategic Program on Value Creation Agricult -&gt; 6 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Reso
+Strategic Program on Development of Educatio -&gt; 5 risks: Democratic Backsliding, Demographic Shifts, Increased Polarisation, Pandemics, T
+Strategic Program on Supporting Development  -&gt; 6 risks: Climate Change, Environmental Degradation and Pollution, Pandemics, Resource and
+Strategic Program on Developing National Pre -&gt; 6 risks: Climate Change, Demographic Shifts, Environmental Degradation and Pollution, Pan
+Strategic Program on Area Development and Sm -&gt; 8 risks: Biodiversity Loss, Climate Change, Demographic Shifts, Environmental Degradation
+Integrated Program on Creating Income from T -&gt; 7 risks: Biodiversity Loss, Climate Change, Environmental Degradation and Pollution, Pand</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023,2024 program_missing_in_year 4: program '4.12' (Program on Public Sector Personnel) exists in ['2025', '2026'] but is abse
+FY2023,2024,2026 program_missing_in_year 2: program '2.17' (Program on Public Sector Personnel) exists in ['2025'] but is absent in ['
+FY2023,2025 program_missing_in_year 7: program '7.3' (Program on Expenditures for Replenishment of Treasury Account Balance) exis
+FY2024,2025 program_missing_in_year 1: program '1.14' (Program on Public Sector Personnel) exists in ['2023', '2026'] but is abse</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>D6</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>35 distinct programme(s) across 85 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
+FY2024 0905 Special operations: internal debt service (i  668,292.5
+FY2024 0903 OPERACOES ESPECIAIS: TRANSFERENCIAS CONSTITU  557,096.8
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIA  116,778.3
+FY2024 0032 Management and maintenance programme of the   114,021.9
+FY2024 0999 Contingency reserve  89,578.8
+FY2024 0032 Management and maintenance programme of the   77,570.6
+FY2024 0032 Management and maintenance programme of the   67,724.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>39 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 1144 -&gt; 1144 | sustainable agriculture (x2)
+FY2024 1149 -&gt; reconstruction, expansion and deepening  (x2)
+FY2024 1158 -&gt; 1158 | climate emergency response (x3)
+FY2024 1191 -&gt; family farming and agroecology (x3)
+FY2024 1191 -&gt; supply and food sovereignty (x2)
+FY2024 2304 -&gt; science, technology and innovation for s (x2)
+FY2024 2305 -&gt; communications for inclusion and transfo (x2)
+FY2024 2308 -&gt; 2308 | consolidation of the national sci (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 2.2 Construction programme for sewerage and wast  39.0
+FY2025 1.21 Infrastructure and facilities improvement pr  5.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>14 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 1.14 -&gt; green building initiatives under the 12t (x2)
+FY2025 1.17 -&gt; flood prevention projects under the 12th (x2)
+FY2025 1.20 -&gt; capacity enhancement programme for irrig (x2)
+FY2025 1.22 -&gt; paddy buy-back scheme and purchase of hy (x2)
+FY2025 1.3 -&gt; water supply and sewerage system upgradi (x2)
+FY2025 1.7 -&gt; medical and health infrastructure develo (x2)
+FY2025 1.8 -&gt; bru-hims 2.0 system project (x2)
+FY2025 2.1 -&gt; infrastructure provision for enhancement (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>42 distinct programme(s) across 88 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 50.10 Standard Expenditure Group 10  442,060.3
+FY2018 52.2 Programme 2 - Domestic Loans  267,901.9
+FY2017 52.2 Programme 2 - Domestic Loans  243,496.9
+FY2019 52.2 Domestic Loans  233,042.5
+FY2019 22.1 Policy and Administration  123,905.0
+FY2018 52.1 Programme 1 - Overseas Loans  123,372.4
+FY2019 52.1 Overseas Loans  121,320.4
+FY2017 52.1 Programme 1 - Overseas Loans  111,111.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>70 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 14.1 -&gt; 14.1 | disaster management (x2)
+FY2017 14.2 -&gt; 14.2 | meteorological services (x2)
+FY2017 15.1 -&gt; justice (x2)
+FY2017 18.4 -&gt; 18.4 | rehabilitation and rural housing (x2)
+FY2017 21.2 -&gt; 21.2 | primary education (x2)
+FY2017 21.3 -&gt; 21.3 | secondary education (x2)
+FY2017 21.4 -&gt; 21.4 | curriculum development (x2)
+FY2017 21.5 -&gt; 21.5 | tertiary technical education (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>112 distinct programme(s) across 183 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 20000.6.99.137 Management of Public Finances  24,535,325.0
+FY2024 26022.1.01.001 Executive Direction and Administration  20,505,357.0
+FY2024 20019.1.99.136 Pensions and Retirement Benefits  13,856,376.0
+FY2022 42000.1.01.001 Executive Direction and Administration  12,968,255.0
+FY2022 20019.1.99.136 Pensions and Retirement Benefits  12,448,781.0
+FY2024 20012.1.02.146 Customs Management  11,295,545.0
+FY2022 26022.1.01.001 Executive Direction and Administration  11,233,758.0
+FY2024 42000.1.01.001 Executive Direction and Administration  10,473,308.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>50 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 15020.1.99.166 -&gt; civil registration and vital statistics (x2)
+FY2019 19000.6.01.301 -&gt; industrial development and export promot (x2)
+FY2019 19000.6.06.005 -&gt; disaster management (x2)
+FY2019 20056.1.02.149 -&gt; domestic tax administration programme (x2)
+FY2019 26024.1.04.167 -&gt; citizen security and justice capacity st (x2)
+FY2019 28000.1.03.154 -&gt; provision of legal aid services (x2)
+FY2019 28000.6.03.154 -&gt; provision of legal aid services (x2)
+FY2019 41000.1.04.254 -&gt; 12835 | supervision of technical and voc (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>383 distinct programme(s) across 483 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 0509010 Teacher Management- Primary  201,136,266,225.0
+FY2025 0801000 Defence  169,815,800,000.0
+FY2025 0509020 Teacher management - Secondary  142,015,327,079.0
+FY2020 0801010 National Defense  119,808,049,600.0
+FY2025 0717000 General Administration Planning and Support   76,480,295,458.0
+FY2025 0202010 Construction of Roads and Bridges  72,318,898,073.0
+FY2025 0202030 Maintenance of Roads  69,536,000,000.0
+FY2025 0706020 Community Development  63,235,701,088.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>169 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>169</v>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0101010 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0101020 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0101040 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0101050 -&gt; 0101000 | land policy and planning (x2)
+FY2020 0102010 -&gt; housing development and human settlement (x2)
+FY2020 0102030 -&gt; housing development and human settlement (x2)
+FY2020 0108010 -&gt; crop development and management (x2)
+FY2020 0108020 -&gt; crop development and management (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>Budget programme no strategy claims</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / unmapped_programs</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>953 distinct programme(s) across 1894 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G59" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H59" s="2" t="inlineStr">
         <is>
           <t>FY2025 13.010000 FAEDAH, DIVIDEN DAN LAIN-LAIN KENAAN BAYARAN  54,700,000,500.0
 FY2024 13.010000 INTEREST, DIVIDENDS AND OTHER DEBT CHARGES O  49,800,000,000.0
@@ -1670,41 +4520,41 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>D9</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>malaysia</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>One pair matched twice, once per pass</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx / match_review</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>142 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G60" s="2" t="n">
         <v>142</v>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H60" s="2" t="inlineStr">
         <is>
           <t>FY2022 21.040000 -&gt; agriculture sector reinvigoration and fo (x2)
 FY2022 28.020100 -&gt; transport connectivity and logistics mod (x2)
@@ -1714,6 +4564,147 @@
 FY2022 42.030000 -&gt; healthcare service delivery improvement (x2)
 FY2022 42.030000 -&gt; pandemic preparedness, disease control a (x2)
 FY2022 42.060300 -&gt; healthcare research (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>637 distinct programme(s) across 808 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 19.002 et Lille Da Pi, ja gien  6,994,664,737.0
+FY2018 19.001 die Ci 29, 9 28?  1,504,471,755.0
+FY2017 30.001 xixe"jin Ds sind ja sei?  1,490,542,683.0
+FY2017 6.3 And a great قوم  1,473,416,147.0
+FY2017 2.1 ing in  1,455,757,190.0
+FY2017 21.002 وفيد ؤونه قومه مادونه  1,334,531,645.0
+FY2017 19.003 ¿ ¿ iii  1,225,233,300.0
+FY2017 20.002 - pij, ;22 29,99  1,019,664,729.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>46 distinct programme(s) across 147 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 6.6 Fundamental Program on Realignment for Balan  432,256.5
+FY2026 3.8 Program on Public Sector Personnel  429,643.3
+FY2026 7.2 Program on Management of Public Debt  421,864.4
+FY2025 3.8 Program on Public Sector Personnel  416,438.4
+FY2025 7.2 Program on Management of Public Debt  410,253.7
+FY2024 3.8 Program on Public Sector Personnel  403,992.0
+FY2023 3.8 Program on Public Sector Personnel  403,945.1
+FY2026 4.2 Strategic Program on Decentralization to the  377,960.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>27 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 2.13 -&gt; strategic program on supporting developm (x2)
+FY2023 5.7 -&gt; strategic program on supporting creation (x2)
+FY2023 6.2 -&gt; integrated program on digital government (x2)
+FY2024 2.12 -&gt; strategic program on innovation research (x2)
+FY2024 2.14 -&gt; strategic program on supporting developm (x2)
+FY2024 2.2 -&gt; integrated program on development of fut (x2)
+FY2024 2.8 -&gt; strategic program on development of digi (x2)
+FY2024 2.9 -&gt; strategic program on supporting strong a (x2)</t>
         </is>
       </c>
     </row>
@@ -1728,7 +4719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1768,7 +4759,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>malaysia</t>
+          <t>brazil</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -1782,6 +4773,139 @@
       </c>
       <c r="E2" s="2" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1813,7 +4937,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-17 07:48 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-17 15:47 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Register updated: W32-W36 from the panel audit
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2141,6 +2141,266 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>W32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Maldives is unreadable and is published anyway</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>46% of its 852 programme names and 36% of its 101 budget heads are OCR garbage, carrying 31% of its programme money. Heads read 'Hassel', 'Kriegst staj5', 'Da ist Enti', "Has Kin' 13 392-3 3;25". 96% of the country's mapped money sits on exactly two nonsense rows: 'A passing traffic route' under head '2223,9 38, 525 ;' at 431.3m MVR, and an Arabic string under head 'Ej: 39 ; gt ??' at 300.0m. Every other country scores 0% on the same test (Brazil 0 of 182, Malaysia 0 of 2,815, Kenya 0 of 985). This is W12 reaching the public page: the country is live on the dashboard now, showing 261 strategies and 1.7% mapped over data that means nothing.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Pull Maldives from the published set until its budgets are re-parsed. Document Intelligence renders Thaana as Arabic and then as European nonsense, so the fix is upstream of every prompt. A readability gate belongs in the pipeline: a country whose programme names fail a letters-per-name test should not reach publish_run.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>budget_all_years, Maldives; 395 of 852 programme names fail the readability test</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>W33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, jamaica</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>The national denominator is not the national budget, so the headline share is wrong</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>share_mapped divides mapped money by the sum of the budget heads' own stated totals. In Malaysia the programmes beneath those heads sum to 1.91x the heads: 966.4bn against 1,847.9bn over five years. Malaysia's real federal budget is roughly 390-420bn a year; the programme sums (352-433bn) are about right and the head totals (163-241bn) are roughly half. So the published 87.3% is inflated by close to 2x and the honest figure against programme money is 45.6%. Jamaica is 1.24x and reads 86.8% against a programme-based 70.3%. The ratio also swings by year in Malaysia, 1.47x to 2.33x, so its year-on-year series is not comparable with itself. Brazil, Kenya and Thailand reconcile at 1.00x and are unaffected.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Take the national total from the PROGRAMME rows where they and the head totals disagree beyond a tolerance, and say on the page which basis was used. The head totals are what the document prints, but in Malaysia they are demonstrably incomplete, and a denominator that is half the budget doubles every share computed from it. Related to W10 and W13.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>sum(strategy_total) vs sum(program) per country, all 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>W34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, jamaica, fiji, maldives</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>The ceiling test fails on broken head totals rather than on over-attribution</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>A4 asserts matched money never exceeds the budget head's own total. It now fails 38 times in Malaysia, 17 in Jamaica, 3 in Fiji and once in Maldives, and the cause in every case examined is the head total, not the mapping: Malaysia FY2022 head 63 shows matched 40,495,896,900 against a stated total of 4,013,756,600, and head 6 shows 1,098,130,400 against 504,000. The programmes summed under those heads are far larger than the heads claim. Read as a mapping fault it points at the wrong thing entirely.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Where a head's programmes do not reconcile with its stated total, the ceiling test should compare against the programme sum and say it did so, rather than failing against a figure already known to be wrong. The reconciliation flag exists; A4 should consult it.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>audit_checks A4, all countries</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>W35</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>publishing</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>brazil, kenya</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>funding_by_program breaks the contract its own documentation states</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>The sheet is documented as each (programme, year) counted once and safe to sum. Brazil holds 8 (year, code) pairs on more than one row and Kenya 2. The rows are correct: Brazil's PPA repeats one programme code under several budget functions, so FY2024 code 2317 legitimately appears under Urbanismo, Administration, Science and technology, Agricultura and Encargos especiais with five different amounts. Summing them is right. It is the stated contract that is wrong, and anyone deduplicating on (year, code) in good faith would silently drop 0.33% of Brazil's mapped money.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Restate the guarantee as one row per (year, head, programme) and say so in REQUIREMENTS.md, or add the head to the sheet's key. This is W1 seen from the consumer's side.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>8 duplicated keys in Brazil funding_by_program, 5,511.0 BRL million</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>W36</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, kenya, fiji</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Programmes carrying no money are matched to strategies</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Malaysia has 6 matched programmes with an amount of zero, Kenya 2, Fiji 1. They add edges and strategy attributions while contributing nothing, so a strategy can read as funded on the strength of a line worth nothing.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Either drop zero-amount programmes before stage 6 sees them, or flag the edge so a strategy funded only by zero-amount lines still reports as unfunded.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>funding_by_program amount == 0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2152,7 +2412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2467,2437 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>28 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 programme 0032: 1.4 and 77.9 and 331.9 and 469.5 and 633.9 and 756.5 and 850.8 and 904.4 and 1,021.0 and 1,192.6 and 1,532.3 and 1,607.8 and 1,809.5 and 1,853.5 and 2,003.2 and 3,005.3 and 3,497.2 and 5,553.3 and 10,446.6 and 10,768.5 and 30,770.3 and 67,724.5 and 77,570.6 and 114,021.9  (under budget strategies 03, 04, 05, 06, 07, 08, 09, 10, 11, 12, 13, 14, 15, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28)
+FY2024 programme 0901: 1,984.7 and 64,985.7  (under budget strategies 28, 99)
+FY2024 programme 0902: 216.8 and 500.0 and 2,000.0 and 6,362.3 and 6,415.9 and 26,568.8 and 27,153.3  (under budget strategies 05, 11, 12, 19, 20, 23, 28)
+FY2024 programme 0903: 2,007.3 and 557,096.8  (under budget strategies 09, 28)
+FY2024 programme 0909: 0.0 and 0.3 and 0.8 and 5.3 and 149.6 and 246.0 and 1,502.0 and 116,778.3  (under budget strategies 04, 07, 12, 19, 23, 25, 26, 28)
+FY2024 programme 0910: 0.1 and 0.7 and 4.4 and 1,525.5  (under budget strategies 10, 14, 26, 28)
+FY2024 programme 1144: 0.0 and 14,910.1  (under budget strategies 20, 28)
+FY2024 programme 1149: 20.2 and 54.2  (under budget strategies 04, 14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brazil/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>3 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>brazil_strategy_rows.xlsx was written 2026-08-10; 3_strategy_extraction.txt was edited 2026-08-19
+brazil_budget_2021.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12
+brazil_budget_2024.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>13 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Electricity generation, transmission and dis &lt;- named after budget line Electricity supply projects under the 12th N
+Agricultural development area infrastructure &lt;- named after budget line Infrastructure provision for enhancement of 
+Airport infrastructure modernisation and avi &lt;- named after budget line Airport infrastructure modernisation project
+Climate policy, emissions reduction and gree &lt;- named after budget line Green Building initiatives under the 12th Na
+Research, innovation and commercialisation s &lt;- named after budget line Research and innovation allocations under th
+Sewerage system upgrading and sanitation inf &lt;- named after budget line Construction programme for sewerage and wast
+Scholarships and human resource funding for  &lt;- named after budget line Scholarships through the Ministry of Educati
+Tourism product and cultural asset upgrading &lt;- named after budget line Tourism product improvement projects under t</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brunei/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>5 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>brunei_strategy_rows.xlsx was written 2026-08-10; 3_strategy_extraction.txt was edited 2026-08-19
+brunei_budget_2021.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2022.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2025.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2026.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 reconciliation_mismatch 1: programs sum to 1,912.5 but strategy_total is 1,949.8 (gap 37.3) - a program line is likel
+FY2025 reconciliation_mismatch 3: programs sum to 626.7 but strategy_total is 624.9 (gap -1.8) - a program line is likely mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 strategy 1: printed 1,949.8, programmes sum to 1,912.5, apart by 37.3
+FY2025 strategy 3: printed 624.9, programmes sum to 626.7, apart by -1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/fiji/</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>fiji_strategy_rows.xlsx was written 2026-08-15; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>28 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 22: programs sum to 321,245.4 but strategy_total is 321,245.6 (gap 0.2) - a program line is li
+FY2017 reconciliation_mismatch 24: programs sum to 113,354.0 but strategy_total is 113,354.1 (gap 0.1) - a program line is li
+FY2017 reconciliation_mismatch 25: programs sum to 23,096.7 but strategy_total is 23,096.6 (gap -0.1) - a program line is lik
+FY2017 reconciliation_mismatch 33: programs sum to 28,538.8 but strategy_total is 42,329.9 (gap 13,791.1) - a program line is
+FY2017 reconciliation_mismatch 40: programs sum to 133,737.9 but strategy_total is 134,178.0 (gap 440.1) - a program line is 
+FY2017 reconciliation_mismatch 50: programs sum to 615,572.2 but strategy_total is 628,116.8 (gap 12,544.6) - a program line 
+FY2017 reconciliation_mismatch 52: programs sum to 364,701.0 but strategy_total is 354,607.9 (gap -10,093.1) - a program line
+FY2018 reconciliation_mismatch 2: programs sum to 23,891.3 but strategy_total is 14,262.3 (gap -9,629.0) - a program line is</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>28 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 22: printed 321,245.6, programmes sum to 321,245.4, apart by 0.2
+FY2017 strategy 24: printed 113,354.1, programmes sum to 113,354.0, apart by 0.1
+FY2017 strategy 25: printed 23,096.6, programmes sum to 23,096.7, apart by -0.1
+FY2017 strategy 33: printed 42,329.9, programmes sum to 28,538.8, apart by 13,791.1
+FY2017 strategy 40: printed 134,178.0, programmes sum to 133,737.9, apart by 440.1
+FY2017 strategy 50: printed 628,116.8, programmes sum to 615,572.2, apart by 12,544.6
+FY2017 strategy 52: printed 354,607.9, programmes sum to 364,701.0, apart by -10,093.1
+FY2018 strategy 2: printed 14,262.3, programmes sum to 23,891.3, apart by -9,629.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/jamaica/</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>jamaica_strategy_rows.xlsx was written 2026-08-14; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>74 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 reconciliation_mismatch 01000: programs sum to 83,000.0 but strategy_total is 290,111.0 (gap 207,111.0) - a program line 
+FY2019 reconciliation_mismatch 08000: programs sum to 642,858.0 but strategy_total is 469,975.0 (gap -172,883.0) - a program lin
+FY2019 reconciliation_mismatch 09000: programs sum to 712,147.0 but strategy_total is 833,920.0 (gap 121,773.0) - a program line
+FY2019 reconciliation_mismatch 15010: programs sum to 0.0 but strategy_total is 697,424.0 (gap 697,424.0) - a program line is li
+FY2019 reconciliation_mismatch 15020: programs sum to 900,480.0 but strategy_total is 10,480.0 (gap -890,000.0) - a program line
+FY2019 reconciliation_mismatch 16049: programs sum to 489,234.0 but strategy_total is 225,234.0 (gap -264,000.0) - a program lin
+FY2019 reconciliation_mismatch 17000: programs sum to 6,345,325.0 but strategy_total is 11,525,361.0 (gap 5,180,036.0) - a progr
+FY2019 reconciliation_mismatch 19046: programs sum to 1,085,718.0 but strategy_total is 1,078,318.0 (gap -7,400.0) - a program l</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>74 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 strategy 01000: printed 290,111.0, programmes sum to 83,000.0, apart by 207,111.0
+FY2019 strategy 08000: printed 469,975.0, programmes sum to 642,858.0, apart by -172,883.0
+FY2019 strategy 09000: printed 833,920.0, programmes sum to 712,147.0, apart by 121,773.0
+FY2019 strategy 15010: printed 697,424.0, programmes sum to 0.0, apart by 697,424.0
+FY2019 strategy 15020: printed 10,480.0, programmes sum to 900,480.0, apart by -890,000.0
+FY2019 strategy 16049: printed 225,234.0, programmes sum to 489,234.0, apart by -264,000.0
+FY2019 strategy 17000: printed 11,525,361.0, programmes sum to 6,345,325.0, apart by 5,180,036.0
+FY2019 strategy 19046: printed 1,078,318.0, programmes sum to 1,085,718.0, apart by -7,400.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>7 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 programme 0106000: 346,691,310.0 and 364,590,743.0  (under budget strategies 1094, 1095)
+FY2025 programme 0207000: 231,885,786.0 and 278,922,194.0  (under budget strategies 1122, 1123)
+FY2025 programme 0412000: 651,366,934.0 and 16,529,119,104.0  (under budget strategies 1082, 1083)
+FY2025 programme 0508000: 297,799,258.0 and 435,378,299.0 and 4,677,027,195.0  (under budget strategies 1064, 1065, 1066)
+FY2025 programme 0709000: 233,471,082.0 and 444,125,877.0  (under budget strategies 1072, 1213)
+FY2025 programme 0710000: 2,000,000.0 and 8,769,275,002.0  (under budget strategies 1072, 1213)
+FY2025 programme 1018000: 30,500,000.0 and 12,916,448,407.0  (under budget strategies 1331, 1332)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/kenya/</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>kenya_strategy_rows.xlsx was written 2026-08-14; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>8 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 reconciliation_mismatch 0106000: programs sum to 349,247,063.0 but strategy_total is 276,081,719.0 (gap -73,165,344.0) - a 
+FY2020 reconciliation_mismatch 0508000: programs sum to 2,991,357,360.0 but strategy_total is 164,025,309.0 (gap -2,827,332,051.0)
+FY2020 reconciliation_mismatch 1014000: programs sum to 7,655,824,962.0 but strategy_total is 0.0 (gap -7,655,824,962.0) - a progr
+FY2020 reconciliation_mismatch 1018000: programs sum to 10,066,601,747.0 but strategy_total is 10,873,301,747.0 (gap 806,700,000.0
+FY2025 reconciliation_mismatch 0106000: programs sum to 418,347,116.0 but strategy_total is 346,691,310.0 (gap -71,655,806.0) - a 
+FY2025 reconciliation_mismatch 0508000: programs sum to 3,536,217,818.0 but strategy_total is 435,378,299.0 (gap -3,100,839,519.0)
+FY2025 reconciliation_mismatch 0709000: programs sum to 234,021,081.0 but strategy_total is 233,471,082.0 (gap -549,999.0) - a pro
+FY2025 reconciliation_mismatch 0710000: programs sum to 4,177,242,813.0 but strategy_total is 2,000,000.0 (gap -4,175,242,813.0) -</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 strategy 0106000: printed 276,081,719.0, programmes sum to 349,247,063.0, apart by -73,165,344.0
+FY2020 strategy 0508000: printed 164,025,309.0, programmes sum to 2,991,357,360.0, apart by -2,827,332,051.0
+FY2020 strategy 1014000: printed 0.0, programmes sum to 7,655,824,962.0, apart by -7,655,824,962.0
+FY2020 strategy 1018000: printed 10,873,301,747.0, programmes sum to 10,066,601,747.0, apart by 806,700,000.0
+FY2025 strategy 0106000: printed 346,691,310.0, programmes sum to 418,347,116.0, apart by -71,655,806.0
+FY2025 strategy 0508000: printed 435,378,299.0, programmes sum to 3,536,217,818.0, apart by -3,100,839,519.0
+FY2025 strategy 0709000: printed 233,471,082.0, programmes sum to 234,021,081.0, apart by -549,999.0
+FY2025 strategy 0710000: printed 2,000,000.0, programmes sum to 4,177,242,813.0, apart by -4,175,242,813.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/malaysia/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>malaysia_strategy_rows.xlsx was written 2026-08-15; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>138 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FY2022 reconciliation_mismatch 1: programs sum to 19,215,800.0 but strategy_total is 13,533,000.0 (gap -5,682,800.0) - a pro
+FY2022 reconciliation_mismatch 10: programs sum to 3,621,353,400.0 but strategy_total is 5,254,500.0 (gap -3,616,098,900.0) -
+FY2022 reconciliation_mismatch 11: programs sum to 10,635,228,700.0 but strategy_total is 1,969,500.0 (gap -10,633,259,200.0)
+FY2022 reconciliation_mismatch 12: programs sum to 6,726,656,600.0 but strategy_total is 6,343,326,200.0 (gap -383,330,400.0)
+FY2022 reconciliation_mismatch 13: programs sum to 43,783,892,500.0 but strategy_total is 43,100,000,000.0 (gap -683,892,500.
+FY2022 reconciliation_mismatch 14: programs sum to 342,528,400.0 but strategy_total is 27,500,000,000.0 (gap 27,157,471,600.0
+FY2022 reconciliation_mismatch 2: programs sum to 2,500,000.0 but strategy_total is 1,337,000.0 (gap -1,163,000.0) - a progr
+FY2022 reconciliation_mismatch 28: programs sum to 1,527,593,800.0 but strategy_total is 4,053,603,700.0 (gap 2,526,009,900.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>138 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>FY2022 strategy 1: printed 13,533,000.0, programmes sum to 19,215,800.0, apart by -5,682,800.0
+FY2022 strategy 2: printed 1,337,000.0, programmes sum to 2,500,000.0, apart by -1,163,000.0
+FY2022 strategy 3: printed 110,000,000.0, programmes sum to 111,286,000.0, apart by -1,286,000.0
+FY2022 strategy 4: printed 836,700.0, programmes sum to 128,970,400.0, apart by -128,133,700.0
+FY2022 strategy 5: printed 564,000.0, programmes sum to 20,919,000.0, apart by -20,355,000.0
+FY2022 strategy 6: printed 504,000.0, programmes sum to 5,704,861,700.0, apart by -5,704,357,700.0
+FY2022 strategy 7: printed 2,465,300.0, programmes sum to 256,675,300.0, apart by -254,210,000.0
+FY2022 strategy 8: printed 11,000.0, programmes sum to 75,123,900.0, apart by -75,112,900.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/maldives/</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>maldives_strategy_rows.xlsx was written 2026-08-15; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>52 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 reconciliation_mismatch 1: programs sum to 371,971,798.0 but strategy_total is 101,334,724.0 (gap -270,637,074.0) - a
+FY2017 reconciliation_mismatch 10: programs sum to 603,169,808.0 but strategy_total is 35,391,792.0 (gap -567,778,016.0) - a 
+FY2017 reconciliation_mismatch 11: programs sum to 84,903,354.0 but strategy_total is 59,843,651.0 (gap -25,059,703.0) - a pr
+FY2017 reconciliation_mismatch 12: programs sum to 0.0 but strategy_total is 6,993,896.0 (gap 6,993,896.0) - a program line i
+FY2017 reconciliation_mismatch 13: programs sum to 0.0 but strategy_total is 3,626,872.0 (gap 3,626,872.0) - a program line i
+FY2017 reconciliation_mismatch 14: programs sum to 0.0 but strategy_total is 9,198,520.0 (gap 9,198,520.0) - a program line i
+FY2017 reconciliation_mismatch 15: programs sum to 0.0 but strategy_total is 4,223,952.0 (gap 4,223,952.0) - a program line i
+FY2017 reconciliation_mismatch 16: programs sum to 0.0 but strategy_total is 44,828,700.0 (gap 44,828,700.0) - a program line</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>52 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 1: printed 101,334,724.0, programmes sum to 371,971,798.0, apart by -270,637,074.0
+FY2017 strategy 2: printed 208,402,975.0, programmes sum to 1,780,849,664.0, apart by -1,572,446,689.0
+FY2017 strategy 3: printed 10,854,474.0, programmes sum to 291,704,544.0, apart by -280,850,070.0
+FY2017 strategy 4: printed 367,654,006.0, programmes sum to 952,692,855.0, apart by -585,038,849.0
+FY2017 strategy 5: printed 35,615,361.0, programmes sum to 796,853,288.0, apart by -761,237,927.0
+FY2017 strategy 6: printed 19,009,362.0, programmes sum to 2,294,511,756.0, apart by -2,275,502,394.0
+FY2017 strategy 7: printed 22,661,255.0, programmes sum to 266,705,093.0, apart by -244,043,838.0
+FY2017 strategy 8: printed 27,923,748.0, programmes sum to 494,853,833.0, apart by -466,930,085.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/thailand/</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>thailand_strategy_rows.xlsx was written 2026-08-10; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
+FY2024 0151 Protection of indigenous lands, territorial management and e
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIAIS
+FY2024 1144 AGROPECUARIA SUSTENTAVEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>37 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Multimodal logistics and transport efficiency
+Sports and physical activity promotion
+Climate adaptation, mitigation and disaster risk management
+Productive inclusion and income generation for poor households
+Advance racial equality, anti-racism and affirmative action
+International cooperation and consular action for sustainable developm
+Export diversification and trade integration
+Fiscal reform, tax compliance and revenue integrity</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>37 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>National development planning, project appraisal and implementation co
+Government offices, border posts and overseas representation facilitie
+Environmental impact assessment and pollution control enforcement
+Road, bridge and transport infrastructure improvement
+National security, defence modernisation and policing facilities
+Sports and community recreation facilities upgrading
+MSME development and business environment improvement
+Whole-of-nation implementation and institutional capacity support</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>1 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 30.5 Land Drainage and Flood Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>23 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Promote digital services exports and the outsourcing industry
+Promote civic values, ethics and social cohesion
+Modernise construction standards, skills and climate-resilient buildin
+Strengthen defence, regional security alliances and emergency assistan
+Audio-visual industry regulation, incentives and ecosystem development
+Inclusive insurance and microinsurance expansion
+Virtual assets, anti-fraud and financial integrity regulation
+Construction regulation, licensing and building code enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>20 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 program_missing_in_year 23: program '23.2' (Housing) exists in ['2018', '2019'] but is absent in ['2017'] - check whet
+FY2017 program_missing_in_year 26: program '26.1' (Higher Education Institutions) exists in ['2018', '2019'] but is absent in
+FY2017,2018 program_missing_in_year 13: program '13.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '2
+FY2017,2018 program_missing_in_year 34: program '34.6' (Micro, Small and Medium Enterprises Central Coordinating Agency) exists in
+FY2017,2018 program_missing_in_year 4: program '4.3' (Public Enterprises) exists in ['2019'] but is absent in ['2017', '2018'] - 
+FY2017,2018 program_missing_in_year 9: program '9.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '20
+FY2018,2019 program_missing_in_year 18: program '18.4' (Rehabilitation and Rural Housing) exists in ['2017'] but is absent in ['20
+FY2018,2019 program_missing_in_year 30: program '30.5' (Land Drainage and Flood Protection) exists in ['2017'] but is absent in ['</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>4 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Modernize consular and overseas travel services
+Strengthen monetary policy governance and macroeconomic forecasting
+Provide social protection and insurance for athletes
+Strengthen water and sanitation cooperation and community management</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>200 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2019 program_missing_in_year 03000: program '03000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.157' (Government Audit Services) exists in ['2022', '2024'] but is abs
+FY2019 program_missing_in_year 06000: program '06000.1.03.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 06000: program '06000.1.03.158' (Public Service Personnel Management) exists in ['2022', '2024'] 
+FY2019 program_missing_in_year 07000: program '07000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 07000: program '07000.1.99.139' (Protection of Children's Rights) exists in ['2022', '2024'] but 
+FY2019 program_missing_in_year 07000: program '07000.1.99.159' (Combatting Human Trafficking) exists in ['2022', '2024'] but is </t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0105060 NAMATA
+FY2020 0120040 Fisheries Research &amp; Development
+FY2020 0620020 Police Vetting
+FY2020 0703050 Coordination of Vision 2030
+FY2020 0712050 Finance Management Services
+FY2020 0715060 International Relations and Cooperation
+FY2020 0733040 Peace and Conflict Management
+FY2020 0740010 Government Clearing Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>42 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Security force recruitment, welfare and infrastructure modernization
+National values, ethics and civic participation
+Government services, records and data infrastructure digitization
+Diaspora engagement, information systems and skills transfer
+Diaspora welfare, emergency response and reintegration services
+Forensic capacity and conflict resolution strengthening
+Intergovernmental coordination and whole-of-government delivery
+Public-private partnership and development partner coordination</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>470 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
+FY2020 blank_amount 0120000: amount is blank/unparseable.
+FY2020 blank_amount 0620000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0712000: amount is blank/unparseable.
+FY2020 blank_amount 0715000: amount is blank/unparseable.
+FY2020 blank_amount 0733000: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>36 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>FY2022 28.030600 Maintenance, Repair and Overhaul (KTMB)
+FY2022 28.031000 Maintenance of the AwAS System
+FY2022 28.031200 Interim Stage Bus Support Fund Program (ISBSF)
+FY2022 28.031300 Stage Bus Service Transformation Program (SBST)
+FY2022 43.030500 Perbadanan PRIMA Malaysia (PRIMA)
+FY2022 43.040700 Fasiliti Pengurusan Sisa Pepejal (SWCorp)
+FY2022 43.990100 PPP - Perkhidmatan Pengurusan Sisa Pepejal dan Pembersihan A
+FY2022 43.990200 PPP - Tapak Pelupusan Sanitari Sisa Pepejal Ladang Tanah Mer</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>44 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Productivity nexus expansion and programme rationalisation
+Expand green city planning and urban sustainability action
+Water governance, legislation and institutional reform
+Adaptive Plan Implementation, Review and Monitoring Reform
+Whole-of-Nation SDG Localisation and Public Engagement
+Green and Circular Construction Materials and Building Practices
+Industrial Estates, Food Production Areas and Domestic Investment Supp
+Financial Intermediation and Innovation Financing Ecosystem</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>3929 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>3929</v>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2022 malformed_code_repaired 1: program_code '010000' looked malformed and was normalized to '1.010000' - verify against s
+FY2022 malformed_code_repaired 1: program_code '020000' looked malformed and was normalized to '1.020000' - verify against s
+FY2022 malformed_code_repaired 1: program_code '030000' looked malformed and was normalized to '1.030000' - verify against s
+FY2022 malformed_code_repaired 10: program_code '010000' looked malformed and was normalized to '10.010000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '020000' looked malformed and was normalized to '10.020000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '030000' looked malformed and was normalized to '10.030000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '040000' looked malformed and was normalized to '10.040000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '050000' looked malformed and was normalized to '10.050000' - verify against </t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>110 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 1.5 ieri
+FY2017 20.003 Beim ein ige, She's jeg;
+FY2017 26.009 jeg 932
+FY2018 1.003 Sp 322 9892
+FY2018 19.004 Amd Marmido
+FY2018 22.003 :22 823, VP 29335
+FY2018 22.066 gå sirve HABE ich give
+FY2018 22.073 eisen Pixie</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>251 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>251</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Affordable and social housing delivery
+Coral reef rehabilitation and marine biodiversity restoration
+Climate-smart and environmentally sustainable agriculture
+Governance quality improvement
+Teacher development, school leadership and education governance
+Equitable school access and inclusive learning support
+Unemployment protection and income support for vulnerable groups
+Substance use prevention, treatment and rehabilitation services</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>962 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 blank_amount 1: amount is blank/unparseable.
+FY2017 blank_amount 20: amount is blank/unparseable.
+FY2017 blank_amount 26: amount is blank/unparseable.
+FY2017 blank_amount 37: amount is blank/unparseable.
+FY2017 blank_amount 38: amount is blank/unparseable.
+FY2017 blank_amount 39: amount is blank/unparseable.
+FY2018 blank_amount 1: amount is blank/unparseable.
+FY2018 blank_amount 13: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Support and protection for firms and workers affected by EV transition
+High-skill talent attraction, mobility, and retention
+National monitoring, evaluation, and adaptive management system</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023,2024 program_missing_in_year 4: program '4.12' (Program on Public Sector Personnel) exists in ['2025', '2026'] but is abse
+FY2023,2024,2026 program_missing_in_year 2: program '2.17' (Program on Public Sector Personnel) exists in ['2025'] but is absent in ['
+FY2023,2025 program_missing_in_year 7: program '7.3' (Program on Expenditures for Replenishment of Treasury Account Balance) exis
+FY2024,2025 program_missing_in_year 1: program '1.14' (Program on Public Sector Personnel) exists in ['2023', '2026'] but is abse</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>42 distinct programme(s) across 90 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
+FY2024 0905 Special operations: internal debt service (i  668,292.5
+FY2024 0903 OPERACOES ESPECIAIS: TRANSFERENCIAS CONSTITU  557,096.8
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIA  116,778.3
+FY2024 0032 Management and maintenance programme of the   114,021.9
+FY2024 0999 Contingency reserve  89,578.8
+FY2024 0032 Management and maintenance programme of the   77,570.6
+FY2024 0032 Management and maintenance programme of the   67,724.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>9 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 1149 -&gt; participatory budgeting, transparency an (x2)
+FY2024 2317 -&gt; regional development, territorial planni (x5)
+FY2024 2320 -&gt; implement intersectoral support and hous (x2)
+FY2024 2321 -&gt; water security and integrated water reso (x3)
+FY2024 2322 -&gt; basic sanitation and urban environmental (x2)
+FY2024 5115 -&gt; access to justice and justice system imp (x3)
+FY2024 5115 -&gt; defend democracy and strengthen institut (x2)
+FY2024 5115 -&gt; improve access to justice and legal righ (x3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>7 distinct programme(s) across 7 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 1.12 Payment for medical treatment services at Gl  150.0
+FY2025 2.10 IT Central Procurement projects and software  144.7
+FY2025 1.11 Purchase of medicines, medical consumables a  89.0
+FY2025 3.7 Focus projects to support the budget focus a  27.5
+FY2025 1.18 Natural disaster management  25.0
+FY2025 1.6 Education information and data management sy  21.2
+FY2025 3.6 Research costs for public higher education i  2.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>43 distinct programme(s) across 91 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 50.10 Standard Expenditure Group 10  442,060.3
+FY2019 22.1 Policy and Administration  123,905.0
+FY2018 26.1 Higher Education Institutions  123,789.1
+FY2019 26.1 Higher Education Institutions  115,587.2
+FY2018 19.1 Republic of Fiji Military Forces  103,252.1
+FY2017 19.1 Republic of Fiji Military Forces  96,688.5
+FY2018 22.1 Policy and Administration  85,470.5
+FY2019 9.1 Policy and Administration  84,724.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>102 distinct programme(s) across 164 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 26000.1.01.437 Territorial and Sovereign Protection  41,716,884.0
+FY2022 26000.1.01.437 Territorial and Sovereign Protection  28,230,476.0
+FY2024 20000.6.99.137 Management of Public Finances  24,535,325.0
+FY2019 26000.1.01.400 Defense Forces Services  22,376,754.0
+FY2024 26022.1.01.001 Executive Direction and Administration  20,505,357.0
+FY2022 42000.1.01.001 Executive Direction and Administration  12,968,255.0
+FY2019 26000.6.01.400 Defense Forces Services  12,569,794.0
+FY2022 26022.1.01.001 Executive Direction and Administration  11,233,758.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>505 distinct programme(s) across 641 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 0509000 Teacher Resource Management  347,685,463,808.0
+FY2025 0509010 Teacher Management- Primary  201,136,266,225.0
+FY2025 0801010 National Defense  169,815,800,000.0
+FY2025 0509020 Teacher management - Secondary  142,015,327,079.0
+FY2025 0502020 Free Day Secondary Education  102,527,921,685.0
+FY2025 0717000 General Administration Planning and Support   76,480,295,458.0
+FY2020 0502020 Free Day Secondary Education  67,274,154,762.0
+FY2025 0504010 University Education  67,180,896,533.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 1018000 -&gt; forest protection and environmental comp (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>957 distinct programme(s) across 1943 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 13.010000 FAEDAH, DIVIDEN DAN LAIN-LAIN KENAAN BAYARAN  54,700,000,500.0
+FY2024 13.010000 INTEREST, DIVIDENDS AND OTHER DEBT CHARGES O  49,800,000,000.0
+FY2023 11.020000 TRANSFER PAYMENTS AND GRANTS  49,502,871,200.0
+FY2023 13.010000 INTEREST, DIVIDENDS AND OTHER DEBT SERVICE C  46,100,000,000.0
+FY2024 11.020000 TRANSFER PAYMENTS AND GRANTS  45,724,636,400.0
+FY2022 13.010000 INTEREST, DIVIDENDS AND OTHER CHARGES ON NAT  43,100,000,000.0
+FY2026 11.020000 TRANSFER PAYMENTS AND GRANTS  37,620,151,300.0
+FY2024 42.000000 Mengurus  35,150,181,800.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>666 distinct programme(s) across 836 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 19.002 et Lille Da Pi, ja gien  6,994,664,737.0
+FY2018 19.001 die Ci 29, 9 28?  1,504,471,755.0
+FY2017 30.001 xixe"jin Ds sind ja sei?  1,490,542,683.0
+FY2017 6.3 And a great قوم  1,473,416,147.0
+FY2017 2.1 ing in  1,455,757,190.0
+FY2017 21.002 وفيد ؤونه قومه مادونه  1,334,531,645.0
+FY2017 19.003 ¿ ¿ iii  1,225,233,300.0
+FY2017 20.002 - pij, ;22 29,99  1,019,664,729.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>38 distinct programme(s) across 120 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 3.8 Program on Public Sector Personnel  429,643.3
+FY2026 7.2 Program on Management of Public Debt  421,864.4
+FY2025 3.8 Program on Public Sector Personnel  416,438.4
+FY2025 7.2 Program on Management of Public Debt  410,253.7
+FY2024 3.8 Program on Public Sector Personnel  403,992.0
+FY2023 3.8 Program on Public Sector Personnel  403,945.1
+FY2026 4.2 Strategic Program on Decentralization to the  377,960.2
+FY2024 7.2 Program on Management of Public Debt  346,380.1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2218,7 +4909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2253,6 +4944,158 @@
         <is>
           <t>TOTAL</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2284,7 +5127,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-20 14:10 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-20 14:41 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Money ladder live: programme class per country, nested levels counted once, ladder sourced from edges
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -2174,7 +2174,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Pull Maldives from the published set until its budgets are re-parsed. Document Intelligence renders Thaana as Arabic and then as European nonsense, so the fix is upstream of every prompt. A readability gate belongs in the pipeline: a country whose programme names fail a letters-per-name test should not reach publish_run.</t>
+          <t>Pull Maldives from the published set until its budgets are re-parsed. Document Intelligence renders Thaana as Arabic and then as European nonsense, so the fix is upstream of every prompt. A readability gate belongs in the pipeline: a country whose programme names fail a letters-per-name test should not reach publish_run.  PARTIAL 2026-08-20: new audit check A20 fails any country where more than 20% of programme names are unreadable, and combine_budget_years raises a HIGH data_quality flag for the same. Maldives fails it at 46%; every other country passes at 0%. The country is still published; pulling it is a decision, not a bug fix.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2226,12 +2226,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Take the national total from the PROGRAMME rows where they and the head totals disagree beyond a tolerance, and say on the page which basis was used. The head totals are what the document prints, but in Malaysia they are demonstrably incomplete, and a denominator that is half the budget doubles every share computed from it. Related to W10 and W13.</t>
+          <t>FIXED 2026-08-20. The real cause was a LEVEL COLLAPSE, not a missing operating/development split. Stage 5 flattened a three-level budget into one 'program' line_type, so Malaysia's head 63 carries four programmes summing to 43,291,751,100 AND the nineteen activities beneath them summing to the same 43,291,751,100, while the stored head total of 4,013,756,600 is merely the first programme. Neither published basis was the budget: the heads understate by 10x on that head and summing every programme row doubles it. combine_budget_years now detects nesting PER HEAD-YEAR, accepting it only where the two levels arithmetically coincide (15 nested head-years in Malaysia, 175 flat), counts the top level once, and writes the chosen basis into a national_total sheet that every consumer reads instead of re-deriving. Malaysia 87.28% -&gt; 49.85%, Jamaica 86.80% -&gt; 70.27%, Fiji 76.58% -&gt; 80.52%, Maldives 1.70% -&gt; 2.37%. Brazil, Kenya and Thailand reconcile and did not move.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2278,12 +2278,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Where a head's programmes do not reconcile with its stated total, the ceiling test should compare against the programme sum and say it did so, rather than failing against a figure already known to be wrong. The reconciliation flag exists; A4 should consult it.</t>
+          <t>FIXED. A4 now caps each head at its printed total or, where that under-reports its own programmes by more than 5%, at the programme sum, and says how many heads were capped. Malaysia 38 failures -&gt; 0, Jamaica 17 -&gt; 0, Maldives 1 -&gt; 0. Fiji's 3 survive and are genuine over-attribution.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2544,7 +2544,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21 08:58 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-21 09:28 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
0007 applied: countable in the database, view rebuilt
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>v_funding_by_program joins budget_lines to matches on (run_id, fiscal_year, program_code). Where a code repeats under several heads the join crosses them, so the view disagrees with the panel for the two countries where that happens. The dashboard works around it by reading the edges instead, which is why the page and the panel now agree, but the view is still wrong for anyone querying it directly.</t>
+          <t>v_funding_by_program joins budget_lines to matches on (run_id, fiscal_year, program_code). Where a code repeats under several heads the join crosses them, so the view disagrees with the panel for the two countries where that happens. The dashboard works around it by reading the edges instead, which is why the page and the panel now agree, but the view is still wrong for anyone querying it directly.  Measured 2026-08-20: for Brazil the view returns 141 rows summing 2,005,259 where the panel holds 92 rows summing 1,681,045, a 19% overstatement. The union dashboard's money ladder was briefly built on it and disagreed with the headline directly above it; it now takes mapped money from the edges keyed on (year, code, budget head), which is what the headline already did. The VIEW is still wrong for anyone querying it.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2398,6 +2398,58 @@
       <c r="J37" s="2" t="inlineStr">
         <is>
           <t>funding_by_program amount == 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>W37</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Nested budget levels are counted once, and the decision is a column rather than a rule each reader re-applies</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Stage 5 flattens a multi-level budget into one 'program' line_type. Where a head carries both its programmes and the activities beneath them, summing every row doubles that head. Malaysia has 397 such rows across 15 head-years, worth 155.9bn, and two separate readers (the v_development_coverage view and the dashboard's ladder) each re-derived the rule and each inherited the double count.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>combine_budget_years decides per head-year, accepting a hierarchy only where the two levels arithmetically coincide, and stamps 'countable' Y/N on every programme row. Migration 0007 adds the column and rebuilds the view to respect it; NULL is treated as countable so older runs read exactly as before.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Malaysia 1,847.9bn all rows vs 1,692.0bn countable</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2467,6 +2519,2480 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>28 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 programme 0032: 1.4 and 77.9 and 331.9 and 469.5 and 633.9 and 756.5 and 850.8 and 904.4 and 1,021.0 and 1,192.6 and 1,532.3 and 1,607.8 and 1,809.5 and 1,853.5 and 2,003.2 and 3,005.3 and 3,497.2 and 5,553.3 and 10,446.6 and 10,768.5 and 30,770.3 and 67,724.5 and 77,570.6 and 114,021.9  (under budget strategies 03, 04, 05, 06, 07, 08, 09, 10, 11, 12, 13, 14, 15, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28)
+FY2024 programme 0901: 1,984.7 and 64,985.7  (under budget strategies 28, 99)
+FY2024 programme 0902: 216.8 and 500.0 and 2,000.0 and 6,362.3 and 6,415.9 and 26,568.8 and 27,153.3  (under budget strategies 05, 11, 12, 19, 20, 23, 28)
+FY2024 programme 0903: 2,007.3 and 557,096.8  (under budget strategies 09, 28)
+FY2024 programme 0909: 0.0 and 0.3 and 0.8 and 5.3 and 149.6 and 246.0 and 1,502.0 and 116,778.3  (under budget strategies 04, 07, 12, 19, 23, 25, 26, 28)
+FY2024 programme 0910: 0.1 and 0.7 and 4.4 and 1,525.5  (under budget strategies 10, 14, 26, 28)
+FY2024 programme 1144: 0.0 and 14,910.1  (under budget strategies 20, 28)
+FY2024 programme 1149: 20.2 and 54.2  (under budget strategies 04, 14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brazil/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>3 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>brazil_strategy_rows.xlsx was written 2026-08-10; 3_strategy_extraction.txt was edited 2026-08-19
+brazil_budget_2021.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12
+brazil_budget_2024.xlsx was written 2026-08-09; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Strategy named after the budget line funding it</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / panel + match_review</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>13 strategy(ies) consolidate an intervention that is not in the plan extraction and whose name is exactly the budget programme funding them. The match is a name matching itself, and it reads on the page as a plan strategy that the budget funds perfectly.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Electricity generation, transmission and dis &lt;- named after budget line Electricity supply projects under the 12th N
+Agricultural development area infrastructure &lt;- named after budget line Infrastructure provision for enhancement of 
+Airport infrastructure modernisation and avi &lt;- named after budget line Airport infrastructure modernisation project
+Climate policy, emissions reduction and gree &lt;- named after budget line Green Building initiatives under the 12th Na
+Research, innovation and commercialisation s &lt;- named after budget line Research and innovation allocations under th
+Sewerage system upgrading and sanitation inf &lt;- named after budget line Construction programme for sewerage and wast
+Scholarships and human resource funding for  &lt;- named after budget line Scholarships through the Ministry of Educati
+Tourism product and cultural asset upgrading &lt;- named after budget line Tourism product improvement projects under t</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/brunei/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>5 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>brunei_strategy_rows.xlsx was written 2026-08-10; 3_strategy_extraction.txt was edited 2026-08-19
+brunei_budget_2021.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2022.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2025.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12
+brunei_budget_2026.xlsx was written 2026-08-10; 5_budget_extraction.txt was edited 2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 reconciliation_mismatch 1: programs sum to 1,912.5 but strategy_total is 1,949.8 (gap 37.3) - a program line is likel
+FY2025 reconciliation_mismatch 3: programs sum to 626.7 but strategy_total is 624.9 (gap -1.8) - a program line is likely mi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>2 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 strategy 1: printed 1,949.8, programmes sum to 1,912.5, apart by 37.3
+FY2025 strategy 3: printed 624.9, programmes sum to 626.7, apart by -1.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/fiji/</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>fiji_strategy_rows.xlsx was written 2026-08-15; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>29 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>FY2018 national_basis_programmes : head totals sum to 4,529,133.6 but the programmes beneath them sum to 3,944,011.0 (13% apa
+FY2017 reconciliation_mismatch 22: programs sum to 321,245.4 but strategy_total is 321,245.6 (gap 0.2) - a program line is li
+FY2017 reconciliation_mismatch 24: programs sum to 113,354.0 but strategy_total is 113,354.1 (gap 0.1) - a program line is li
+FY2017 reconciliation_mismatch 25: programs sum to 23,096.7 but strategy_total is 23,096.6 (gap -0.1) - a program line is lik
+FY2017 reconciliation_mismatch 33: programs sum to 28,538.8 but strategy_total is 42,329.9 (gap 13,791.1) - a program line is
+FY2017 reconciliation_mismatch 40: programs sum to 133,737.9 but strategy_total is 134,178.0 (gap 440.1) - a program line is 
+FY2017 reconciliation_mismatch 50: programs sum to 615,572.2 but strategy_total is 628,116.8 (gap 12,544.6) - a program line 
+FY2017 reconciliation_mismatch 52: programs sum to 364,701.0 but strategy_total is 354,607.9 (gap -10,093.1) - a program line</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>28 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 22: printed 321,245.6, programmes sum to 321,245.4, apart by 0.2
+FY2017 strategy 24: printed 113,354.1, programmes sum to 113,354.0, apart by 0.1
+FY2017 strategy 25: printed 23,096.6, programmes sum to 23,096.7, apart by -0.1
+FY2017 strategy 33: printed 42,329.9, programmes sum to 28,538.8, apart by 13,791.1
+FY2017 strategy 40: printed 134,178.0, programmes sum to 133,737.9, apart by 440.1
+FY2017 strategy 50: printed 628,116.8, programmes sum to 615,572.2, apart by 12,544.6
+FY2017 strategy 52: printed 354,607.9, programmes sum to 364,701.0, apart by -10,093.1
+FY2018 strategy 2: printed 14,262.3, programmes sum to 23,891.3, apart by -9,629.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/jamaica/</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>jamaica_strategy_rows.xlsx was written 2026-08-14; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>77 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 national_basis_programmes : head totals sum to 278,267,320.0 but the programmes beneath them sum to 239,480,965.0 (14%
+FY2022 national_basis_programmes : head totals sum to 302,576,866.0 but the programmes beneath them sum to 404,258,046.0 (25%
+FY2024 national_basis_programmes : head totals sum to 458,257,529.0 but the programmes beneath them sum to 639,705,043.0 (28%
+FY2019 reconciliation_mismatch 01000: programs sum to 83,000.0 but strategy_total is 290,111.0 (gap 207,111.0) - a program line 
+FY2019 reconciliation_mismatch 08000: programs sum to 642,858.0 but strategy_total is 469,975.0 (gap -172,883.0) - a program lin
+FY2019 reconciliation_mismatch 09000: programs sum to 712,147.0 but strategy_total is 833,920.0 (gap 121,773.0) - a program line
+FY2019 reconciliation_mismatch 15010: programs sum to 0.0 but strategy_total is 697,424.0 (gap 697,424.0) - a program line is li
+FY2019 reconciliation_mismatch 15020: programs sum to 900,480.0 but strategy_total is 10,480.0 (gap -890,000.0) - a program line</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>74 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>FY2019 strategy 01000: printed 290,111.0, programmes sum to 83,000.0, apart by 207,111.0
+FY2019 strategy 08000: printed 469,975.0, programmes sum to 642,858.0, apart by -172,883.0
+FY2019 strategy 09000: printed 833,920.0, programmes sum to 712,147.0, apart by 121,773.0
+FY2019 strategy 15010: printed 697,424.0, programmes sum to 0.0, apart by 697,424.0
+FY2019 strategy 15020: printed 10,480.0, programmes sum to 900,480.0, apart by -890,000.0
+FY2019 strategy 16049: printed 225,234.0, programmes sum to 489,234.0, apart by -264,000.0
+FY2019 strategy 17000: printed 11,525,361.0, programmes sum to 6,345,325.0, apart by 5,180,036.0
+FY2019 strategy 19046: printed 1,078,318.0, programmes sum to 1,085,718.0, apart by -7,400.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a year</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>7 programme-year(s) carry more than one amount, because the same code appears under more than one budget strategy. Every consumer that keys on (year, programme) then has to pick one, and they do not all pick the same one.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 programme 0106000: 346,691,310.0 and 364,590,743.0  (under budget strategies 1094, 1095)
+FY2025 programme 0207000: 231,885,786.0 and 278,922,194.0  (under budget strategies 1122, 1123)
+FY2025 programme 0412000: 651,366,934.0 and 16,529,119,104.0  (under budget strategies 1082, 1083)
+FY2025 programme 0508000: 297,799,258.0 and 435,378,299.0 and 4,677,027,195.0  (under budget strategies 1064, 1065, 1066)
+FY2025 programme 0709000: 233,471,082.0 and 444,125,877.0  (under budget strategies 1072, 1213)
+FY2025 programme 0710000: 2,000,000.0 and 8,769,275,002.0  (under budget strategies 1072, 1213)
+FY2025 programme 1018000: 30,500,000.0 and 12,916,448,407.0  (under budget strategies 1331, 1332)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/kenya/</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>kenya_strategy_rows.xlsx was written 2026-08-14; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>8 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 reconciliation_mismatch 0106000: programs sum to 349,247,063.0 but strategy_total is 276,081,719.0 (gap -73,165,344.0) - a 
+FY2020 reconciliation_mismatch 0508000: programs sum to 2,991,357,360.0 but strategy_total is 164,025,309.0 (gap -2,827,332,051.0)
+FY2020 reconciliation_mismatch 1014000: programs sum to 7,655,824,962.0 but strategy_total is 0.0 (gap -7,655,824,962.0) - a progr
+FY2020 reconciliation_mismatch 1018000: programs sum to 10,066,601,747.0 but strategy_total is 10,873,301,747.0 (gap 806,700,000.0
+FY2025 reconciliation_mismatch 0106000: programs sum to 418,347,116.0 but strategy_total is 346,691,310.0 (gap -71,655,806.0) - a 
+FY2025 reconciliation_mismatch 0508000: programs sum to 3,536,217,818.0 but strategy_total is 435,378,299.0 (gap -3,100,839,519.0)
+FY2025 reconciliation_mismatch 0709000: programs sum to 234,021,081.0 but strategy_total is 233,471,082.0 (gap -549,999.0) - a pro
+FY2025 reconciliation_mismatch 0710000: programs sum to 4,177,242,813.0 but strategy_total is 2,000,000.0 (gap -4,175,242,813.0) -</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>8 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 strategy 0106000: printed 276,081,719.0, programmes sum to 349,247,063.0, apart by -73,165,344.0
+FY2020 strategy 0508000: printed 164,025,309.0, programmes sum to 2,991,357,360.0, apart by -2,827,332,051.0
+FY2020 strategy 1014000: printed 0.0, programmes sum to 7,655,824,962.0, apart by -7,655,824,962.0
+FY2020 strategy 1018000: printed 10,873,301,747.0, programmes sum to 10,066,601,747.0, apart by 806,700,000.0
+FY2025 strategy 0106000: printed 346,691,310.0, programmes sum to 418,347,116.0, apart by -71,655,806.0
+FY2025 strategy 0508000: printed 435,378,299.0, programmes sum to 3,536,217,818.0, apart by -3,100,839,519.0
+FY2025 strategy 0709000: printed 233,471,082.0, programmes sum to 234,021,081.0, apart by -549,999.0
+FY2025 strategy 0710000: printed 2,000,000.0, programmes sum to 4,177,242,813.0, apart by -4,175,242,813.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/malaysia/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>malaysia_strategy_rows.xlsx was written 2026-08-15; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>143 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>FY2022 national_basis_programmes : head totals sum to 171,388,197,600.0 but the programmes beneath them sum to 207,930,952,40
+FY2023 national_basis_programmes : head totals sum to 172,422,614,400.0 but the programmes beneath them sum to 400,992,145,50
+FY2024 national_basis_programmes : head totals sum to 240,919,693,600.0 but the programmes beneath them sum to 383,800,740,10
+FY2025 national_basis_programmes : head totals sum to 162,973,371,700.0 but the programmes beneath them sum to 332,910,058,30
+FY2026 national_basis_programmes : head totals sum to 218,690,309,800.0 but the programmes beneath them sum to 366,392,668,00
+FY2022 reconciliation_mismatch 1: programs sum to 19,215,800.0 but strategy_total is 13,533,000.0 (gap -5,682,800.0) - a pro
+FY2022 reconciliation_mismatch 10: programs sum to 3,621,353,400.0 but strategy_total is 5,254,500.0 (gap -3,616,098,900.0) -
+FY2022 reconciliation_mismatch 11: programs sum to 10,635,228,700.0 but strategy_total is 1,969,500.0 (gap -10,633,259,200.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>138 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>FY2022 strategy 1: printed 13,533,000.0, programmes sum to 19,215,800.0, apart by -5,682,800.0
+FY2022 strategy 2: printed 1,337,000.0, programmes sum to 2,500,000.0, apart by -1,163,000.0
+FY2022 strategy 3: printed 110,000,000.0, programmes sum to 111,286,000.0, apart by -1,286,000.0
+FY2022 strategy 4: printed 836,700.0, programmes sum to 128,970,400.0, apart by -128,133,700.0
+FY2022 strategy 5: printed 564,000.0, programmes sum to 20,919,000.0, apart by -20,355,000.0
+FY2022 strategy 6: printed 504,000.0, programmes sum to 5,704,861,700.0, apart by -5,704,357,700.0
+FY2022 strategy 7: printed 2,465,300.0, programmes sum to 256,675,300.0, apart by -254,210,000.0
+FY2022 strategy 8: printed 11,000.0, programmes sum to 75,123,900.0, apart by -75,112,900.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/maldives/</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>maldives_strategy_rows.xlsx was written 2026-08-15; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>56 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 national_basis_programmes : head totals sum to 23,007,352,858.0 but the programmes beneath them sum to 30,206,084,611.
+FY2018 national_basis_programmes : head totals sum to 21,753,879,903.0 but the programmes beneath them sum to 1,899,491,365.0
+FY2019 national_basis_programmes : head totals sum to 121,034,448.3 but the programmes beneath them sum to 26,257.5 (100% apa
+FY2017 reconciliation_mismatch 1: programs sum to 371,971,798.0 but strategy_total is 101,334,724.0 (gap -270,637,074.0) - a
+FY2017 reconciliation_mismatch 10: programs sum to 603,169,808.0 but strategy_total is 35,391,792.0 (gap -567,778,016.0) - a 
+FY2017 reconciliation_mismatch 11: programs sum to 84,903,354.0 but strategy_total is 59,843,651.0 (gap -25,059,703.0) - a pr
+FY2017 reconciliation_mismatch 12: programs sum to 0.0 but strategy_total is 6,993,896.0 (gap 6,993,896.0) - a program line i
+FY2017 reconciliation_mismatch 13: programs sum to 0.0 but strategy_total is 3,626,872.0 (gap 3,626,872.0) - a program line i</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>52 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 strategy 1: printed 101,334,724.0, programmes sum to 371,971,798.0, apart by -270,637,074.0
+FY2017 strategy 2: printed 208,402,975.0, programmes sum to 1,780,849,664.0, apart by -1,572,446,689.0
+FY2017 strategy 3: printed 10,854,474.0, programmes sum to 291,704,544.0, apart by -280,850,070.0
+FY2017 strategy 4: printed 367,654,006.0, programmes sum to 952,692,855.0, apart by -585,038,849.0
+FY2017 strategy 5: printed 35,615,361.0, programmes sum to 796,853,288.0, apart by -761,237,927.0
+FY2017 strategy 6: printed 19,009,362.0, programmes sum to 2,294,511,756.0, apart by -2,275,502,394.0
+FY2017 strategy 7: printed 22,661,255.0, programmes sum to 266,705,093.0, apart by -244,043,838.0
+FY2017 strategy 8: printed 27,923,748.0, programmes sum to 494,853,833.0, apart by -466,930,085.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>D12</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>An output predates the prompt that produced it</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/thailand/</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>1 output(s) were produced by a version of the prompt that no longer exists. Whatever the edit fixed is not fixed here, and the country's figures are from the older rule.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>thailand_strategy_rows.xlsx was written 2026-08-10; 3_strategy_extraction.txt was edited 2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2024. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>4 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0033 Management and maintenance programme of the Judiciary Branch
+FY2024 0151 Protection of indigenous lands, territorial management and e
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIAIS
+FY2024 1144 AGROPECUARIA SUSTENTAVEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>37 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Multimodal logistics and transport efficiency
+Sports and physical activity promotion
+Climate adaptation, mitigation and disaster risk management
+Productive inclusion and income generation for poor households
+Advance racial equality, anti-racism and affirmative action
+International cooperation and consular action for sustainable developm
+Export diversification and trade integration
+Fiscal reform, tax compliance and revenue integrity</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>4 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 zero_amount_programme 02: programme carries no money; a strategy matched only to lines like this reads as funded whi
+FY2024 zero_amount_programme 14: programme carries no money; a strategy matched only to lines like this reads as funded whi
+FY2024 zero_amount_programme 23: programme carries no money; a strategy matched only to lines like this reads as funded whi
+FY2024 zero_amount_programme 28: programme carries no money; a strategy matched only to lines like this reads as funded whi</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2025. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>37 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>National development planning, project appraisal and implementation co
+Government offices, border posts and overseas representation facilitie
+Environmental impact assessment and pollution control enforcement
+Road, bridge and transport infrastructure improvement
+National security, defence modernisation and policing facilities
+Sports and community recreation facilities upgrading
+MSME development and business environment improvement
+Whole-of-nation implementation and institutional capacity support</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>1 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 30.5 Land Drainage and Flood Protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>23 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Promote digital services exports and the outsourcing industry
+Promote civic values, ethics and social cohesion
+Modernise construction standards, skills and climate-resilient buildin
+Strengthen defence, regional security alliances and emergency assistan
+Audio-visual industry regulation, incentives and ecosystem development
+Inclusive insurance and microinsurance expansion
+Virtual assets, anti-fraud and financial integrity regulation
+Construction regulation, licensing and building code enforcement</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>21 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 program_missing_in_year 23: program '23.2' (Housing) exists in ['2018', '2019'] but is absent in ['2017'] - check whet
+FY2017 program_missing_in_year 26: program '26.1' (Higher Education Institutions) exists in ['2018', '2019'] but is absent in
+FY2017,2018 program_missing_in_year 13: program '13.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '2
+FY2017,2018 program_missing_in_year 34: program '34.6' (Micro, Small and Medium Enterprises Central Coordinating Agency) exists in
+FY2017,2018 program_missing_in_year 4: program '4.3' (Public Enterprises) exists in ['2019'] but is absent in ['2017', '2018'] - 
+FY2017,2018 program_missing_in_year 9: program '9.1' (Policy and Administration) exists in ['2019'] but is absent in ['2017', '20
+FY2018,2019 program_missing_in_year 18: program '18.4' (Rehabilitation and Rural Housing) exists in ['2017'] but is absent in ['20
+FY2018,2019 program_missing_in_year 30: program '30.5' (Land Drainage and Flood Protection) exists in ['2017'] but is absent in ['</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>4 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Modernize consular and overseas travel services
+Strengthen monetary policy governance and macroeconomic forecasting
+Provide social protection and insurance for athletes
+Strengthen water and sanitation cooperation and community management</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>200 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2019 program_missing_in_year 03000: program '03000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 05000: program '05000.1.99.157' (Government Audit Services) exists in ['2022', '2024'] but is abs
+FY2019 program_missing_in_year 06000: program '06000.1.03.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 06000: program '06000.1.03.158' (Public Service Personnel Management) exists in ['2022', '2024'] 
+FY2019 program_missing_in_year 07000: program '07000.1.99.001' (Executive Direction and Administration) exists in ['2022', '2024
+FY2019 program_missing_in_year 07000: program '07000.1.99.139' (Protection of Children's Rights) exists in ['2022', '2024'] but 
+FY2019 program_missing_in_year 07000: program '07000.1.99.159' (Combatting Human Trafficking) exists in ['2022', '2024'] but is </t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>19 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 0105060 NAMATA
+FY2020 0120040 Fisheries Research &amp; Development
+FY2020 0620020 Police Vetting
+FY2020 0703050 Coordination of Vision 2030
+FY2020 0712050 Finance Management Services
+FY2020 0715060 International Relations and Cooperation
+FY2020 0733040 Peace and Conflict Management
+FY2020 0740010 Government Clearing Services</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>42 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Security force recruitment, welfare and infrastructure modernization
+National values, ethics and civic participation
+Government services, records and data infrastructure digitization
+Diaspora engagement, information systems and skills transfer
+Diaspora welfare, emergency response and reintegration services
+Forensic capacity and conflict resolution strengthening
+Intergovernmental coordination and whole-of-government delivery
+Public-private partnership and development partner coordination</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>489 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>489</v>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>FY2020 blank_amount 0105000: amount is blank/unparseable.
+FY2020 blank_amount 0120000: amount is blank/unparseable.
+FY2020 blank_amount 0620000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0703000: amount is blank/unparseable.
+FY2020 blank_amount 0712000: amount is blank/unparseable.
+FY2020 blank_amount 0715000: amount is blank/unparseable.
+FY2020 blank_amount 0733000: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>36 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>FY2022 28.030600 Maintenance, Repair and Overhaul (KTMB)
+FY2022 28.031000 Maintenance of the AwAS System
+FY2022 28.031200 Interim Stage Bus Support Fund Program (ISBSF)
+FY2022 28.031300 Stage Bus Service Transformation Program (SBST)
+FY2022 43.030500 Perbadanan PRIMA Malaysia (PRIMA)
+FY2022 43.040700 Fasiliti Pengurusan Sisa Pepejal (SWCorp)
+FY2022 43.990100 PPP - Perkhidmatan Pengurusan Sisa Pepejal dan Pembersihan A
+FY2022 43.990200 PPP - Tapak Pelupusan Sanitari Sisa Pepejal Ladang Tanah Mer</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>44 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Productivity nexus expansion and programme rationalisation
+Expand green city planning and urban sustainability action
+Water governance, legislation and institutional reform
+Adaptive Plan Implementation, Review and Monitoring Reform
+Whole-of-Nation SDG Localisation and Public Engagement
+Green and Circular Construction Materials and Building Practices
+Industrial Estates, Food Production Areas and Domestic Investment Supp
+Financial Intermediation and Innovation Financing Ecosystem</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>3965 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="n">
+        <v>3965</v>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FY2022 malformed_code_repaired 1: program_code '010000' looked malformed and was normalized to '1.010000' - verify against s
+FY2022 malformed_code_repaired 1: program_code '020000' looked malformed and was normalized to '1.020000' - verify against s
+FY2022 malformed_code_repaired 1: program_code '030000' looked malformed and was normalized to '1.030000' - verify against s
+FY2022 malformed_code_repaired 10: program_code '010000' looked malformed and was normalized to '10.010000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '020000' looked malformed and was normalized to '10.020000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '030000' looked malformed and was normalized to '10.030000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '040000' looked malformed and was normalized to '10.040000' - verify against 
+FY2022 malformed_code_repaired 10: program_code '050000' looked malformed and was normalized to '10.050000' - verify against </t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Programme lines carrying zero</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / budget_all_years</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>110 programme line(s) extracted with an amount of 0. Either the document prints a nil allocation, or the amount sat somewhere the extractor did not look.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 1.5 ieri
+FY2017 20.003 Beim ein ige, She's jeg;
+FY2017 26.009 jeg 932
+FY2018 1.003 Sp 322 9892
+FY2018 19.004 Amd Marmido
+FY2018 22.003 :22 823, VP 29335
+FY2018 22.066 gå sirve HABE ich give
+FY2018 22.073 eisen Pixie</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>251 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>251</v>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Affordable and social housing delivery
+Coral reef rehabilitation and marine biodiversity restoration
+Climate-smart and environmentally sustainable agriculture
+Governance quality improvement
+Teacher development, school leadership and education governance
+Equitable school access and inclusive learning support
+Unemployment protection and income support for vulnerable groups
+Substance use prevention, treatment and rehabilitation services</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>1072 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>1072</v>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 blank_amount 1: amount is blank/unparseable.
+FY2017 blank_amount 20: amount is blank/unparseable.
+FY2017 blank_amount 26: amount is blank/unparseable.
+FY2017 blank_amount 37: amount is blank/unparseable.
+FY2017 blank_amount 38: amount is blank/unparseable.
+FY2017 blank_amount 39: amount is blank/unparseable.
+FY2018 blank_amount 1: amount is blank/unparseable.
+FY2018 blank_amount 13: amount is blank/unparseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>3 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Support and protection for firms and workers affected by EV transition
+High-skill talent attraction, mobility, and retention
+National monitoring, evaluation, and adaptive management system</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>6 medium flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>FY2023 program_missing_in_year 2: program '2.16' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023 program_missing_in_year 5: program '5.10' (Program on Public Sector Personnel) exists in ['2024', '2025', '2026'] but
+FY2023,2024 program_missing_in_year 4: program '4.12' (Program on Public Sector Personnel) exists in ['2025', '2026'] but is abse
+FY2023,2024,2026 program_missing_in_year 2: program '2.17' (Program on Public Sector Personnel) exists in ['2025'] but is absent in ['
+FY2023,2025 program_missing_in_year 7: program '7.3' (Program on Expenditures for Replenishment of Treasury Account Balance) exis
+FY2024,2025 program_missing_in_year 1: program '1.14' (Program on Public Sector Personnel) exists in ['2023', '2026'] but is abse</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>42 distinct programme(s) across 90 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 0907 Special operations: refinancing of internal   1,663,914.8
+FY2024 0905 Special operations: internal debt service (i  668,292.5
+FY2024 0903 OPERACOES ESPECIAIS: TRANSFERENCIAS CONSTITU  557,096.8
+FY2024 0909 OPERACOES ESPECIAIS: OUTROS ENCARGOS ESPECIA  116,778.3
+FY2024 0032 Management and maintenance programme of the   114,021.9
+FY2024 0999 Contingency reserve  89,578.8
+FY2024 0032 Management and maintenance programme of the   77,570.6
+FY2024 0032 Management and maintenance programme of the   67,724.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>9 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 1149 -&gt; participatory budgeting, transparency an (x2)
+FY2024 2317 -&gt; regional development, territorial planni (x5)
+FY2024 2320 -&gt; implement intersectoral support and hous (x2)
+FY2024 2321 -&gt; water security and integrated water reso (x3)
+FY2024 2322 -&gt; basic sanitation and urban environmental (x2)
+FY2024 5115 -&gt; access to justice and justice system imp (x3)
+FY2024 5115 -&gt; defend democracy and strengthen institut (x2)
+FY2024 5115 -&gt; improve access to justice and legal righ (x3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>7 distinct programme(s) across 7 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 1.12 Payment for medical treatment services at Gl  150.0
+FY2025 2.10 IT Central Procurement projects and software  144.7
+FY2025 1.11 Purchase of medicines, medical consumables a  89.0
+FY2025 3.7 Focus projects to support the budget focus a  27.5
+FY2025 1.18 Natural disaster management  25.0
+FY2025 1.6 Education information and data management sy  21.2
+FY2025 3.6 Research costs for public higher education i  2.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>43 distinct programme(s) across 91 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 50.10 Standard Expenditure Group 10  442,060.3
+FY2019 22.1 Policy and Administration  123,905.0
+FY2018 26.1 Higher Education Institutions  123,789.1
+FY2019 26.1 Higher Education Institutions  115,587.2
+FY2018 19.1 Republic of Fiji Military Forces  103,252.1
+FY2017 19.1 Republic of Fiji Military Forces  96,688.5
+FY2018 22.1 Policy and Administration  85,470.5
+FY2019 9.1 Policy and Administration  84,724.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>102 distinct programme(s) across 164 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>FY2024 26000.1.01.437 Territorial and Sovereign Protection  41,716,884.0
+FY2022 26000.1.01.437 Territorial and Sovereign Protection  28,230,476.0
+FY2024 20000.6.99.137 Management of Public Finances  24,535,325.0
+FY2019 26000.1.01.400 Defense Forces Services  22,376,754.0
+FY2024 26022.1.01.001 Executive Direction and Administration  20,505,357.0
+FY2022 42000.1.01.001 Executive Direction and Administration  12,968,255.0
+FY2019 26000.6.01.400 Defense Forces Services  12,569,794.0
+FY2022 26022.1.01.001 Executive Direction and Administration  11,233,758.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>505 distinct programme(s) across 641 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 0509000 Teacher Resource Management  347,685,463,808.0
+FY2025 0509010 Teacher Management- Primary  201,136,266,225.0
+FY2025 0801010 National Defense  169,815,800,000.0
+FY2025 0509020 Teacher management - Secondary  142,015,327,079.0
+FY2025 0502020 Free Day Secondary Education  102,527,921,685.0
+FY2025 0717000 General Administration Planning and Support   76,480,295,458.0
+FY2020 0502020 Free Day Secondary Education  67,274,154,762.0
+FY2025 0504010 University Education  67,180,896,533.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>D9</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>One pair matched twice, once per pass</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / match_review</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>1 programme-strategy pair(s) were reached by both the strategy pass and the reverse pass, so they carry two rationales. The panel credits the pair once; only a row COUNT would double it.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 1018000 -&gt; forest protection and environmental comp (x2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>957 distinct programme(s) across 1943 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>FY2025 13.010000 FAEDAH, DIVIDEN DAN LAIN-LAIN KENAAN BAYARAN  54,700,000,500.0
+FY2024 13.010000 INTEREST, DIVIDENDS AND OTHER DEBT CHARGES O  49,800,000,000.0
+FY2023 11.020000 TRANSFER PAYMENTS AND GRANTS  49,502,871,200.0
+FY2023 13.010000 INTEREST, DIVIDENDS AND OTHER DEBT SERVICE C  46,100,000,000.0
+FY2024 11.020000 TRANSFER PAYMENTS AND GRANTS  45,724,636,400.0
+FY2022 13.010000 INTEREST, DIVIDENDS AND OTHER CHARGES ON NAT  43,100,000,000.0
+FY2026 11.020000 TRANSFER PAYMENTS AND GRANTS  37,620,151,300.0
+FY2024 42.000000 Mengurus  35,150,181,800.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>666 distinct programme(s) across 836 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>FY2017 19.002 et Lille Da Pi, ja gien  6,994,664,737.0
+FY2018 19.001 die Ci 29, 9 28?  1,504,471,755.0
+FY2017 30.001 xixe"jin Ds sind ja sei?  1,490,542,683.0
+FY2017 6.3 And a great قوم  1,473,416,147.0
+FY2017 2.1 ing in  1,455,757,190.0
+FY2017 21.002 وفيد ؤونه قومه مادونه  1,334,531,645.0
+FY2017 19.003 ¿ ¿ iii  1,225,233,300.0
+FY2017 20.002 - pij, ;22 29,99  1,019,664,729.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>38 distinct programme(s) across 120 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 3.8 Program on Public Sector Personnel  429,643.3
+FY2026 7.2 Program on Management of Public Debt  421,864.4
+FY2025 3.8 Program on Public Sector Personnel  416,438.4
+FY2025 7.2 Program on Management of Public Debt  410,253.7
+FY2024 3.8 Program on Public Sector Personnel  403,992.0
+FY2023 3.8 Program on Public Sector Personnel  403,945.1
+FY2026 4.2 Strategic Program on Decentralization to the  377,960.2
+FY2024 7.2 Program on Management of Public Debt  346,380.1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2478,7 +5004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2513,6 +5039,158 @@
         <is>
           <t>TOTAL</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>fiji</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>thailand</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2544,7 +5222,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21 09:28 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-21 09:52 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Final regression rebuild: head capacity, config and handoff gates, Maldives withheld
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -561,12 +561,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>See F1 in FIXES.xlsx. The unit is (year, budget strategy, programme), not (year, programme). Stage 6 must record which budget strategy the matched line sits under, load_budget must key on all three, and the Supabase view must join on all three. Until then the dashboard shows the lower bound. The remaining work is upstream: stage 5 should emit a code that is unique within the year, at which point A3 passes on its own.</t>
+          <t>See F1 in FIXES.xlsx. The unit is (year, budget strategy, programme), not (year, programme). Stage 6 must record which budget strategy the matched line sits under, load_budget must key on all three, and the Supabase view must join on all three. Until then the dashboard shows the lower bound. The remaining work is upstream: stage 5 should emit a code that is unique within the year, at which point A3 passes on its own. DONE 2026-08-21: new check A21 asserts that every accepted edge on a repeated code names its budget head, so the last-row-read fallback is never reached. Brazil has 28 repeated codes and Kenya 7, and no edge in any country omits its head. Migration 0008 fixes the same fault in v_funding_by_program.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Kenya needs nothing further. Jamaica needs stage 5 re-run with a structure hint that emits a total for every head, keeps recurrent and capital apart in the code, and ignores the object-of-expenditure detail. Until then its coverage figure should not be read. More generally, program_code_style should be chosen by measurement rather than defaulted: a code that never matches and a code that matches too much look identical until the totals are compared.</t>
+          <t>Kenya needs nothing further. Jamaica needs stage 5 re-run with a structure hint that emits a total for every head, keeps recurrent and capital apart in the code, and ignores the object-of-expenditure detail. Until then its coverage figure should not be read. More generally, program_code_style should be chosen by measurement rather than defaulted: a code that never matches and a code that matches too much look identical until the totals are compared. DONE 2026-08-21: the style cannot be inferred safely, because Malaysia at 49% code reuse needs prefixing and Brazil at 27% must not have it, so combine_budget_years now FLAGS the contradiction instead of guessing: hierarchical style where under 5% of raw codes begin with their head and under 5% recur across heads raises a HIGH code_style_suspect flag naming the setting to change.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -769,12 +769,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Per-strategy coverage for Malaysia should not be read until this is fixed. The national total and the strategy inventory are unaffected, as is every mapping. The fix is to have Prompt 5 emit the head's short code as printed in the page corner (B.62), which is on every page of the document, and to reject a strategy_total whose source_location does not name a head.</t>
+          <t>Per-strategy coverage for Malaysia should not be read until this is fixed. The national total and the strategy inventory are unaffected, as is every mapping. The fix is to have Prompt 5 emit the head's short code as printed in the page corner (B.62), which is on every page of the document, and to reject a strategy_total whose source_location does not name a head. DONE 2026-08-21: see W13; a head whose printed total under-reports its own programmes is now measured against the programmes.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1185,12 +1185,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Stage 5, not stage 6. Have the extraction emit a total for every strategy and reconcile it against its own programme rows before the layer is written, so the contradiction is caught where it is created. Until then read the ceiling sheet as a report on the budget layer rather than on the edges, and treat a rounding-scale exceedance separately from a structural one.</t>
+          <t>Stage 5, not stage 6. Have the extraction emit a total for every strategy and reconcile it against its own programme rows before the layer is written, so the contradiction is caught where it is created. Until then read the ceiling sheet as a report on the budget layer rather than on the edges, and treat a rounding-scale exceedance separately from a structural one. DONE 2026-08-21: build_final_panel derives a head's CAPACITY, its printed total or, where that under-reports its own countable programmes by more than 5%, the programme sum, and both the ceiling and the coverage share use it. 101 of Malaysia's 200 head-years and 43 of Jamaica's 79 are recomputed, and coverage above 105% falls from 5 head-years to zero across all countries. Both sheets now carry printed_total and total_basis so the substitution is visible.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1498,12 +1498,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Remove that line from 6b only and re-run one country, diffing against the coverage workbook already on disk. Jamaica was the obvious candidate until its budget turned out to be genuinely administration-heavy; Fiji is the cleaner test. Gated on W18, because without precision numbers a rise in edges cannot be read either way.</t>
+          <t>Remove that line from 6b only and re-run one country, diffing against the coverage workbook already on disk. Jamaica was the obvious candidate until its budget turned out to be genuinely administration-heavy; Fiji is the cleaner test. Gated on W18, because without precision numbers a rise in edges cannot be read either way. DONE 2026-08-21: prompt 6b no longer carries prompt 6's clamp. It states why its bar is deliberately lower (it exists to recover the siblings the strategy-side pass missed, and cannot inflate a strategy's money because the amount is attributed per programme once), while still refusing sector adjacency alone and overhead lines. Takes effect on the next 6b run.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1602,12 +1602,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>One document profile per country, in one file, with four mechanisms: how to read it, where the levels sit, how the codes are shaped, and how the amounts are labelled. The code is already generic; it is the configuration that is scattered.</t>
+          <t>One document profile per country, in one file, with four mechanisms: how to read it, where the levels sit, how the codes are shaped, and how the amounts are labelled. The code is already generic; it is the configuration that is scattered. DONE 2026-08-21: check_configs.py compares the two per-country config files and the paths they name, and runs in the test suite. It found two real faults on its first run: bhutan and kiribati name mapping folders that are not here. HIGH blocks, advisory does not, because a country not yet mapped is a normal state.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1654,12 +1654,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Decide whether the pack is maintained or retired. If maintained, generate it rather than copying it, which needs the pack's dependency set worked out because the live runner reaches for validators the pack does not have. check_handoff_drift.py measures the gap in the meantime.</t>
+          <t>Decide whether the pack is maintained or retired. If maintained, generate it rather than copying it, which needs the pack's dependency set worked out because the live runner reaches for validators the pack does not have. check_handoff_drift.py measures the gap in the meantime. DONE 2026-08-21: sync_handoff.py copies the five pipeline scripts and all seven prompts into the pack and --check runs in the test suite. It was shipping build_final_panel at 677 lines against a live 977 and combine_budget_years at 372 against 819, and had never carried prompt 5b at all.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Pull Maldives from the published set until its budgets are re-parsed. Document Intelligence renders Thaana as Arabic and then as European nonsense, so the fix is upstream of every prompt. A readability gate belongs in the pipeline: a country whose programme names fail a letters-per-name test should not reach publish_run.  PARTIAL 2026-08-20: new audit check A20 fails any country where more than 20% of programme names are unreadable, and combine_budget_years raises a HIGH data_quality flag for the same. Maldives fails it at 46%; every other country passes at 0%. The country is still published; pulling it is a decision, not a bug fix.</t>
+          <t>Pull Maldives from the published set until its budgets are re-parsed. Document Intelligence renders Thaana as Arabic and then as European nonsense, so the fix is upstream of every prompt. A readability gate belongs in the pipeline: a country whose programme names fail a letters-per-name test should not reach publish_run.  PARTIAL 2026-08-20: new audit check A20 fails any country where more than 20% of programme names are unreadable, and combine_budget_years raises a HIGH data_quality flag for the same. Maldives fails it at 46%; every other country passes at 0%. The country is still published; pulling it is a decision, not a bug fix. DONE 2026-08-21: publish_run now REFUSES a country whose programme names are more than 20% unreadable, naming the share and two examples, and offering --allow-unreadable for a deliberate override. Maldives is refused and its eleven previously published runs were deleted, so it is off the dashboard until its budgets parse.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2596,7 +2596,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21 13:37 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-21 16:38 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Trend chart shows the full ten-year window, with a reason on every gap
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1133,12 +1133,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Do not spend on another stage 5 run until the parse is fixed; no prompt can recover text the parser destroyed. Document Intelligence has no locale for Dhivehi. The options are to parse these documents outside DI with a Thaana-capable extractor and accept the loss of table structure, or to treat Maldives as out of scope for the current toolchain. The translation hint is left in the config so it applies once the text arrives intact.</t>
+          <t>Do not spend on another stage 5 run until the parse is fixed; no prompt can recover text the parser destroyed. Document Intelligence has no locale for Dhivehi. The options are to parse these documents outside DI with a Thaana-capable extractor and accept the loss of table structure, or to treat Maldives as out of scope for the current toolchain. The translation hint is left in the config so it applies once the text arrives intact. FIXED 2026-08-22 by not using OCR at all. These PDFs carry their own embedded text layer holding the real Thaana Unicode: 526,059 Thaana characters in FY2019 against the 0 Document Intelligence returned, because the OCR was matching rendered Thaana glyphs to the nearest Arabic letter. parse.read_text_layer reads the characters directly, which is free, instant and exact, and "parser": "text_layer" in the country config selects it. parse._warn_if_script_mismatch compares the OCR against the file's own text layer on every un-cached parse and names the setting to change, so the whole class is caught for any country. Maldives programme names went from 395 of 852 unreadable to 0 of 56, A20 passes, and the audit went from 15/18 to 17/18.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -2450,6 +2450,58 @@
       <c r="J38" s="2" t="inlineStr">
         <is>
           <t>Malaysia 1,847.9bn all rows vs 1,692.0bn countable</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>W38</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Only about a quarter of the Maldivian budget is extracted, so its coverage share is not comparable</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>With the text layer in place the names are correct English and every check but one passes, but stage 5 takes a sector section rather than the whole budget: 7.99bn MVR for FY2017 and 7.08bn for FY2019 against a national budget of roughly 27-30bn a year, and FY2018 returns nothing at all from a document holding 9,275 printed amounts. The resulting 90.57% is a share of what was extracted, not of the national budget, and sitting beside Brazil's 31.6%, which is a whole budget, it invites exactly the comparison this pipeline exists to make safe. The cause is layout, not script: these tables are right-to-left Thaana in columns, the text layer returns correct characters without column structure, and PyMuPDF's table detection fires on 7 of 60 pages and fragments the cells.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Either give stage 5 the table structure (pymupdf_layout, or reconstructing rows from block coordinates) or extract the per-ministry tables deterministically as was done for Jamaica in W16. Until then Maldives should not be published beside countries whose whole budget is present, or should carry the share of what was extracted under a different label.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>national_total: FY2017 7,988,962,654 and FY2019 7,076,705,474; FY2018 empty</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2648,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21 16:38 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-22 10:22 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Transcript stage at table accuracy; Maldives whole-budget; tiles name their years
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2502,6 +2502,682 @@
       <c r="J39" s="2" t="inlineStr">
         <is>
           <t>national_total: FY2017 7,988,962,654 and FY2019 7,076,705,474; FY2018 empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>W39</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>publishing</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Two migrations in the repo had never been applied to the live database, and the code was designed to hide it</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>0003_access_log.sql and 0005_source_document_type.sql sit in supabase/migrations/ and neither had been run. publish_sources() checks for the doc_type column with column_exists() and, not finding it, publishes every source document with no type and prints one warning line among many. So every publish since 0005 was written silently dropped the field, and the access log has been writing to Files/logs/db_access.jsonl alone with a one-line 'stayed local only' notice. Both degradations are deliberate and correct in isolation; together they mean the repo and the database can diverge indefinitely with nothing that fails.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Apply 0003 and 0005 in the SQL editor. Longer term the publish step should assert the migration level it expects rather than adapting to whatever it finds, so an unapplied migration is a red run rather than a warning.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>select source_documents?select=doc_type -&gt; 400 'column source_documents.doc_type does not exist'; select access_log -&gt; 404 'Could not find the table public.access_log'</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>brunei, malaysia</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>The filename rule types any document containing the substring 'plan' as an NDP, which would have filed two sector strategies as the national plan</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>fetch_sources.type_from_name() matches the bare substring 'plan', so 'Digital Economy Masterplan 2025.pdf' (Brunei) and 'Industrial Masterplan 2030.pdf' (Malaysia) both come out doc_type 'ndp'. The NDP is the anchor of the whole analysis: Prompts 1 and 3 read it, its interventions become the strategies that money is matched to, and its risk grid drives every funding_priority. A sector strategy entering that set would contaminate the anchor with no check able to see it, because nothing downstream records which document a strategy came from.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. type_from_folder() now outranks every other signal, so the mirror subdirectory decides the type and the filename is only consulted for a file sitting at the top level. run_llm_pipeline.py additionally refuses a config that lists one document as both an NDP and a sector strategy.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>type_from_name('Digital Economy Masterplan 2025.pdf') returned 'ndp' before the change; both files now type as 'sector'</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>W41</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>A dry run spent real money on Document Intelligence while reporting that it spent none</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>--dry-run is documented as 'cost estimate, 0 calls' and stops the model calls, but parsing runs before the ledger exists and Document Intelligence bills per page. Estimating Brunei's sector corpus parsed 86 pages at $0.01 before timing out on the next document, so the command that exists to avoid spending money spent $0.86 and then crashed. It went unnoticed until now because every previous dry run was over documents already in the parse cache, where parsing is free.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. parse.DRY_RUN makes an uncached document read from its own text layer instead, which is free, and counts the pages the real run will be billed for so the estimate still carries them.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>HttpResponseError (Timeout) raised from _analyze during --dry-run; PAGES_PARSED['parsed'] was 86 at the time</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>W42</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Document Intelligence slicing triggered on page count alone, so a short but very large document still timed out</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Long documents are split into 150-page slices because the service gives up on one long operation. Size was never part of the rule. Brunei's 'Digital Brunei 2030' is 22 pages and 38 MB, full-page images at 1.8 MB each: it passed under the page threshold, went up as a single 38 MB operation and returned '(Timeout) The operation was timeout'.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. The slice size is now the smaller of the page limit and a 10 MB byte budget, and a timeout retries once at half the slice size.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>39,843,726 bytes over 22 pages; sliced at 5 pages it parsed to 759 paragraphs across all 22 pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>W43</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Nothing could read the pv2-sources bucket, so a document added to it by hand was invisible to the pipeline</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>db.Supabase had upload() and ensure_bucket() and no list or download. The bucket is described as the library of record and is where the sector strategies were added, but the flow was one-way: the only way to get a document into Files/sources/&lt;slug&gt;/ was to already have it. countries/malaysia.json had also been declaring sources.backend 'http', which is not a backend fetch_sources.py supports; it fell through to graph and the country had never been published to source_documents at all.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. db.list_objects() and db.download() added, a 'supabase' backend in fetch_sources.py with --from-bucket and --type, and an unknown backend is now a config error instead of a silent fallback. Both configs corrected.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>source_documents held 7 brunei rows and 0 malaysia rows; the bucket held 15 brunei objects including 8 under 'sector strategies/'</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>W44</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>The sector risk grid counts mentions per paragraph like the plan grid, but the two grids are still not comparable on that number alone</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Prompt 2's 'mentions' is the count of evidence-bearing chunks, and salience is read from it together with the Likert key-part score. The sector pass runs the same prompt at the same paragraph granularity, so the counts ARE on the same scale, but the documents are not: a 100-page sector blueprint and a 184-page national plan produce different chunk counts for the same emphasis. Salience bands and direction are the comparable fields; raw mentions are not, and subtracting one from the other would be meaningless.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Compare on salience and direction. v_ndp_sector_gap does exactly that and never differences the two mention counts. If a numeric comparison is ever wanted, normalise by chunks per document first.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Brunei NDP risk grid 2,970 chunks over three plans; Economic Blueprint 2035 alone 493 chunks</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>W45</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Stage 5 now emits a 'grand_total' line_type that the L2 schema gate, and the database, both refuse</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>The grand-total row was added so a budget layer can prove itself against the document's own printed total. Two things downstream were not moved with it. validate_stage_schema.py still allows only ['strategy_total', 'program'], so the L2 gate - a blocking gate - now reports FAIL on clean data for every country whose budget carries one; tamper_test.py reads that as 'schema is not protecting anything', which is a FALSE POSITIVE and worse than a miss, because a gate that cries wolf on good data is a gate people learn to ignore. And budget_lines.line_type carries a CHECK constraint allowing only strategy_total / program / national (0006), so those rows are refused at publish exactly as the 'national' rows were before 0006 (see the fallback already written into publish_run.push).</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22, in three places, because the value had to be accepted at each. validate_stage_schema.py allows 'grand_total' in the stage 5 line_type enum, so the L2 gate passes on clean data and still catches an injected bad value. publish_run.budget_rows() accepts it instead of raising - the raise was the real blocker, because it fired before the existing degrade-gracefully fallback could run, so the publish failed rather than dropping a row. Migration 0010 extends the budget_lines CHECK constraint, and the fallback in publish_run.push is now a LIST of optional line types rather than one hard-coded value, since this has now happened twice ('national' needed 0006, 'grand_total' needs 0010). No view was touched: every one filters line_type by positive equality, so a new value cannot fall into an existing total.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Brunei stage 5 output: {'grand_total': 3, 'strategy_total': 3, 'program': 41}; tamper_test --country brunei -&gt; FALSE POSITIVE schema; live budget_lines holds only strategy_total and program</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>W46</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>precision-recall</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>'Not in the NDP' mixes a genuine gap with a specification of something the plan already carries, and the flag does not separate them</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>198 of Brunei's 414 sector interventions came back in_ndp='no' (48%). Reading them, the flag is doing what Prompt 7 asks - the prompt states that being BROADER is not a match, so where the plan holds the aspiration and the sector strategy holds the actual intervention the answer is 'no' - but two quite different findings end up under one label. 'The NDP includes reforestation itself but does not specifically carry dedicated funding and financing mechanisms for it' is a specification of an existing plan commitment. 'The NDP does not include a specific programme of language promotion, legislation and education' is a topic the plan is silent on. A reader taking 198 as 'policy areas the plan ignores' would be wrong about most of them.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>The rationale text distinguishes the two on every row and the dashboard shows it, so nothing is hidden. To separate them properly Prompt 7 needs a third state (silent / broader / present) rather than a boolean, which is a prompt change and a re-run. Until then read the rationale, not the count.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>brunei_sector_responses.xlsx: 198 of 414 in_ndp='no'; per document 29% (Education) to 58% (Climate Change Policy)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>W47</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>One control character in a document's text layer destroyed a run after every model call for it had been paid for</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>openpyxl raises IllegalCharacterError on the control characters XML forbids, rather than dropping them, and writer.py passed extracted text straight through. Malaysia's Education 2026-2035 carries a mangled heading, 'Sekola^ Sedia Masa &gt;adapan &lt;ktkre Ready Sc^ool # &lt;RS', holding a raw control byte. Stage 1 extracted all 3,600 chunks, the write then threw, and the process died with nothing saved for that document. It is not sector-specific: any country whose text layer carries one such byte would lose the run at the same point. The spend was recoverable only because llm.py caches responses - the re-run replayed all 3,600 chunks at $0.00.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. writer._cell strips the forbidden control characters (tab, newline and carriage return are legal and are kept). Stripped rather than escaped: they are artefacts of the PDF's encoding and carry no meaning, and the alternative is losing the file.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>openpyxl.utils.exceptions.IllegalCharacterError raised from writer.write_results via stages.run_stage7_risk; run died at $5.05, re-run replayed from cache at $0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>W48</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>The layer on disk was stale against the code, so a working parser looked like a broken one</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>national_total.grand_total read null for all four Brunei years while three grand_total rows sat in the stage 5 files, which looked like a parsing failure: the amounts are 'B$5,860,000,000.00' beside 'BND6.35 billion', a currency prefix, separators and a magnitude word. combine_budget_years.num() already handles all of that and returns the right figure. The layer had simply been built before that code existed and nothing on disk says how old a derived file is relative to the script that derives it. The wrong conclusion cost real time, and would have cost more had the 'fix' been a second parser competing with the working one.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>No code change needed; re-running combine_budget_years populates it. The general lesson is the one worth keeping: a derived artefact carries no record of the code version that built it, so a stale layer is indistinguishable from a broken stage. Brunei's four years were re-extracted on 2026-08-22 and grand_total now reads 5,860 / 5,860 / 6,250 / 6,350 BND million with extracted_pct against each.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Before re-run: grand_total None for 2021, 2022, 2025, 2026. After: 5860 / 5860 / 6250 / 6350, basis 'grand_total', extracted_pct 96 / 102.9 / 38.4 / 16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>W49</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>lineage.py printed every country's name UNDER the rows it labelled, so the whole table read one country out of step</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>report() printed a country's hop rows and main() printed the country header afterwards, so each heading sat beneath its own rows. Read top-down, Kenya's 36.9% consolidation loss appeared under the JAMAICA heading and the rows under KENYA were Malaysia's. The summary beneath was correct throughout. That is the worse way round: a reader who distrusts a verdict opens the detail, finds a different number against the same country and hop, and stops believing the gate. It cost this session an hour and a wrong conclusion - the contradiction was reported to the user as a defect in the numbers before the cause was found.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22: report() prints the header above its own rows and main() no longer prints one. With the table readable, a second real loss became visible that the misalignment had been hiding (maldives stage 5 -&gt; budget layer, 34.1%).</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Before: KENYA section showed '1451 -&gt; 1438 lost 13 (0.9%)' (Malaysia's row) against a summary of 'kenya ... 509 of 1378'. After: KENYA shows '1378 -&gt; 869 lost 509 (36.9%)', matching the summary exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>W50</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>precision-recall</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Consolidation drops 36.9% of Kenya's extracted interventions, against 0.4-3.1% everywhere else</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Stage 4 consumed 869 of the 1,378 chunks stage 3 extracted an intervention from, so 509 extracted interventions are cited by nothing in the strategy inventory. Every other country loses between 0.4% and 3.1% at the same hop, so this is not the normal cost of folding duplicates away. Kenya carries 281 strategies on the panel and 239 of them are funded, so whatever was dropped was dropped before the money was attached and no downstream check can see it: the panel is internally consistent about the strategies it kept. This was visible only after the lineage table's country labels were fixed (W49).</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Re-run stage 4 for Kenya and compare, or read a sample of the 509 orphaned chunks against the inventory to find what class of intervention is being folded away. Not yet diagnosed; the loss is measured, its cause is not.</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>lineage.py: kenya stage 3 -&gt; stage 4 (consolidation) 1378 -&gt; 869, lost 509 (36.9%); brazil 1.6%, brunei 3.1%, fiji 2.2%, jamaica 0.4%, malaysia 0.9%, maldives 0.8%, thailand 1.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>W51</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>29 of 85 extracted Maldivian programmes do not reach the budget layer</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>stage 5 -&gt; budget layer is a conservation hop: combine_budget_years joins the per-year extractions and should keep every programme row it is given. Maldives loses 34.1% of them, where every other country loses none. It became visible only once the lineage table's country labels were corrected (W49), and it is distinct from W38, which is about how much of the national budget the extraction reaches in the first place; this is loss AFTER extraction, inside our own Python.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Gone on re-extraction, not by a code change here. The Maldives budget was re-extracted on 2026-08-22 and the hop now reads 454 -&gt; 454, nothing lost, where it had read 85 -&gt; 56. The 29 rows were never dropped by combine_budget_years; the extraction they came from was the incomplete one W38 describes. Recorded because the two findings look alike from the lineage table and are not the same thing.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Before: maldives stage 5 -&gt; budget layer 85 -&gt; 56, lost 29 (34.1%). After a re-extraction: 454 -&gt; 454, lost 0 (0.0%), and the country passes every conservation hop.</t>
         </is>
       </c>
     </row>
@@ -2648,7 +3324,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22 10:22 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-22 11:57 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Scale conversion: Fiji 208.6% -> 45.1%; eight Fiji budget years, eleven Maldivian
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>'Not in the NDP' mixes a genuine gap with a specification of something the plan already carries, and the flag does not separate them</t>
+          <t>'The plan does not carry this' merged a subject the plan is silent on with a mechanism for something it already commits to</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2902,12 +2902,13 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>The rationale text distinguishes the two on every row and the dashboard shows it, so nothing is hidden. To separate them properly Prompt 7 needs a third state (silent / broader / present) rather than a boolean, which is a prompt change and a re-run. Until then read the rationale, not the count.</t>
+          <t>Fixed 2026-08-22. Prompt 7's binary in_ndp became ndp_relation with three values - carried, broader_only, silent - and in_ndp is now DERIVED from it (carried -&gt; yes, otherwise no), so audit check A23, the published column, the dashboard and any query already written are unaffected by construction rather than by being updated in step. Migration 0011 adds the column; publish_sector drops it with a warning where 0011 has not been applied. verify_sector_layer.py asserts in_ndp and ndp_relation never disagree, on every row.
+The split is large enough to have changed the reading: Brunei 240 broader_only against 76 silent, Malaysia 573 against 126. So 202 of 756, not 756, are subjects a plan has not addressed.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2917,7 +2918,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>brunei_sector_responses.xlsx: 198 of 414 in_ndp='no'; per document 29% (Education) to 58% (Climate Change Policy)</t>
+          <t>brunei carried 97 / broader_only 240 / silent 76; malaysia carried 414 / broader_only 573 / silent 126. Measured against a golden baseline taken before the prompt change: on the 251 interventions present in both Brunei runs, related_risks held at 94% and HDICategory at 99%.</t>
         </is>
       </c>
     </row>
@@ -3088,9 +3089,9 @@
           <t>precision-recall</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -3100,22 +3101,25 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Consolidation drops 36.9% of Kenya's extracted interventions, against 0.4-3.1% everywhere else</t>
+          <t>Kenya cannot trace 36.9% of its extracted interventions back to a plan chunk, but only 2.8% are actually missing</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Stage 4 consumed 869 of the 1,378 chunks stage 3 extracted an intervention from, so 509 extracted interventions are cited by nothing in the strategy inventory. Every other country loses between 0.4% and 3.1% at the same hop, so this is not the normal cost of folding duplicates away. Kenya carries 281 strategies on the panel and 239 of them are funded, so whatever was dropped was dropped before the money was attached and no downstream check can see it: the panel is internally consistent about the strategies it kept. This was visible only after the lineage table's country labels were fixed (W49).</t>
+          <t>Stage 4 cites 869 of the 1,378 chunks stage 3 extracted an intervention from, leaving 509 uncited against 0.4-3.1% everywhere else. Read as loss - which is how A22 and lineage.py both phrased it - that says a third of Kenya's plan never reached the inventory. It did not. Reading the 509 against the inventory's own strategy names and component_interventions, 470 of them ARE there: Prompt 4 merged them into a strategy and did not list their chunk in source_chunks. Only 39, 2.8% of the plan, are absent by wording too, which is the same rate as every other country.
+Three explanations were tested and rejected before that one: batch size (Kenya's batches are 215 rows, the same as Brunei's 215 and smaller than Fiji's 245, and both of those lose under 3.1%); a stale strategyclean (every country's stage 4 output is newer than its stage 3); and a truncated tail (the uncited chunks run from 452 to 4499, scattered through the document, and none lie beyond the highest cited chunk).
+So the damage is to PROVENANCE, not to the inventory. audit_evidence.py joins a panel figure back to the plan text through source_chunks, and that join is what a high number here breaks.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Re-run stage 4 for Kenya and compare, or read a sample of the 509 orphaned chunks against the inventory to find what class of intervention is being folded away. Not yet diagnosed; the loss is measured, its cause is not.</t>
+          <t>Fixed 2026-08-22, and not by editing Prompt 4. The prompt already states the rule twice ('Preserve every ref', 'Every input ref number appears in exactly one source_chunks array') and Kenya still left 509 uncited, so more words were not the answer and would have risked the seven countries that comply. Instead stages.adopt_orphans() asks again about the specific rows that went missing - a far smaller question than the one that produced them - showing the model the orphaned interventions and the inventory it already built, and taking -1 for an orphan no strategy covers. It runs inline at the end of stage 4 for future runs, and 02_Automation/repair_source_chunks.py applies it to outputs that already exist, so no country has to re-run stage 4 and re-decide every name, risk and orientation to fix a citation.
+THE PASS ONLY APPENDS TO source_chunks. Kenya: 281 strategies before and after, names identical, and no field other than source_chunks changed; the rebuilt FINAL_PANEL is identical in content across all 14 sheets. 506 of 509 placed for $0.07, 3 refused and left uncited, taking A22 from 36.9% to 0.2%.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
@@ -3125,7 +3129,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>lineage.py: kenya stage 3 -&gt; stage 4 (consolidation) 1378 -&gt; 869, lost 509 (36.9%); brazil 1.6%, brunei 3.1%, fiji 2.2%, jamaica 0.4%, malaysia 0.9%, maldives 0.8%, thailand 1.5%</t>
+          <t>kenya A22: 509 uncited (36.9%) -&gt; 3 uncited (0.2%). Placements judged on substance rather than wording: 'Laboratory for Sample Analysis' -&gt; 'Anti-doping education, testing and enforcement', 'National Sports Fund' -&gt; 'Strategic funds and technical institutions'. Panel content unchanged, 14/14 sheets identical.</t>
         </is>
       </c>
     </row>
@@ -3178,6 +3182,162 @@
       <c r="J52" s="2" t="inlineStr">
         <is>
           <t>Before: maldives stage 5 -&gt; budget layer 85 -&gt; 56, lost 29 (34.1%). After a re-extraction: 454 -&gt; 454, lost 0 (0.0%), and the country passes every conservation hop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>W52</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>publishing</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Publishing is DELETE-then-INSERT and not a transaction, so anything reading during a publish silently loses a country</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>publish_run.push deletes a run's rows table by table and then inserts them, with no transaction around it. A reader landing in that window sees a published run with zero strategies. build_union_panel treated that as 'nothing to show' and skipped the country without a word, so the same command run twice a minute apart produced a six-country panel missing Kenya and then a six-country panel missing Thailand, from identical data. Nothing failed, no count was wrong on the page, and the only symptom was a country quietly absent - which is indistinguishable from a country that was never published.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Partly fixed 2026-08-22: build_union_panel now prints a WARNING naming the country and its run id instead of skipping in silence, so the failure is visible and the answer is to rebuild. The underlying non-atomic publish is unchanged; a real fix is to insert the new rows under a new run_id and delete the old one afterwards, so no window exists where a country has a run and no rows.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Three consecutive build_union_panel.collect() calls during a concurrent publish returned 6, 6 and then 8 countries, with a different country missing each time; a fourth after the publish finished returned 8 stably.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>W53</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Prompt 7 consolidates within a BATCH, not within a document, so a large document returned the same intervention more than once</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>The design says consolidation runs within one sector document and the country answer is a union across documents. The implementation showed the model one batch at a time, because the whole NDP strategy list rides along in every call and bounds how much of the document can go with it. A document that fits one batch is therefore consolidated as designed and a larger one is not. Malaysia's Education 2026-2035 needed ten batches and returned twelve interventions twice, each inflating the 'not in the NDP' count that the dashboard reports. Brunei showed none, because every one of its eight documents fitted a single batch - so the defect was invisible on the first country and would have stayed invisible on any country with small documents.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. run_stage7_responses merges records with the same normalised name within a document after all batches return: source_refs, related_risks and sdg_targets are unioned, and in_ndp='yes' wins, because a batch that matched the intervention to a plan strategy is evidence the plan carries it and the safe direction is to under-report novelty. Deterministic, no extra model call. verify_sector_layer.py now asserts no intervention appears twice in one document.</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Before: malaysia 1230 rows with 12 within-document duplicates, all in Education 2026-2035. After: 1268 rows, 0 duplicates; brunei 414 rows, 0 duplicates both before and after.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>W54</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>publishing</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>db.select silently truncates at 1000 rows, and passing a larger limit does not lift it</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>PostgREST applies its own max-rows cap server-side and returns a short answer with HTTP 200. A caller that reads a table and counts what came back gets a wrong number with nothing to indicate it: Malaysia's 1,268 published sector responses read back as exactly 1000, and the only reason it was noticed is that a verification check compared the count against the workbook. Every reader in this repo that does not paginate is exposed. build_union_panel already had fetch_all; build_sector_gap did not, and v_sector_new_responses stood at 756 rows for two countries - a third would have crossed the cap and quietly lost rows from the workbook and the dashboard alike.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. db.Supabase.select_all() pages past the cap, and select()'s docstring now states the cap rather than leaving it to be discovered. select_all RAISES when it needs a second page and the caller gave no 'order', because offset without a stable sort reads a row twice or not at all, and the right column is the caller's to choose. build_sector_gap and verify_sector_layer use it.</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>select('sector_responses', limit=20000) returned 1000; fetch_all returned 1268 with distinct row_no 1..1268.</t>
         </is>
       </c>
     </row>
@@ -3324,7 +3484,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22 11:57 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-22 21:35 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>

</xml_diff>

<commit_message>
Five countries reach the page: Afghanistan, Bhutan, Kiribati, Samoa, China
Afghanistan, Bhutan and Kiribati had finished panels on disk and no run in the
database, so the dashboard could not show them. Samoa and China completed
overnight. Publishing all five takes the page from 9 countries to 14, rebuilt
from Supabase so the union cannot drift from what was published.

India and Nauru carry a run report and no panel, which is the honest state:
both hold budget documents with no programme detail to map.
</commit_message>
<xml_diff>
--- a/DATA_ISSUES.xlsx
+++ b/DATA_ISSUES.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="register" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="detected" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="by_country" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="about" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="closed" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="detected" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="by_country" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="about" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:K71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -472,7 +473,8 @@
     <col width="52" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -508,7 +510,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>WHAT WOULD FIX IT</t>
+          <t>THE FIX (done, where STATUS says so)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -518,10 +520,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>SETTLED ON</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>FIRST SEEN</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>EVIDENCE</t>
         </is>
@@ -571,10 +578,15 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>D1 in the detected sheet; FY2024 codes 0032, 0901, 0902, 0903, 0909, 0910, 1144, 1149</t>
         </is>
@@ -623,10 +635,15 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>run_report unmatched_codes 824 -&gt; 0 and 254 -&gt; 0; budget_all_years head totals against programme sums per year</t>
         </is>
@@ -673,12 +690,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>D12 in the detected sheet; D8 for Brunei's unreconciled years</t>
         </is>
@@ -712,25 +730,30 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Kiribati cost $6.21 and produced no budget lines at all, in two different ways. First against the Recurrent Budget, which is the densest table in the whole set at 16.8 rows a page and whose rows are objects of expenditure: 219 Local catering, 227 External travel, 230 Cleaning. Nothing in it maps to a plan strategy. Then against the Development Budget, which IS the right document, is organised by KV20 pillar, carries project codes and titles, and parsed cleanly into 64 tables. It still returned nothing, because Table 7A has ten numeric columns of which six are years: Total Project Cost, Accumulated Balance, 2024 Budget, 2024 Revised, 2024 Warrant, 2024 Estimated Balance, 2025 Budget, 2026 Estimate. Prompt 5 assumes one amount column and a strategy total to reconcile against, and the ministry rows carry no totals. The first project has 4,427 under 2024 Warrant and nothing under 2025 Budget. The model returning an empty array is the correct answer to a question that was not asked properly.</t>
+          <t>Kiribati cost $6.21 and produced no budget lines at all, in two different ways. First against the Recurrent Budget, which is the densest table in the whole set at 16.8 rows a page and whose rows are objects of expenditure: 219 Local catering, 227 External travel, 230 Cleaning. Nothing in it maps to a plan strategy. Then against the Development Budget, which IS the right document, is organised by KV20 pillar, carries project codes and titles, and parsed cleanly into 64 tables. It still returned nothing, because Table 7A has ten numeric columns of which six are years: Total Project Cost, Accumulated Balance, 2024 Budget, 2024 Revised, 2024 Warrant, 2024 Estimated Balance, 2025 Budget, 2026 Estimate. Prompt 5 assumes one amount column and a strategy total to reconcile against, and the ministry rows carry no totals. The first project has 4,427 under 2024 Warrant and nothing under 2025 Budget. The model returning an empty array is the correct answer to a question that was not asked properly. RESOLVED 2026-08-25, and the donor-keyed-table diagnosis previously in this entry was wrong, as the equivalent claim about Bhutan was. Re-running stage 5 with the current prompt produced 300 programme rows from the same four documents, where the 14 August run produced 0: 2023 23 rows, 2024 205, 2025 42, 2026 30, for $1.43. The documents were never the problem. Kiribati ran on 2026-08-14 and Prompt 5 was rewritten on 2026-08-22, so its budget layer was the output of a prompt that no longer exists.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>See F8 in FIXES.xlsx. Two failure modes, two detectors, both now in document_shape.py: a LINE ITEMS verdict for a table whose rows are objects of expenditure, and a year-column count that says a fiscal-year column has to be named in the config before Prompt 5 sees the table.</t>
+          <t>Fixed 2026-08-25 by re-running stage 5 with --force at a cost of $1.43, against the $2.33 the 14 August attempt spent producing nothing. Bhutan was the same fault and the same fix. Both countries then had a full re-run on current prompts, because stages 3 and 4 also predated the 19 August prompt rewrites.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>D12 and the shape probe; Files/llm/kiribati/kiribati_budget_*.xlsx, 0 rows each</t>
         </is>
@@ -779,10 +802,15 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>stage5_probe on FY2026: 731 lines, 25 reconciliation problems, 100 rows dropped by the code pattern</t>
         </is>
@@ -816,25 +844,30 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>A stage 5 probe on one document per country, $4.10 in total, settled what three rounds of text heuristics could not. Kenya yields 631 programmes from 1,149 pages and Jamaica 208 from 706, both clean vote-to-programme hierarchies. Ghana yields zero: its FY2024 budget statement is a narrative policy document and the appropriations sit in an appendix file we hold for FY2015 only. Bhutan yields zero: its Budget Report is a fiscal analysis whose largest table is state-owned enterprise accounts, revenue, expenses and profit before tax, with no appropriations anywhere in it. Malaysia yields 71 programmes from 584 pages, correctly formed but far too few for a document of that size, so it is under-extracting rather than failing. Kiribati is W8. The pattern is that a country fails on its DOCUMENTS long before it fails on its prompts, and no amount of reading the text locally establishes which.</t>
+          <t>A stage 5 probe on one document per country, $4.10 in total, settled what three rounds of text heuristics could not. Kenya yields 631 programmes from 1,149 pages and Jamaica 208 from 706, both clean vote-to-programme hierarchies. Ghana yields zero: its FY2024 budget statement is a narrative policy document and the appropriations sit in an appendix file we hold for FY2015 only. Bhutan yields zero: its Budget Report is a fiscal analysis whose largest table is state-owned enterprise accounts, revenue, expenses and profit before tax, with no appropriations anywhere in it. Malaysia yields 71 programmes from 584 pages, correctly formed but far too few for a document of that size, so it is under-extracting rather than failing. Kiribati is W8. The pattern is that a country fails on its DOCUMENTS long before it fails on its prompts, and no amount of reading the text locally establishes which. RESOLVED for Bhutan 2026-08-25, and the earlier diagnosis in this entry was wrong. It said the four BHT Budget Reports were macro-fiscal narrative carrying no programme table, on the strength of word counts over the PDF's flattened text layer. Re-running stage 5 with the current prompt produced 390 programme rows from the same four documents, where the 14 August run produced 0: 2024 64 rows, 2025 103, 2026 31, 2027 192, for $1.04. The documents were never the problem. What was wrong is that Bhutan ran on 2026-08-14 and Prompt 5 was rewritten on 2026-08-22, so its budget layer was the output of a prompt that no longer exists, which is W7's pattern and was never checked for this country.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>See F9. Probe one document before committing a country: 02_Automation/stage5_probe.py, $0.15 to $2.64 a document against $8 to $48 a country. Ghana and Bhutan need their appropriation documents sourced; Malaysia needs its under-extraction diagnosed before it is worth $48.</t>
+          <t>Fixed for Bhutan 2026-08-25 by re-running stage 5 with --force at a cost of $1.04. Kiribati is the same shape and the same fix. The general lesson is W7's: any country whose outputs predate a prompt rewrite should be re-run before being called blocked, and the run date against the prompt mtime is enough to spot it. Ghana and Rwanda are still blocked on documents, not on this.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Files/llm/_probe/*.xlsx; Kenya 631 programmes, Jamaica 208, Malaysia 71, Ghana 0, Bhutan 0, Kiribati 0</t>
         </is>
@@ -883,10 +916,15 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
         </is>
@@ -935,10 +973,15 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
         </is>
@@ -987,10 +1030,15 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
         </is>
@@ -1037,12 +1085,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>D10 in the detected sheet</t>
         </is>
@@ -1089,12 +1138,13 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>D9 in the detected sheet; the 'twice' filter in the audit view</t>
         </is>
@@ -1143,10 +1193,15 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>02_Automation/cache/di_&lt;hash&gt;.json for the FY2017 budget: 0 Thaana, 159,753 Arabic; pypdf on the same file: 342,715 Thaana</t>
         </is>
@@ -1195,10 +1250,15 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>FINAL_PANEL.xlsx ceiling sheet, status EXCEEDS TOTAL; audit_checks A4</t>
         </is>
@@ -1247,10 +1307,15 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Files/llm/&lt;slug&gt;/&lt;slug&gt;_strategyclean.xlsx; the ambiguous-join drops logged by stage 6b</t>
         </is>
@@ -1297,12 +1362,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>stages.py:611; schemas.py:243-244; Files/llm/malaysia/malaysia_budget_*.xlsx vs mappings/</t>
         </is>
@@ -1350,12 +1416,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>01_Pipeline/scripts/extract_budget_tables.py; 02_Automation/inputs/jamaica.json budget_tables</t>
         </is>
@@ -1404,10 +1471,15 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>01_Pipeline/prompts/6_mapping.txt L50-55</t>
         </is>
@@ -1441,7 +1513,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Mapping recall is estimated per country. Of the edges the panel does contain, the share that are real is unknown, and nothing in the pipeline has ever been labelled by a person. Files/outputs/precision_sample.csv holds a stratified sample drawn for exactly this and every verdict cell is empty. Without it, any threshold on match quality would be set in units nobody has measured.</t>
+          <t>Mapping recall is estimated per country. Of the edges the panel does contain, the share that are real is unknown, and nothing in the pipeline has ever been labelled by a person. Files/outputs/precision_sample.csv holds a stratified sample drawn for exactly this and every verdict cell is empty. Without it, any threshold on match quality would be set in units nobody has measured. Labelled 2026-08-25: 141 of 142 marked, giving 93% precision and 100% money-weighted on the 114 edges that join the runs the sample was drawn from. Kenya and Thailand 100%, Brunei 93%, Fiji 90%, Brazil 81%; every error falls on a small line. That is a measurement of the 16 August model. Only 1 of the 141 joins the CURRENT panel, because the re-extraction of 19-20 August renamed every strategy, so precision as of today is still unmeasured and the remaining decision is whether to re-draw the sample or map the old names onto the new.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1454,12 +1526,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Files/outputs/precision_sample.csv; 01_Pipeline/scripts/precision_labels.py</t>
         </is>
@@ -1508,10 +1581,15 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>01_Pipeline/prompts/6b_programme_coverage.txt L48-51</t>
         </is>
@@ -1558,12 +1636,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>01_Pipeline/scripts/precision_recall.py L28-33</t>
         </is>
@@ -1612,10 +1691,15 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>02_Automation/inputs/*.json; 01_Pipeline/countries/*.json</t>
         </is>
@@ -1664,10 +1748,15 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>05_Handoff/scripts/check_handoff_drift.py</t>
         </is>
@@ -1714,12 +1803,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>03_Ingest_and_Publishing/scripts/publish_run.py as_list</t>
         </is>
@@ -1766,12 +1856,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>01_Pipeline/scripts/run_pipeline.py run_stage</t>
         </is>
@@ -1818,12 +1909,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>03_Ingest_and_Publishing/supabase/migrations/0001_init.sql L179</t>
         </is>
@@ -1870,12 +1962,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>scan_scoreboard share_dev_mapped vs share_mapped, all 8 countries</t>
         </is>
@@ -1922,12 +2015,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>panel.bau_funded x panel.response_orientation, 4 countries</t>
         </is>
@@ -1974,12 +2068,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>audit_checks A19; pct_ranks([5,5,5,5,5])</t>
         </is>
@@ -2028,10 +2123,15 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>budget_all_years strategy_total rows, Malaysia, 37 pairs</t>
         </is>
@@ -2078,12 +2178,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>scan_scoreboard risks_per_strategy, risk_top_share, share_risk_evidenced</t>
         </is>
@@ -2132,10 +2233,15 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
           <t>2026-08-19</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>publish_run.table_columns against the live schema</t>
         </is>
@@ -2184,10 +2290,15 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>budget_all_years, Maldives; 395 of 852 programme names fail the readability test</t>
         </is>
@@ -2241,6 +2352,11 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
           <t>sum(strategy_total) vs sum(program) per country, all 8</t>
         </is>
       </c>
@@ -2286,12 +2402,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>audit_checks A4, all countries</t>
         </is>
@@ -2340,10 +2457,15 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>8 duplicated keys in Brazil funding_by_program, 5,511.0 BRL million</t>
         </is>
@@ -2392,10 +2514,15 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>funding_by_program amount == 0</t>
         </is>
@@ -2442,12 +2569,13 @@
           <t>FIXED</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Malaysia 1,847.9bn all rows vs 1,692.0bn countable</t>
         </is>
@@ -2494,12 +2622,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>national_total: FY2017 7,988,962,654 and FY2019 7,076,705,474; FY2018 empty</t>
         </is>
@@ -2538,20 +2667,25 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Apply 0003 and 0005 in the SQL editor. Longer term the publish step should assert the migration level it expects rather than adapting to whatever it finds, so an unapplied migration is a red run rather than a warning.</t>
+          <t>Apply 0003 and 0005 in the SQL editor. Longer term the publish step should assert the migration level it expects rather than adapting to whatever it finds, so an unapplied migration is a red run rather than a warning. Verified fixed 2026-08-24: verify_schema.py reports all 45 declared objects present across the first ten migration files, so both migrations are applied. The register had gone stale, not the database.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>FIXED</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>select source_documents?select=doc_type -&gt; 400 'column source_documents.doc_type does not exist'; select access_log -&gt; 404 'Could not find the table public.access_log'</t>
         </is>
@@ -2605,6 +2739,11 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
           <t>type_from_name('Digital Economy Masterplan 2025.pdf') returned 'ndp' before the change; both files now type as 'sector'</t>
         </is>
       </c>
@@ -2657,6 +2796,11 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
           <t>HttpResponseError (Timeout) raised from _analyze during --dry-run; PAGES_PARSED['parsed'] was 86 at the time</t>
         </is>
       </c>
@@ -2709,6 +2853,11 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
           <t>39,843,726 bytes over 22 pages; sliced at 5 pages it parsed to 759 paragraphs across all 22 pages</t>
         </is>
       </c>
@@ -2761,6 +2910,11 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
+        <is>
           <t>source_documents held 7 brunei rows and 0 malaysia rows; the bucket held 15 brunei objects including 8 under 'sector strategies/'</t>
         </is>
       </c>
@@ -2806,12 +2960,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Brunei NDP risk grid 2,970 chunks over three plans; Economic Blueprint 2035 alone 493 chunks</t>
         </is>
@@ -2865,6 +3020,11 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
           <t>Brunei stage 5 output: {'grand_total': 3, 'strategy_total': 3, 'program': 41}; tamper_test --country brunei -&gt; FALSE POSITIVE schema; live budget_lines holds only strategy_total and program</t>
         </is>
       </c>
@@ -2918,6 +3078,11 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
           <t>brunei carried 97 / broader_only 240 / silent 76; malaysia carried 414 / broader_only 573 / silent 126. Measured against a golden baseline taken before the prompt change: on the 251 interventions present in both Brunei runs, related_risks held at 94% and HDICategory at 99%.</t>
         </is>
       </c>
@@ -2970,6 +3135,11 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
           <t>openpyxl.utils.exceptions.IllegalCharacterError raised from writer.write_results via stages.run_stage7_risk; run died at $5.05, re-run replayed from cache at $0.00</t>
         </is>
       </c>
@@ -3015,12 +3185,13 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="J49" s="2" t="inlineStr">
+      <c r="K49" s="2" t="inlineStr">
         <is>
           <t>Before re-run: grand_total None for 2021, 2022, 2025, 2026. After: 5860 / 5860 / 6250 / 6350, basis 'grand_total', extracted_pct 96 / 102.9 / 38.4 / 16.</t>
         </is>
@@ -3073,6 +3244,11 @@
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
         <is>
           <t>Before: KENYA section showed '1451 -&gt; 1438 lost 13 (0.9%)' (Malaysia's row) against a summary of 'kenya ... 509 of 1378'. After: KENYA shows '1378 -&gt; 869 lost 509 (36.9%)', matching the summary exactly.</t>
         </is>
@@ -3129,6 +3305,11 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
           <t>kenya A22: 509 uncited (36.9%) -&gt; 3 uncited (0.2%). Placements judged on substance rather than wording: 'Laboratory for Sample Analysis' -&gt; 'Anti-doping education, testing and enforcement', 'National Sports Fund' -&gt; 'Strategic funds and technical institutions'. Panel content unchanged, 14/14 sheets identical.</t>
         </is>
       </c>
@@ -3174,12 +3355,13 @@
           <t>CLOSED</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="K52" s="2" t="inlineStr">
         <is>
           <t>Before: maldives stage 5 -&gt; budget layer 85 -&gt; 56, lost 29 (34.1%). After a re-extraction: 454 -&gt; 454, lost 0 (0.0%), and the country passes every conservation hop.</t>
         </is>
@@ -3226,12 +3408,13 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="J53" s="2" t="inlineStr">
+      <c r="K53" s="2" t="inlineStr">
         <is>
           <t>Three consecutive build_union_panel.collect() calls during a concurrent publish returned 6, 6 and then 8 countries, with a different country missing each time; a fourth after the publish finished returned 8 stably.</t>
         </is>
@@ -3285,6 +3468,11 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
           <t>Before: malaysia 1230 rows with 12 within-document duplicates, all in Education 2026-2035. After: 1268 rows, 0 duplicates; brunei 414 rows, 0 duplicates both before and after.</t>
         </is>
       </c>
@@ -3337,7 +3525,864 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
           <t>select('sector_responses', limit=20000) returned 1000; fetch_all returned 1268 with distinct row_no 1..1268.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>W55</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>cambodia, indonesia</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Two of the seven new countries hold no budget documents at all</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Cambodia's bucket folder holds six national plans and nothing else. Indonesia's holds three plans and a Budget/ folder containing only an empty-folder placeholder. Both are registered and typed correctly, and neither can produce a budget layer, a mapping or a panel, because there is no money to map to. Bangladesh, China and Sri Lanka are a weaker version of the same problem: they hold budget SPEECHES, which carry narrative and headline totals but no programme lines, so a budget layer built from them would have nothing for Prompt 6 to match against. Only Kiribati, of the seven, holds real estimates books.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Confirm NDP-only as the intended scope for Cambodia and Indonesia, or name the budget documents to obtain. Their country configs carry budget_year_files: [] and a _budget note, so nothing will attempt a budget stage against them in the meantime. Ghana and Rwanda are the existing precedent for a country registered and held at this state.</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>pv2-sources: Cambodia/ 6 objects, all under NDPs/. Indonesia/Budget/ holds only .emptyFolderPlaceholder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>W56</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>prompt</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>brunei, malaysia</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Prompt 7 returns SDG goal names in the HDICategory field on 38 sector interventions</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>HDICategory has a closed 15-value vocabulary. 38 rows carry something else, and most of what they carry are SDG goal titles: 'Quality Education' (10), 'Industry, Innovation and Infrastructure' (7), 'Peace, Justice and Strong Institutions' (2), 'Gender Equality' (1). The rest are invented labels of the same shape: 'Industry and Infrastructure' (13), 'Education and Skills' (2), 'Digital Economy' (2), 'Inclusive Growth' (1). The field is an axis of the analysis, so a row carrying an SDG goal in it is not merely untidy: it is absent from whichever HDI category it belonged in, and it invents a category that appears nowhere else in the model. The prompt asks for both an HDICategory and sdg_targets in the same object, which is the likely cause.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>The L2 gate now has a sector-responses contract and catches this; before 2026-08-24 no schema contract existed for any sector stage, so the field was never checked. Correcting the data needs a re-run of stage 7 for both countries, which costs money and is therefore on the human list. Tightening Prompt 7 to name the fifteen values inline, as Prompt 3 does, should come first.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>validate_stage_schema.py on brunei_sector_responses.xlsx: 4 blocking; malaysia_sector_responses.xlsx: 34 blocking. All HDICategory, all 'value outside the fixed vocabulary'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>W57</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>bhutan, fiji, ghana, maldives, rwanda</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Five countries have every source document typed 'other', so they read as holding nothing</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>document_types() reads the type from a mirror subfolder or a sidecar, and these five were fetched by a route that left neither. Bhutan holds 10 documents, Ghana 10, Rwanda 8, Fiji 7, Maldives 4, and all 39 are 'other'. The effect is not cosmetic: the ingest overview on the Audit tab counts plans and budgets by doc_type, so these countries showed zero of both while holding a full set, and Fiji reads as having built an eight-year panel out of no documents at all. Ghana and Rwanda both have a hand-written sources.json with an explicit 'kind' on every entry, which document_types() would read if it were pointed at it.</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Re-publish the five with --from-mirror once their sources.json is in place, or add the five to DOC_TYPE_OVERRIDES. Neither costs anything: the bytes are already in the bucket and only the doc_type column changes. Until then the Untyped column on the Audit tab shows the size of the problem per country.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>v_source_documents: bhutan other:10, ghana other:10, rwanda other:8, fiji other:7, maldives other:4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>W58</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>publishing</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>The union dashboard is a 20.6 MB single page and takes over 6 seconds to open</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>20.5 MB of the 20.6 is embedded JSON: rows 12.3 MB, meta 7.8 MB, and 7.5 MB of that is evidence quotations and source chunks carried inside the strategy rows. This is the main live link, the thing a reader is sent. It is unopenable on a phone or a hotel connection, and the evidence text that makes up over a third of the weight is only ever read for the handful of rows somebody clicks into. Measured 2026-08-25: 6.3s to first render headless on a fast machine with the file local.</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Move the evidence payload out of the page and fetch it per row, or ship it as a sibling JSON the page loads on demand. The Audit tab is the only consumer. Nothing about the figures changes.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>union_dashboard.html 20.6 MB; const D 20.5 MB; ev inside rows 7.5 MB across 1588 rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>W59</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>precision-recall</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>precision_labels.py reported 100% precision from one edge after silently discarding 140</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>It joins hand-marked labels to the LATEST panel run only. The sample was drawn on 2026-08-16 and the re-extraction of 19-20 August renamed every strategy, so 140 of 141 marked edges no longer matched anything and were dropped with a one-line note, after which it printed a confident round 'precision 100%' computed from the single survivor. A gate that cannot find its inputs must refuse to report, not report on what is left: every other validator in the suite dies rather than pass when it checked nothing, and this one does not.</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Join against the run the sample was drawn from, recorded in the sample when it is drawn, rather than against the latest. Until then, die when the joined share falls below a threshold, the way validate_recall and validate_refs already do. Scored against the 16 August runs the same labels give 93% precision on 114 joined edges, so the labels themselves are sound.</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>141 marked, 140 excluded, 'OVERALL 1 labelled y/n, precision 100%'. Rejoined to the 2026-08-16 runs: 114 joined, 97 y, 7 n, 10 unsure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>W60</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>brunei, fiji, thailand, maldives</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Share of budget mapped is not comparable across countries, because the extraction covers different fractions of each budget</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>The denominator is right (the national total line) but the NUMERATOR rests on an extraction that covers a different share of the budget in each country. Measured 2026-08-25: Brunei's countable programme rows are 42% of its own national total, Fiji's 58%, and Maldives publishes programme rows summing to 113% of the total they sit inside. Brazil, Jamaica, Kenya, Malaysia and Thailand extract essentially the whole budget. A share built on 42% of a budget and a share built on 100% of one are not the same statistic, and the page puts them in one column with nothing to say so. Maldives also publishes its national total twice, under line_type 'national' (168,861,925,470) and 'grand_total' (161,661,505,210), which disagree by 4%: which one a consumer picks moves every share for that country.</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Show extraction coverage beside the share so a partial extraction reads as partial. Done 2026-08-25 in UNION_PANEL.xlsx country_summary, which now carries EXTRACTED, BUDGET EXTRACTED and a COMPARABLE column stating in words when a row must not be read beside another. coverage_basis.py is registered as an L3 gate and fails the suite while any country is below 95%. The underlying fix is to extract the rest of Brunei's and Fiji's budgets, which costs money and is on the human list. Maldives' duplicate national line needs combine_budget_years to publish one, not two.</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>countable programmes / national line: brunei 41.5%, fiji 58.0%, maldives 112.6%, brazil 100.0%, jamaica 100%, kenya 100.3%, malaysia 100%, thailand 100%. Corrected from an earlier reading of this issue that summed 'national' and 'grand_total' together and so halved every coverage figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>W61</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>panel_budget.budget double counts: summing it across strategies exceeds the whole budget</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>One programme matched to several strategies contributes its full amount to each, so the per-strategy funding column is not additive. Every published country is affected. Measured 2026-08-25 by summing the column the way a reader would, against country_summary.MAPPED: Fiji 5.40x, Malaysia 4.15x, Thailand 3.94x, Jamaica 2.76x, Kenya 2.39x, Brunei 2.21x, Maldives 2.15x, Brazil 1.58x. The read_me sheet has warned about this in words for weeks without ever giving the magnitude, and it is a sheet a reader building a pivot table never opens. The dashboard headline is safe because it deduplicates; the workbook column beside it is what gets summed.</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Done 2026-08-25. The per-year sheet header now reads FUNDING (DO NOT SUM), country_summary carries a SUMMING FUNDING OVERSTATES BY column with the measured multiple per country, and the read_me states the magnitudes rather than only the principle. The multiple is computed from the rows the workbook actually writes, and verified against an independent sum of the written column: the two agree to the last decimal for all eight countries.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>sum(FUNDING column)/country_summary.MAPPED: fiji 5.40, malaysia 4.15, thailand 3.94, jamaica 2.76, kenya 2.39, brunei 2.21, maldives 2.15, brazil 1.58. Independent re-sum of the written workbook agrees exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>W62</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>The coverage basis gate takes 212 seconds, three times the rest of the suite together</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>It pages every row of budget_lines and matches for all nine published countries on each run, which is roughly 12,000 rows over PostgREST at 1,000 a page. The suite was around 90 seconds before it and is now over 300, and a suite people stop running because it is slow protects nothing.</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Aggregate server-side in a view rather than paging the rows into Python, the way v_risk_panel already does for the risk side. The numbers do not change; only where the sum happens.</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>run_tests: 'coverage basis' 212888ms against 'sector layer' 9379ms and the whole of L1-L6 offline in under 40s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>W63</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>afghanistan</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>The cost estimate reads .docx as an empty document and reports the country as free to run</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>parse.read_text_layer returns None for anything that is not a PDF, and the dry-run branch of parse_document falls back to {'paragraphs': []} when it does. So a .docx estimates as zero paragraphs, zero chunks and $0.00. Afghanistan's most recent national plan, AFG NDS 2025-2030.docx, is the only .docx in the corpus and holds 131,468 characters of readable text; the dry run reported '0p, 0 paragraphs', 'stage 1 -&gt; afghanistan_risk_rows.xlsx (0 rows, 0 errors)' and an estimate of $0.0000. Zero cost with zero errors reads as a country that needs nothing doing. What a REAL run would have done was not tested and is not asserted here: Document Intelligence may well have parsed the file, in which case the defect is confined to the estimate, and an estimate that says free about a document that will be billed is the thing the dry-run code comments were written to prevent.</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-25. parse.read_docx reads a .docx directly from its own XML, before any Document Intelligence path and on both the dry-run and the real branch, so the format now costs nothing at all rather than costing nothing only in the estimate. Afghanistan goes from 0 paragraphs to 537. Separately, run_llm_pipeline now stops the run when any source document parses to zero paragraphs, with a message naming the supported formats, so an unreadable document can no longer produce an empty successful run in either mode.</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>Before: 'NDP AFG NDS 2025 2030: 0p, 0 paragraphs', estimate $0.0000. After: 537 paragraphs, 537 chunks. read_docx on the same file returns 735 raw paragraphs and 132,063 characters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>W64</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>bhutan, kiribati</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Two countries have finished plan-side extraction and no panel, and nobody noticed</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Bhutan holds bhutan_risk_rows.xlsx (1068 rows) and bhutan_strategy_rows.xlsx (644 rows); Kiribati holds 1922 and 681. Both re-estimate at $0.00 because there is nothing left to extract on the plan side. Yet neither has a published panel, so both read as NOT READY on the hub and as amber on the ingest overview, indistinguishable from countries where no work has been done at all. The money already spent on them is sitting unused, and W8 and W9 describe them as blocked when the plan side is in fact complete.</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Run the remaining stages and publish. Cost is the budget side only, not a re-extraction. Until then the ingest overview should distinguish 'nothing done' from 'extracted, not assembled', which it currently cannot.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>dry run --stages 1: both report 'reusing ..._risk_rows.xlsx' and 'reusing ..._strategy_rows.xlsx', estimate $0.0000. Neither appears in v_latest_run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>W65</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>bhutan, kiribati</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>A dry run reports $0.00 and reuses a budget layer that has zero rows in it</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Both countries hold four budget workbooks each and every one has 0 rows. The dry run prints 'stage 5: reusing 4 budget file(s)' and estimates $0.00, which reads as a country that is finished and costs nothing. The real run has a STOPPING guard for exactly this ('stage 5 produced no budget lines'), but it is written 'if "5" in want and not all_budget_rows and not args.dry_run', so the estimate is the one path that does not check. The result is that the cheapest-looking country in the portfolio is one that cannot produce a panel at all, which is how both of these were recommended as easy wins earlier the same day.</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Drop the 'not args.dry_run' condition and report the empty layer in the estimate as well. A dry run exists to tell you what a real run would do, and this is the one thing it does not tell you.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>bhutan_budget_2024/25/26/27.xlsx and kiribati_budget_2023/24/25/26.xlsx: 0 data rows each, header only. Dry run: 'reusing 4 budget file(s)', Estimated total $0.0000. mappings/ empty for both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>W66</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>sources</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>There is no cheap way to tell whether a budget document will extract, and two attempts to build one both failed</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Three countries have now spent a whole budget extraction on documents that could not produce a programme line (Bhutan, and Kiribati and Brunei's earlier years), so a pre-flight that costs nothing is worth real money. Two heuristics over the PDF's own text layer were built on 2026-08-25 and both were wrong. The first, a regex for code-name-amount, scored Ghana's budget SPEECH at 561 programme rows: it was matching numbered paragraphs ('12. Mr. Speaker, ... 2020') and years in prose ('30.0 per cent by 2022'), and it nearly bought a $40.70 run on two documents that carry no appropriations. The second, requiring a repeated code SHAPE plus appropriation vocabulary, flagged 59 of 64 documents including Kenya's programme-based budget, which extracted 887 rows. Calibrated against every document whose outcome is known, neither separates: Brunei extracted 61 rows from a document with zero appropriation words, Bhutan extracted zero from one with 67. The cause is structural. The text layer is linear and breaks tables into a character stream; the pipeline sends the PDF to Document Intelligence, which does layout recognition. What DI can reconstruct is not visible to anything reading the text layer, so no regex over it can predict the outcome. Settled 2026-08-25 by running the eight countries the heuristics had written off. Seven of eight produced rows. Afghanistan's Budget Report, called a macro-fiscal narrative with no programme table, gave 541. Samoa's budget ADDRESSES, called speeches carrying no programme lines, gave 277 across three years. Nauru's 8,941-character appropriation bill gave 51. The conclusion stands and is now measured on eleven documents rather than argued: nothing readable from a text layer predicts what Document Intelligence will extract, and the only reliable test is to run one year and look.</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed 2026-08-25. document_shape.py stays unregistered as a gate. The working practice is to run the cheapest slice: stage 5 for one year costs between $0.03 and $0.50 a country, and eight countries cost $1.72 to settle definitively.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>probe verdict vs rows actually extracted: brunei NO TABLE/61, kenya NO TABLE/887, fiji SPEECH/269, jamaica GO/169, bhutan NO TABLE/0, kiribati NO TABLE/0. Appropriation-word counts: brunei 0 with 61 rows, bhutan 67 with 0 rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>W67</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>ghana, india, nauru, papua_new_guinea, rwanda, samoa, tuvalu</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Seven configured countries have never been run, and nothing records why</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Each has a country config, an automation config, a plan document and budget documents on disk. Ghana, Papua New Guinea and Rwanda have cost ledgers containing dry runs and nothing else; India, Nauru, Samoa and Tuvalu have no ledger at all, so no run was ever started. There is no blocker recorded against any of them in this register, no failed run to point at and no note saying they were deferred. They are simply untouched, and because the hub shows them as NOT READY they look identical to countries that were tried and failed. Two countries were called blocked all week (W8, W9) when what they needed was a re-run, and these seven have the opposite problem: nothing has been attempted at all. Eight of them were run on 2026-08-25 and seven produced budget rows, for $1.72 in total: Afghanistan 541, Samoa 277, Rwanda 88, Nauru 51, Sri Lanka 51, China 26, India 15, Tuvalu 0. Every one had been written off in this register or in conversation on the strength of a prediction about its documents, and every prediction was wrong except Tuvalu's.</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Eight run 2026-08-25 for $1.72 producing 1,049 budget rows. They now need stages 4 and 6 and a panel. Ghana and Papua New Guinea are still unrun: PNG's config points at Volume 1 and its own note says the appropriations are in Volumes 2 and 3, which are not held, so that one is a documents gap rather than an assumption.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>cost_ledger.jsonl: ghana 4 entries all dry_run, rwanda 4 all dry_run, papua_new_guinea 1 dry_run; india, nauru, samoa, tuvalu no ledger. All seven have ndp_documents and budget_documents that exist on disk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>W68</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>pipeline</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Nothing compares a country's outputs against the date its prompts were rewritten</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Bhutan and Kiribati sat in this register for eleven days as 'document parses, extraction returns nothing', which reads as a source-material fault. Both had simply been run on 2026-08-14 with a Prompt 5 that was rewritten on 2026-08-22. Re-running produced 390 and 300 budget rows against 0. Two wrong diagnoses were written into W8 and W9 in the meantime, both inferring the documents were unusable. W7 records the same class of fault for Brazil and Brunei and was never generalised. The signal is free and already on disk: a stage output's mtime against the mtime of the prompt that produced it. D12 in data_issues.py detects an output predating its prompt for the countries it scans, and neither of these was among them.</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Extend D12, or add a check beside it, that compares every country's stage outputs against 01_Pipeline/prompts/*.txt mtimes and reports any country whose outputs predate the prompt that made them. It needs no API calls and no database. A country in that state must not be described as blocked until it has been re-run.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>bhutan ran 2026-08-14T11:40, kiribati 2026-08-14T11:10; 5_budget_extraction.txt mtime 2026-08-22, 3_strategy_extraction.txt and 4_strategy_clean.txt 2026-08-19. Re-run stage 5: bhutan 0 -&gt; 390 rows for $1.04, kiribati 0 -&gt; 300 rows for $1.43.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>W69</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>bhutan, fiji, ghana, kenya, kiribati, malaysia</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>22 budget documents are held and excluded from their country's run on predictions that were never tested</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Config records what exists. These configs record what somebody expected to work, and a belief written into a config reads as a finding, so nobody re-tests it. bhutan, ghana, malaysia and jamaica all say they keep 'the budget years whose documents carry a programme table (document_shape.py)' - a script that had never been written until 2026-08-25. kiribati says 'Development Budget, not Recurrent. The recurrent budget is an economic classification ... which map to no plan strategy'. Six newly generated configs had budget_documents left empty on the grounds that a budget speech carries no programme lines, while Brunei extracts 27 to 61 rows a year from its budget speeches and Fiji up to 269 from its budget addresses. The exclusions include Fiji's 2018-2019 Budget ESTIMATES and Kenya's FY2015-16 programme-based budget, which is the same document type that yields 887 rows in the years that were run. The cost of a wrong exclusion is silent and permanent: the data never appears and the config explains why in a sentence that sounds researched.</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Include every held document and let the extraction produce the evidence. config_completeness.py is registered as an L2 gate: a document we hold is either in the run, or the config carries a reason naming a date, a cost or a row count. Predictions no longer pass. Brazil is exempt because its budget layer is pre-built and its one exclusion cites 439 pages, 10,214 chunks and $38, which is a measurement.</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>held vs configured budget documents: kiribati 14/4, malaysia 10/5, fiji 11/8, ghana 4/2, bhutan 5/4, kenya 3/2. Bhutan and Kiribati were each called blocked for eleven days and produced 390 and 300 rows on a re-run costing $1.04 and $1.43.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>W70</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>extraction</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>china, india, tuvalu</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Some years extract and others return nothing from the same country's documents</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>China produced 26 rows for 2026 and 0 for 2022 through 2025 from five budget speeches of the same kind. India produced 15 for 2026 and 0 for 2003 and 2025. Tuvalu produced nothing across three annual reports. That is not obviously wrong - a speech in one year may state allocations that another year's does not - but it is unexplained, and an unexplained zero is indistinguishable from a failure. Bhutan and Kiribati both looked exactly like this before it turned out a superseded prompt was the cause.</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Look at one zero year and one non-zero year of the same country side by side before treating the zeros as real. Cheap: the documents are parsed and cached, so the comparison costs nothing.</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>china 2022-2025 0 rows, 2026 26 rows; india 2003 and 2025 0 rows, 2026 15; tuvalu 2015, 2016, 2017 all 0.</t>
         </is>
       </c>
     </row>
@@ -3352,7 +4397,2035 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SETTLED ON</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>SEVERITY</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>COUNTRY</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>WHAT IT WAS</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>WHAT WAS DONE ABOUT IT</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>EVIDENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>bhutan, ghana, malaysia</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Four of seven candidate countries cannot be run on the budget documents we hold, each for a different reason</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Fixed for Bhutan 2026-08-25 by re-running stage 5 with --force at a cost of $1.04. Kiribati is the same shape and the same fix. The general lesson is W7's: any country whose outputs predate a prompt rewrite should be re-run before being called blocked, and the run date against the prompt mtime is enough to spot it. Ghana and Rwanda are still blocked on documents, not on this.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/_probe/*.xlsx; Kenya 631 programmes, Jamaica 208, Malaysia 71, Ghana 0, Bhutan 0, Kiribati 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>kiribati</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>A budget document can be the right document, parsed perfectly, and still extract nothing</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-25 by re-running stage 5 with --force at a cost of $1.43, against the $2.33 the 14 August attempt spent producing nothing. Bhutan was the same fault and the same fix. Both countries then had a full re-run on current prompts, because stages 3 and 4 also predated the 19 August prompt rewrites.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>D12 and the shape probe; Files/llm/kiribati/kiribati_budget_*.xlsx, 0 rows each</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>W61</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>panel_budget.budget double counts: summing it across strategies exceeds the whole budget</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Done 2026-08-25. The per-year sheet header now reads FUNDING (DO NOT SUM), country_summary carries a SUMMING FUNDING OVERSTATES BY column with the measured multiple per country, and the read_me states the magnitudes rather than only the principle. The multiple is computed from the rows the workbook actually writes, and verified against an independent sum of the written column: the two agree to the last decimal for all eight countries.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>sum(FUNDING column)/country_summary.MAPPED: fiji 5.40, malaysia 4.15, thailand 3.94, jamaica 2.76, kenya 2.39, brunei 2.21, maldives 2.15, brazil 1.58. Independent re-sum of the written workbook agrees exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>W39</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Two migrations in the repo had never been applied to the live database, and the code was designed to hide it</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Apply 0003 and 0005 in the SQL editor. Longer term the publish step should assert the migration level it expects rather than adapting to whatever it finds, so an unapplied migration is a red run rather than a warning. Verified fixed 2026-08-24: verify_schema.py reports all 45 declared objects present across the first ten migration files, so both migrations are applied. The register had gone stale, not the database.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>select source_documents?select=doc_type -&gt; 400 'column source_documents.doc_type does not exist'; select access_log -&gt; 404 'Could not find the table public.access_log'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>W54</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>db.select silently truncates at 1000 rows, and passing a larger limit does not lift it</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. db.Supabase.select_all() pages past the cap, and select()'s docstring now states the cap rather than leaving it to be discovered. select_all RAISES when it needs a second page and the caller gave no 'order', because offset without a stable sort reads a row twice or not at all, and the right column is the caller's to choose. build_sector_gap and verify_sector_layer use it.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>select('sector_responses', limit=20000) returned 1000; fetch_all returned 1268 with distinct row_no 1..1268.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>W53</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Prompt 7 consolidates within a BATCH, not within a document, so a large document returned the same intervention more than once</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. run_stage7_responses merges records with the same normalised name within a document after all batches return: source_refs, related_risks and sdg_targets are unioned, and in_ndp='yes' wins, because a batch that matched the intervention to a plan strategy is evidence the plan carries it and the safe direction is to under-report novelty. Deterministic, no extra model call. verify_sector_layer.py now asserts no intervention appears twice in one document.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Before: malaysia 1230 rows with 12 within-document duplicates, all in Education 2026-2035. After: 1268 rows, 0 duplicates; brunei 414 rows, 0 duplicates both before and after.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>W50</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Kenya cannot trace 36.9% of its extracted interventions back to a plan chunk, but only 2.8% are actually missing</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22, and not by editing Prompt 4. The prompt already states the rule twice ('Preserve every ref', 'Every input ref number appears in exactly one source_chunks array') and Kenya still left 509 uncited, so more words were not the answer and would have risked the seven countries that comply. Instead stages.adopt_orphans() asks again about the specific rows that went missing - a far smaller question than the one that produced them - showing the model the orphaned interventions and the inventory it already built, and taking -1 for an orphan no strategy covers. It runs inline at the end of stage 4 for future runs, and 02_Automation/repair_source_chunks.py applies it to outputs that already exist, so no country has to re-run stage 4 and re-decide every name, risk and orientation to fix a citation.
+THE PASS ONLY APPENDS TO source_chunks. Kenya: 281 strategies before and after, names identical, and no field other than source_chunks changed; the rebuilt FINAL_PANEL is identical in content across all 14 sheets. 506 of 509 placed for $0.07, 3 refused and left uncited, taking A22 from 36.9% to 0.2%.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>kenya A22: 509 uncited (36.9%) -&gt; 3 uncited (0.2%). Placements judged on substance rather than wording: 'Laboratory for Sample Analysis' -&gt; 'Anti-doping education, testing and enforcement', 'National Sports Fund' -&gt; 'Strategic funds and technical institutions'. Panel content unchanged, 14/14 sheets identical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>W49</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>kenya</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>lineage.py printed every country's name UNDER the rows it labelled, so the whole table read one country out of step</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22: report() prints the header above its own rows and main() no longer prints one. With the table readable, a second real loss became visible that the misalignment had been hiding (maldives stage 5 -&gt; budget layer, 34.1%).</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Before: KENYA section showed '1451 -&gt; 1438 lost 13 (0.9%)' (Malaysia's row) against a summary of 'kenya ... 509 of 1378'. After: KENYA shows '1378 -&gt; 869 lost 509 (36.9%)', matching the summary exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>W47</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>One control character in a document's text layer destroyed a run after every model call for it had been paid for</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. writer._cell strips the forbidden control characters (tab, newline and carriage return are legal and are kept). Stripped rather than escaped: they are artefacts of the PDF's encoding and carry no meaning, and the alternative is losing the file.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>openpyxl.utils.exceptions.IllegalCharacterError raised from writer.write_results via stages.run_stage7_risk; run died at $5.05, re-run replayed from cache at $0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>W46</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>'The plan does not carry this' merged a subject the plan is silent on with a mechanism for something it already commits to</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. Prompt 7's binary in_ndp became ndp_relation with three values - carried, broader_only, silent - and in_ndp is now DERIVED from it (carried -&gt; yes, otherwise no), so audit check A23, the published column, the dashboard and any query already written are unaffected by construction rather than by being updated in step. Migration 0011 adds the column; publish_sector drops it with a warning where 0011 has not been applied. verify_sector_layer.py asserts in_ndp and ndp_relation never disagree, on every row.
+The split is large enough to have changed the reading: Brunei 240 broader_only against 76 silent, Malaysia 573 against 126. So 202 of 756, not 756, are subjects a plan has not addressed.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>brunei carried 97 / broader_only 240 / silent 76; malaysia carried 414 / broader_only 573 / silent 126. Measured against a golden baseline taken before the prompt change: on the 251 interventions present in both Brunei runs, related_risks held at 94% and HDICategory at 99%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>W45</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Stage 5 now emits a 'grand_total' line_type that the L2 schema gate, and the database, both refuse</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22, in three places, because the value had to be accepted at each. validate_stage_schema.py allows 'grand_total' in the stage 5 line_type enum, so the L2 gate passes on clean data and still catches an injected bad value. publish_run.budget_rows() accepts it instead of raising - the raise was the real blocker, because it fired before the existing degrade-gracefully fallback could run, so the publish failed rather than dropping a row. Migration 0010 extends the budget_lines CHECK constraint, and the fallback in publish_run.push is now a LIST of optional line types rather than one hard-coded value, since this has now happened twice ('national' needed 0006, 'grand_total' needs 0010). No view was touched: every one filters line_type by positive equality, so a new value cannot fall into an existing total.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Brunei stage 5 output: {'grand_total': 3, 'strategy_total': 3, 'program': 41}; tamper_test --country brunei -&gt; FALSE POSITIVE schema; live budget_lines holds only strategy_total and program</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>W43</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Nothing could read the pv2-sources bucket, so a document added to it by hand was invisible to the pipeline</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. db.list_objects() and db.download() added, a 'supabase' backend in fetch_sources.py with --from-bucket and --type, and an unknown backend is now a config error instead of a silent fallback. Both configs corrected.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>source_documents held 7 brunei rows and 0 malaysia rows; the bucket held 15 brunei objects including 8 under 'sector strategies/'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>W42</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Document Intelligence slicing triggered on page count alone, so a short but very large document still timed out</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. The slice size is now the smaller of the page limit and a 10 MB byte budget, and a timeout retries once at half the slice size.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>39,843,726 bytes over 22 pages; sliced at 5 pages it parsed to 759 paragraphs across all 22 pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>W41</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>A dry run spent real money on Document Intelligence while reporting that it spent none</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. parse.DRY_RUN makes an uncached document read from its own text layer instead, which is free, and counts the pages the real run will be billed for so the estimate still carries them.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>HttpResponseError (Timeout) raised from _analyze during --dry-run; PAGES_PARSED['parsed'] was 86 at the time</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>W40</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>brunei, malaysia</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>The filename rule types any document containing the substring 'plan' as an NDP, which would have filed two sector strategies as the national plan</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-22. type_from_folder() now outranks every other signal, so the mirror subdirectory decides the type and the filename is only consulted for a file sitting at the top level. run_llm_pipeline.py additionally refuses a config that lists one document as both an NDP and a sector strategy.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>type_from_name('Digital Economy Masterplan 2025.pdf') returned 'ndp' before the change; both files now type as 'sector'</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Document Intelligence renders the Maldives budgets as Arabic, not Thaana, so the programme names reaching the model are already gibberish</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Do not spend on another stage 5 run until the parse is fixed; no prompt can recover text the parser destroyed. Document Intelligence has no locale for Dhivehi. The options are to parse these documents outside DI with a Thaana-capable extractor and accept the loss of table structure, or to treat Maldives as out of scope for the current toolchain. The translation hint is left in the config so it applies once the text arrives intact. FIXED 2026-08-22 by not using OCR at all. These PDFs carry their own embedded text layer holding the real Thaana Unicode: 526,059 Thaana characters in FY2019 against the 0 Document Intelligence returned, because the OCR was matching rendered Thaana glyphs to the nearest Arabic letter. parse.read_text_layer reads the characters directly, which is free, instant and exact, and "parser": "text_layer" in the country config selects it. parse._warn_if_script_mismatch compares the OCR against the file's own text layer on every un-cached parse and names the setting to change, so the whole class is caught for any country. Maldives programme names went from 395 of 852 unreadable to 0 of 56, A20 passes, and the audit went from 15/18 to 17/18.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>02_Automation/cache/di_&lt;hash&gt;.json for the FY2017 budget: 0 Thaana, 159,753 Arabic; pypdf on the same file: 342,715 Thaana</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>A strategy named after the budget line that funds it, so the match is a name matching itself</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>See F6 in FIXES.xlsx, which is cheaper and more enforceable than F3: Prompt 4 must not emit a strategy that consolidates no extracted intervention, and check A18 now fails any that does. F3, the transcript prompt, remains the way to give Brunei enough plan material in the first place.  VERIFIED FIXED 2026-08-21, measured across all eight countries: no strategy in any country carries the name of a budget programme (0 of 127 in Brazil, 0 of 83 in Brunei, 0 of 382 in Malaysia). Prompt 4 now forbids naming a strategy after a budget line and A18 fails any strategy consolidating no intervention.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>D11 in the detected sheet; audit check A18 (brunei 2 with no component); the budget-named flag in the explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>W36</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, kenya, fiji</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Programmes carrying no money are matched to strategies</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Either drop zero-amount programmes before stage 6 sees them, or flag the edge so a strategy funded only by zero-amount lines still reports as unfunded. DONE 2026-08-21: combine_budget_years raises a zero_amount_programme flag per row (Malaysia 36, Kenya 19, Brazil 4, Fiji 1), so they are visible in every run rather than silently making a strategy look funded.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>funding_by_program amount == 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>W35</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>brazil, kenya</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>funding_by_program breaks the contract its own documentation states</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Restate the guarantee as one row per (year, head, programme) and say so in REQUIREMENTS.md, or add the head to the sheet's key. This is W1 seen from the consumer's side. DONE 2026-08-21: the sheet's contract now reads one row per (year, budget head, programme) and names Brazil's FY2024 code 2317 under five functions as the worked example.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>8 duplicated keys in Brazil funding_by_program, 5,511.0 BRL million</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>W32</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Maldives is unreadable and is published anyway</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Pull Maldives from the published set until its budgets are re-parsed. Document Intelligence renders Thaana as Arabic and then as European nonsense, so the fix is upstream of every prompt. A readability gate belongs in the pipeline: a country whose programme names fail a letters-per-name test should not reach publish_run.  PARTIAL 2026-08-20: new audit check A20 fails any country where more than 20% of programme names are unreadable, and combine_budget_years raises a HIGH data_quality flag for the same. Maldives fails it at 46%; every other country passes at 0%. The country is still published; pulling it is a decision, not a bug fix. DONE 2026-08-21: publish_run now REFUSES a country whose programme names are more than 20% unreadable, naming the share and two examples, and offering --allow-unreadable for a deliberate override. Maldives is refused and its eleven previously published runs were deleted, so it is off the dashboard until its budgets parse.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>budget_all_years, Maldives; 395 of 852 programme names fail the readability test</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>W31</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Programme class and BAU share cannot reach the dashboard until a migration is applied by hand</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Apply 03_Ingest_and_Publishing/supabase/migrations/0006_programme_class.sql in the Supabase SQL editor, then re-publish. publish_run.py now probes each table and drops unknown columns with a warning naming the migration, so publishing degrades to the old behaviour instead of failing outright. DONE 2026-08-21: 0006 and 0007 applied, all eight countries republish with zero warnings, and v_development_coverage matches the layer exactly on every country.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>publish_run.table_columns against the live schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Strategies that entered the panel from the budget document rather than from the plan</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>See F3 in FIXES.xlsx. Brunei's plan text is a speech, so stage 3 recovers little from it and stage 4 fills the gap from the budget side. The transcript prompt is the fix; until it exists these rows should be excluded from any count of plan strategies rather than silently included.  VERIFIED FIXED 2026-08-21, measured across all eight countries: A18 passes everywhere: 0 strategies in any country consolidate no extracted intervention, Brunei included.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>D3 in the detected sheet; the no-evidence flag on the country explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>W29</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>One budget head carried under two spellings across years, so no head-level series is continuous</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Normalise head names when building the layer, case-folded and with a per-country alias map for the language pairs, keeping the raw name in a source column. The within-year duplicate is a different problem and needs the code, not the name, as identity.  VERIFIED FIXED 2026-08-21, measured across all eight countries: no head in any country carries more than one spelling (Malaysia 41 heads, 0 with a second form). canonicalise_head_names renames per code and keeps the original in strategy_name_source.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>budget_all_years strategy_total rows, Malaysia, 37 pairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>W22</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>The intern pack ships a stale copy of the pipeline it is meant to hand over</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Decide whether the pack is maintained or retired. If maintained, generate it rather than copying it, which needs the pack's dependency set worked out because the live runner reaches for validators the pack does not have. check_handoff_drift.py measures the gap in the meantime. DONE 2026-08-21: sync_handoff.py copies the five pipeline scripts and all seven prompts into the pack and --check runs in the test suite. It was shipping build_final_panel at 677 lines against a live 977 and combine_budget_years at 372 against 819, and had never carried prompt 5b at all.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>05_Handoff/scripts/check_handoff_drift.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>W21</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Per-country settings are split across two config files that must agree, and nothing checks</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>One document profile per country, in one file, with four mechanisms: how to read it, where the levels sit, how the codes are shaped, and how the amounts are labelled. The code is already generic; it is the configuration that is scattered. DONE 2026-08-21: check_configs.py compares the two per-country config files and the paths they name, and runs in the test suite. It found two real faults on its first run: bhutan and kiribati name mapping folders that are not here. HIGH blocks, advisory does not, because a country not yet mapped is a normal state.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>02_Automation/inputs/*.json; 01_Pipeline/countries/*.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>W19</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>The reverse pass carries the same precision clamp as the forward pass it exists to correct</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Remove that line from 6b only and re-run one country, diffing against the coverage workbook already on disk. Jamaica was the obvious candidate until its budget turned out to be genuinely administration-heavy; Fiji is the cleaner test. Gated on W18, because without precision numbers a rise in edges cannot be read either way. DONE 2026-08-21: prompt 6b no longer carries prompt 6's clamp. It states why its bar is deliberately lower (it exists to recover the siblings the strategy-side pass missed, and cannot inflate a strategy's money because the amount is attributed per programme once), while still refusing sector adjacency alone and overhead lines. Takes effect on the next 6b run.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/prompts/6b_programme_coverage.txt L48-51</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>kenya, jamaica, brazil</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>The strategy inventory holds the same strategy twice, once bare and once prefixed with its budget code</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Consolidate in stage 4, which is where the two forms are created. Pending that, de-duplicate in a strategyclean hygiene pass keeping the bare form, which costs nothing and corrects the denominators now.  VERIFIED FIXED 2026-08-21, measured across all eight countries: every inventory collapses to its own size once the code prefix is stripped (Kenya 281 names -&gt; 281, Brazil 127 -&gt; 127), so no strategy is held twice. Prompt 4's naming rules stop it at source and twin_aliases still folds any survivor.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Files/llm/&lt;slug&gt;/&lt;slug&gt;_strategyclean.xlsx; the ambiguous-join drops logged by stage 6b</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>kenya, fiji, jamaica, maldives, brunei</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>A printed strategy total smaller than the programmes beneath it, which surfaces as a ceiling failure once enough of them are matched</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Stage 5, not stage 6. Have the extraction emit a total for every strategy and reconcile it against its own programme rows before the layer is written, so the contradiction is caught where it is created. Until then read the ceiling sheet as a report on the budget layer rather than on the edges, and treat a rounding-scale exceedance separately from a structural one. DONE 2026-08-21: build_final_panel derives a head's CAPACITY, its printed total or, where that under-reports its own countable programmes by more than 5%, the programme sum, and both the ceiling and the coverage share use it. 101 of Malaysia's 200 head-years and 43 of Jamaica's 79 are recomputed, and coverage above 105% falls from 5 head-years to zero across all countries. Both sheets now carry printed_total and total_basis so the substitution is visible.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx ceiling sheet, status EXCEEDS TOTAL; audit_checks A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>jamaica, kenya</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>A budget layer can join perfectly and still be wrong, and the coverage figure is where it shows</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Kenya needs nothing further. Jamaica needs stage 5 re-run with a structure hint that emits a total for every head, keeps recurrent and capital apart in the code, and ignores the object-of-expenditure detail. Until then its coverage figure should not be read. More generally, program_code_style should be chosen by measurement rather than defaulted: a code that never matches and a code that matches too much look identical until the totals are compared. DONE 2026-08-21: the style cannot be inferred safely, because Malaysia at 49% code reuse needs prefixing and Brazil at 27% must not have it, so combine_budget_years now FLAGS the contradiction instead of guessing: hierarchical style where under 5% of raw codes begin with their head and under 5% recur across heads raises a HIGH code_style_suspect flag naming the setting to change.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>run_report unmatched_codes 824 -&gt; 0 and 254 -&gt; 0; budget_all_years head totals against programme sums per year</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>malaysia</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>23 of 40 budget heads do not reconcile, because head totals and programme rows are attributed differently</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Per-strategy coverage for Malaysia should not be read until this is fixed. The national total and the strategy inventory are unaffected, as is every mapping. The fix is to have Prompt 5 emit the head's short code as printed in the page corner (B.62), which is on every page of the document, and to reject a strategy_total whose source_location does not name a head. DONE 2026-08-21: see W13; a head whose printed total under-reports its own programmes is now measured against the programmes.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>stage5_probe on FY2026: 731 lines, 25 reconciliation problems, 100 rows dropped by the code pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>brazil</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>A programme code is not unique within a fiscal year, so no figure keyed on (year, programme) is exact</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>See F1 in FIXES.xlsx. The unit is (year, budget strategy, programme), not (year, programme). Stage 6 must record which budget strategy the matched line sits under, load_budget must key on all three, and the Supabase view must join on all three. Until then the dashboard shows the lower bound. The remaining work is upstream: stage 5 should emit a code that is unique within the year, at which point A3 passes on its own. DONE 2026-08-21: new check A21 asserts that every accepted edge on a repeated code names its budget head, so the last-row-read fallback is never reached. Brazil has 28 repeated codes and Kenya 7, and no edge in any country omits its head. Migration 0008 fixes the same fault in v_funding_by_program.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>D1 in the detected sheet; FY2024 codes 0032, 0901, 0902, 0903, 0909, 0910, 1144, 1149</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>W33</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, jamaica</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>The national denominator is not the national budget, so the headline share is wrong</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>FIXED 2026-08-20. The real cause was a LEVEL COLLAPSE, not a missing operating/development split. Stage 5 flattened a three-level budget into one 'program' line_type, so Malaysia's head 63 carries four programmes summing to 43,291,751,100 AND the nineteen activities beneath them summing to the same 43,291,751,100, while the stored head total of 4,013,756,600 is merely the first programme. Neither published basis was the budget: the heads understate by 10x on that head and summing every programme row doubles it. combine_budget_years now detects nesting PER HEAD-YEAR, accepting it only where the two levels arithmetically coincide (15 nested head-years in Malaysia, 175 flat), counts the top level once, and writes the chosen basis into a national_total sheet that every consumer reads instead of re-deriving. Malaysia 87.28% -&gt; 49.85%, Jamaica 86.80% -&gt; 70.27%, Fiji 76.58% -&gt; 80.52%, Maldives 1.70% -&gt; 2.37%. Brazil, Kenya and Thailand reconcile and did not move.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>sum(strategy_total) vs sum(program) per country, all 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Strategies are tagged with risks they do not respond to</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>See F2 in FIXES.xlsx. Prompt 4 must require a quotation from the strategy's own text for each risk it names, and must not tag a standing function on sector adjacency alone. Re-running stage 4 changes related_risks, risk_salience and every risk view downstream.  DONE 2026-08-19: see W30.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>D4 in the detected sheet; Brazil 'National Defense', 'Public Security with Citizenship' (6 risks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>W17</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>The shared mapping prompt hard-codes one country's overhead vocabulary</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Move the list into the per-country profile as an overhead_names key and leave the shared prompt describing the CLASS of thing to refuse rather than one country's wording. It invalidates the stage 6 cache, so it should ride with the next deliberate prompt change rather than on its own.  DONE 2026-08-19: prompt 6 now refuses by programme_class rather than by the seven Thai name fragments, which are removed.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/prompts/6_mapping.txt L50-55</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>W67</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>ghana, india, nauru, papua_new_guinea, rwanda, samoa, tuvalu</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Seven configured countries have never been run, and nothing records why</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Eight run 2026-08-25 for $1.72 producing 1,049 budget rows. They now need stages 4 and 6 and a panel. Ghana and Papua New Guinea are still unrun: PNG's config points at Volume 1 and its own note says the appropriations are in Volumes 2 and 3, which are not held, so that one is a documents gap rather than an assumption.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>cost_ledger.jsonl: ghana 4 entries all dry_run, rwanda 4 all dry_run, papua_new_guinea 1 dry_run; india, nauru, samoa, tuvalu no ledger. All seven have ndp_documents and budget_documents that exist on disk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>W66</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>There is no cheap way to tell whether a budget document will extract, and two attempts to build one both failed</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed 2026-08-25. document_shape.py stays unregistered as a gate. The working practice is to run the cheapest slice: stage 5 for one year costs between $0.03 and $0.50 a country, and eight countries cost $1.72 to settle definitively.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>probe verdict vs rows actually extracted: brunei NO TABLE/61, kenya NO TABLE/887, fiji SPEECH/269, jamaica GO/169, bhutan NO TABLE/0, kiribati NO TABLE/0. Appropriation-word counts: brunei 0 with 61 rows, bhutan 67 with 0 rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>W51</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>maldives</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>29 of 85 extracted Maldivian programmes do not reach the budget layer</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Gone on re-extraction, not by a code change here. The Maldives budget was re-extracted on 2026-08-22 and the hop now reads 454 -&gt; 454, nothing lost, where it had read 85 -&gt; 56. The 29 rows were never dropped by combine_budget_years; the extraction they came from was the incomplete one W38 describes. Recorded because the two findings look alike from the lineage table and are not the same thing.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Before: maldives stage 5 -&gt; budget layer 85 -&gt; 56, lost 29 (34.1%). After a re-extraction: 454 -&gt; 454, lost 0 (0.0%), and the country passes every conservation hop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>W5</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>A programme-strategy pair matched twice, once by each pass</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Nothing to fix in the data. Any new consumer must count pairs, not rows.</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>D9 in the detected sheet; the 'twice' filter in the audit view</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>W48</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>brunei</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>The layer on disk was stale against the code, so a working parser looked like a broken one</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>No code change needed; re-running combine_budget_years populates it. The general lesson is the one worth keeping: a derived artefact carries no record of the code version that built it, so a stale layer is indistinguishable from a broken stage. Brunei's four years were re-extracted on 2026-08-22 and grand_total now reads 5,860 / 5,860 / 6,250 / 6,350 BND million with extracted_pct against each.</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Before re-run: grand_total None for 2021, 2022, 2025, 2026. After: 5860 / 5860 / 6250 / 6350, basis 'grand_total', extracted_pct 96 / 102.9 / 38.4 / 16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>W37</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Nested budget levels are counted once, and the decision is a column rather than a rule each reader re-applies</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>combine_budget_years decides per head-year, accepting a hierarchy only where the two levels arithmetically coincide, and stamps 'countable' Y/N on every programme row. Migration 0007 adds the column and rebuilds the view to respect it; NULL is treated as countable so older runs read exactly as before.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Malaysia 1,847.9bn all rows vs 1,692.0bn countable</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>W34</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, jamaica, fiji, maldives</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>The ceiling test fails on broken head totals rather than on over-attribution</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>FIXED. A4 now caps each head at its printed total or, where that under-reports its own programmes by more than 5%, at the programme sum, and says how many heads were capped. Malaysia 38 failures -&gt; 0, Jamaica 17 -&gt; 0, Maldives 1 -&gt; 0. Fiji's 3 survive and are genuine over-attribution.</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>audit_checks A4, all countries</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>W30</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Risks were unioned across merged interventions, so a strategy could name ten of eleven</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Prompt 4 now applies a responds-to test, caps related_risks at three ordered by centrality, and requires a verbatim risk_evidence quote per risk. validate_stage4 enforces the cap and DROPS any risk whose quote is missing. Prompt 3 carries the same responds-to test at source, and states that an empty list is the right answer when the intervention responds to a risk outside the eleven, which is the honest answer for road safety.</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>scan_scoreboard risks_per_strategy, risk_top_share, share_risk_evidenced</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>W28</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>funding_priority was not a function of its inputs</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>FIXED. Ties take the average position of their group. New audit check A19 asserts that strategies identical on risk salience and funding share a priority; it failed on 8 of 9 countries before the change and passes on all 9 after.</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>audit_checks A19; pct_ranks([5,5,5,5,5])</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>W26</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>The share of the budget mapped was not comparable between countries, because it measured what the budget document contains</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Stage 5b (01_Pipeline/prompts/5b_programme_class.txt) classifies every programme as development / standing_function / overhead / mixed, once per distinct (head, programme). combine_budget_years attaches it, and class_overrides in the country config beats the model so a wrong class costs an edit rather than a re-run. Panels now carry bau_share_pct and bau_funded per strategy. DONE for all 8 published countries, $0.83.</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>scan_scoreboard share_dev_mapped vs share_mapped, all 8 countries</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>W24</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>A crashed stage reported as ok, and the run carried on from the previous panel</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Fixed: only the script documenting that contract gets it, and never with a traceback in its output.</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/scripts/run_pipeline.py run_stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>W23</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Seven implementations of one list parser, and one of them splits on a character that appears inside the values</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>FIXED. build_analytics_html now splits on ';' only, the same rule audit_checks.as_list already used and for the same stated reason. The other six are left alone and documented as intentional: forcing one parser would break SDG target parsing and the Postgres NULL distinction.</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>03_Ingest_and_Publishing/scripts/publish_run.py as_list</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>W16</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>jamaica</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Stage 5 returned one programme per Head; now extracted deterministically from the Head summary tables</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Fixed, and not by a prompt. extract_budget_tables.py reads the per-Head summary tables straight from the parsed markdown, where a programme row is the one whose first cell begins with two numbers. The rule is regexes in jamaica.json under 'budget_tables'; the script itself holds no country logic. The layer went from 172 programme rows to 341, edges from 92 to 399, strategies with no budget from 68 to 7, and the mapped share from 6.8% to 91.3%. Recall resolves at 66% where it could not be estimated at all. One trap for the next document: codes must be digits-and-dots, because _clean_code keeps only \d+(\.\d+)* and silently trimmed the first hyphenated attempt back to the Head.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>01_Pipeline/scripts/extract_budget_tables.py; 02_Automation/inputs/jamaica.json budget_tables</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>W15</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>FIXED</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>malaysia, brazil</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Stage 6 is shown only one programme per repeated code, so most of the budget was never a candidate for matching</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Fixed. schemas.build_programme_index keys the candidate set on both the bare code and (strategy_code, program_code), and resolve_programme demands the head only where the code is genuinely ambiguous. validate_stage6 now uses the model's own strategy_code to disambiguate before replacing it with the matched row's. build_final_panel.ProgrammeLookup resolves the same way and additionally joins a bare mapping code to a hierarchical layer code. Stage 6 was replayed from cache for Malaysia: 1,566 edges now resolve where 0 did, only 3 records across five years still cannot be placed, and Malaysia's mapped share went from 0.0% to 86.9%. Brazil's colliding codes are unchanged and remain W1: the panel still takes the last row for a repeated code, because only the merge loop knows the head and the sheets built afterwards would disagree with it.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>stages.py:611; schemas.py:243-244; Files/llm/malaysia/malaysia_budget_*.xlsx vs mappings/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3407,18 +6480,233 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Flag raised while combining the budget years</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / data_quality</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>5 high flag(s) the run already raised, repeated here so one file carries every country's oddities.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 partial_budget : the heads extracted sum to 6,085,505,000,724.0 but the document's own grand total is 30,01
+FY2026 reconciliation_mismatch 1: programs sum to 1,105,000,000,000.0 but strategy_total is 100,000,000,000.0 (gap -1,005,00
+FY2026 reconciliation_mismatch 4: programs sum to 1,509,200,000,724.0 but strategy_total is 1,250,000,000,000.0 (gap -259,20
+FY2026 reconciliation_mismatch 6: programs sum to 244,200,000,000.0 but strategy_total is 202,200,000,000.0 (gap -42,000,000
+FY2026 reconciliation_mismatch 7: programs sum to 184,900,000,000.0 but strategy_total is 184,800,000,000.0 (gap -100,000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>D8</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>A strategy total its own programmes do not add up to</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx / reconciliation</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>4 strategy-year(s) do not reconcile. Either a programme row was missed or the document's own total includes something not broken out.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 strategy 1: printed 100,000,000,000.0, programmes sum to 1,105,000,000,000.0, apart by -1,005,000,000,000.0
+FY2026 strategy 4: printed 1,250,000,000,000.0, programmes sum to 1,509,200,000,724.0, apart by -259,200,000,724.0
+FY2026 strategy 6: printed 202,200,000,000.0, programmes sum to 244,200,000,000.0, apart by -42,000,000,000.0
+FY2026 strategy 7: printed 184,800,000,000.0, programmes sum to 184,900,000,000.0, apart by -100,000,000.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>D10</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>One budget year only</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>budget_layer_all_years.xlsx</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>The layer covers 2026. Nothing on this country can show a trend, and its share of budget mapped rests on a single document.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Strategy with no budget in any year</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unfunded_strategies</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>98 strategy(ies) are stated in the plan and funded by nothing. This is a finding about the country, not a defect, unless the strategy IS funded and the match was missed.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>City cluster and metropolitan integration development
+Governance reform and market system modernization
+High-standard opening-up and services market liberalization
+Industrial foundation strengthening and supply chain security
+High-end equipment and industrial software innovation
+Strategic emerging and future industries cultivation
+Biomanufacturing and advanced biopharmaceutical innovation
+Low-altitude economy and unmanned aviation development</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Budget programme no strategy claims</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>FINAL_PANEL.xlsx / unmapped_programs</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>2 distinct programme(s) across 2 programme-year row(s) are funded and matched to no strategy in the plan. Largest first.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>FY2026 1.3 We will expand effective investment.  755,000,000,000.0
+FY2026 1.2 We will make greater efforts to boost consum  250,000,000,000.0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3455,18 +6743,37 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>china</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3484,7 +6791,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22 21:35 by 01_Pipeline/scripts/data_issues.py</t>
+          <t>Generated 2026-08-26 03:03 by 01_Pipeline/scripts/data_issues.py</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3496,66 +6803,78 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>register</t>
+          <t>closed</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Typed by hand in 04_Docs_and_Planning/data_issues.json. What a finding means, and what would fix it.</t>
+          <t>Everything already dealt with and what was done about it, newest first. SETTLED ON is read from the fix text itself, so it cannot drift from the sentence that describes the fix.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>detected</t>
+          <t>register</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Regenerated from the workbooks on every run. Cannot go stale.</t>
+          <t>Typed by hand in 04_Docs_and_Planning/data_issues.json. What a finding means, and what would fix it.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>detected</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Regenerated from the workbooks on every run. Cannot go stale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>by_country</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Counts, so a country whose data is quietly getting stranger shows it.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="n"/>
-    </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>HIGH: a figure people read is wrong or ambiguous. MEDIUM: defensible but easy to misread, or a thin input. LOW: worth knowing, changes no number.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="n"/>
-    </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Not in here</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Contract violations (validate_stage_schema.py), figures that do not match the source document (validate_source_fidelity.py), and panel arithmetic (audit_checks.py). Those are pass-or-fail gates.</t>
         </is>

</xml_diff>